<commit_message>
fix(maps): use clean maps.google.com universal deep link and add 1-tap copyable address
</commit_message>
<xml_diff>
--- a/danh_sach_dinh_vi_winmart_mt01.xlsx
+++ b/danh_sach_dinh_vi_winmart_mt01.xlsx
@@ -559,7 +559,7 @@
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VinMart%20Ninh%20Ki%E1%BB%81u%2C%20S%E1%BB%91%2042%20%C4%90%C6%B0%E1%BB%9Dng%2030/4%2C%20Ph%C6%B0%E1%BB%9Dng%20An%20Ph%C3%BA%2C%20Qu%E1%BA%ADn%20Ninh%20ki%E1%BB%81u%2C%20Th%C3%A0nh%20ph%E1%BB%91%20C%E1%BA%A7n%20Th%C6%A1</t>
+          <t>https://maps.google.com/?q=VinMart+Ninh+Ki%E1%BB%81u%2C+S%E1%BB%91+42+%C4%90%C6%B0%E1%BB%9Dng+30%2F4%2C+Ph%C6%B0%E1%BB%9Dng+An+Ph%C3%BA%2C+Qu%E1%BA%ADn+Ninh+ki%E1%BB%81u%2C+Th%C3%A0nh+ph%E1%BB%91+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VinMart%20Can%20Tho%2C%20S%E1%BB%91%202%20H%C3%B9ng%20V%C6%B0%C6%A1ng%2C%20P.%20Th%E1%BB%9Bi%20B%C3%ACnh%2C%20Q.%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=VinMart+Can+Tho%2C+S%E1%BB%91+2+H%C3%B9ng+V%C6%B0%C6%A1ng%2C+P.+Th%E1%BB%9Bi+B%C3%ACnh%2C+Q.+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VinMart%20Xuan%20Khanh%2C%20B1-06%2C%20Tang%201%2C%20So%20209%20Duong%2030/4%2C%20Phuong%20Xuan%20Khanh%2C%20Quan%20Ninh%20Kieu%2C%20Thanh%20pho%20Can%20Tho</t>
+          <t>https://maps.google.com/?q=VinMart+Xuan+Khanh%2C+B1-06%2C+Tang+1%2C+So+209+Duong+30%2F4%2C+Phuong+Xuan+Khanh%2C+Quan+Ninh+Kieu%2C+Thanh+pho+Can+Tho</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VinMart%20V%C4%A9nh%20Long%2C%20TTTM%20Vincom%20Plaza%20V%C4%A9nh%20Long%2C%20T%E1%BB%95%209%2C%20Kh%C3%B3m%203%2C%20Ph%C6%B0%E1%BB%9Dng%204%2C%20Th%C3%A0nh%20ph%E1%BB%91%20V%C4%A9nh%20Long%2C%20T%E1%BB%89nh%20V%C4%A9nh%20Long</t>
+          <t>https://maps.google.com/?q=VinMart+V%C4%A9nh+Long%2C+TTTM+Vincom+Plaza+V%C4%A9nh+Long%2C+T%E1%BB%95+9%2C+Kh%C3%B3m+3%2C+Ph%C6%B0%E1%BB%9Dng+4%2C+Th%C3%A0nh+ph%E1%BB%91+V%C4%A9nh+Long%2C+T%E1%BB%89nh+V%C4%A9nh+Long</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VinMart%20Ki%C3%AAn%20Giang%2C%20TTTM%20Vincom%20Plaza%20Ki%C3%AAn%20Giang%2C%20L%C3%B4%20A12%2C%20Khu%20ph%E1%BB%91%201%2C%20Ph%C6%B0%E1%BB%9Dng%20V%C4%A9nh%20B%E1%BA%A3o%2C%20Th%C3%A0nh%20ph%E1%BB%91%20R%E1%BA%A1ch%20Gi%C3%A1%2C%20T%E1%BB%89nh%20Ki%C3%AAn%20Giang</t>
+          <t>https://maps.google.com/?q=VinMart+Ki%C3%AAn+Giang%2C+TTTM+Vincom+Plaza+Ki%C3%AAn+Giang%2C+L%C3%B4+A12%2C+Khu+ph%E1%BB%91+1%2C+Ph%C6%B0%E1%BB%9Dng+V%C4%A9nh+B%E1%BA%A3o%2C+Th%C3%A0nh+ph%E1%BB%91+R%E1%BA%A1ch+Gi%C3%A1%2C+T%E1%BB%89nh+Ki%C3%AAn+Giang</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VinMart%20H%E1%BA%ADu%20Giang%2C%20TTTM%20Vincom%20Plaza%20V%E1%BB%8B%20Thanh%2C%20Khu%20v%E1%BB%B1c%203%2C%20Ph%C6%B0%E1%BB%9Dng%205%2C%20Th%C3%A0nh%20Ph%E1%BB%91%20V%E1%BB%8B%20Thanh%2C%20T%E1%BB%89nh%20H%E1%BA%ADu%20Giang</t>
+          <t>https://maps.google.com/?q=VinMart+H%E1%BA%ADu+Giang%2C+TTTM+Vincom+Plaza+V%E1%BB%8B+Thanh%2C+Khu+v%E1%BB%B1c+3%2C+Ph%C6%B0%E1%BB%9Dng+5%2C+Th%C3%A0nh+Ph%E1%BB%91+V%E1%BB%8B+Thanh%2C+T%E1%BB%89nh+H%E1%BA%ADu+Giang</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20404/12%20Nguy%E1%BB%85n%20V%C4%83n%20Linh%2C%20404/12%20Nguy%E1%BB%85n%20V%C4%83n%20Linh%2C%20An%20Kh%C3%A1nh%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+404%2F12+Nguy%E1%BB%85n+V%C4%83n+Linh%2C+An+Kh%C3%A1nh%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%201B%20Tr%E1%BA%A7n%20Quang%20Kh%E1%BA%A3i%2C%201B%20Tr%E1%BA%A7n%20Quang%20Kh%E1%BA%A3i%2C%20Ph%C6%B0%E1%BB%9Dng%20C%C3%A1i%20Kh%E1%BA%BF%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+1B+Tr%E1%BA%A7n+Quang+Kh%E1%BA%A3i%2C+Ph%C6%B0%E1%BB%9Dng+C%C3%A1i+Kh%E1%BA%BF%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2053/64%20Nguy%E1%BB%85n%20Vi%E1%BB%87t%20D%C5%A9ng%2C%2053/64/%20Nguy%E1%BB%85n%20Vi%E1%BB%87t%20D%C5%A9ng%2C%20Ph%C6%B0%E1%BB%9Dng%20An%20Th%E1%BB%9Bi%2C%20Qu%E1%BA%ADn%20B%C3%ACnh%20Th%E1%BB%A7y</t>
+          <t>https://maps.google.com/?q=WinMart+53%2F64+Nguy%E1%BB%85n+Vi%E1%BB%87t+D%C5%A9ng%2C+53%2F64%2F+Nguy%E1%BB%85n+Vi%E1%BB%87t+D%C5%A9ng%2C+Ph%C6%B0%E1%BB%9Dng+An+Th%E1%BB%9Bi%2C+Qu%E1%BA%ADn+B%C3%ACnh+Th%E1%BB%A7y%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -928,7 +928,7 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%201B%20%C4%90inh%20Ti%C3%AAn%20Ho%C3%A0ng%2C%201B%20%C4%90inh%20Ti%C3%AAn%20Ho%C3%A0ng%2C%20Ph%C6%B0%E1%BB%9Dng%20Th%E1%BB%9Bi%20B%C3%ACnh%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+1B+%C4%90inh+Ti%C3%AAn+Ho%C3%A0ng%2C+Ph%C6%B0%E1%BB%9Dng+Th%E1%BB%9Bi+B%C3%ACnh%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -969,7 +969,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2029-31%20%C4%90%C6%B0%E1%BB%9Dng%20A3%2C%2029-31%20%C4%90%C6%B0%E1%BB%9Dng%20A3%20KDC%20H%C6%B0ng%20Ph%C3%BA%2C%20Ph%C6%B0%E1%BB%9Dng%20H%C6%B0ng%20Ph%C3%BA%2C%20Qu%E1%BA%ADn%20C%C3%A1i%20R%C4%83ng</t>
+          <t>https://maps.google.com/?q=WinMart+29-31+%C4%90%C6%B0%E1%BB%9Dng+A3+KDC+H%C6%B0ng+Ph%C3%BA%2C+Ph%C6%B0%E1%BB%9Dng+H%C6%B0ng+Ph%C3%BA%2C+Qu%E1%BA%ADn+C%C3%A1i+R%C4%83ng%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2038%20V%C3%B5%20V%C4%83n%20Ki%E1%BB%87t%2C%2038%20V%C3%B5%20V%C4%83n%20Ki%E1%BB%87t%2C%20Ph%C6%B0%E1%BB%9Dng%20An%20H%C3%B2a%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+38+V%C3%B5+V%C4%83n+Ki%E1%BB%87t%2C+Ph%C6%B0%E1%BB%9Dng+An+H%C3%B2a%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20216%20%C4%90%C6%B0%E1%BB%9Dng%203/2%2C%20216%20%C4%90%C6%B0%E1%BB%9Dng%203/2%2C%20Ph%C6%B0%E1%BB%9Dng%20H%C6%B0ng%20L%E1%BB%A3i%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+216+%C4%90%C6%B0%E1%BB%9Dng+3%2F2%2C+Ph%C6%B0%E1%BB%9Dng+H%C6%B0ng+L%E1%BB%A3i%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2021-22%20V%C3%B5%20Nguy%C3%AAn%20Gi%C3%A1p%2C%20Di%E1%BB%87u%2C%2021-22%20V%C3%B5%20Nguy%C3%AAn%20Gi%C3%A1p%2C%20Khu%20D%C3%A2n%20C%C6%B0%20Di%E1%BB%87u%20Hi%E1%BB%81n%2C%20Khu%20V%E1%BB%B1c%20Th%E1%BA%A1nh%20L%E1%BB%A3i%2C%20Ph%C6%B0%E1%BB%9Dng%20Ph%C3%BA%20Th%E1%BB%A9%2C%20Qu%E1%BA%ADn%20C%C3%A1i%20R%C4%83ng</t>
+          <t>https://maps.google.com/?q=WinMart+21-22+V%C3%B5+Nguy%C3%AAn+Gi%C3%A1p%2C+Di%E1%BB%87u%2C+21-22+V%C3%B5+Nguy%C3%AAn+Gi%C3%A1p%2C+Khu+D%C3%A2n+C%C6%B0+Di%E1%BB%87u+Hi%E1%BB%81n%2C+Khu+V%E1%BB%B1c+Th%E1%BA%A1nh+L%E1%BB%A3i%2C+Ph%C6%B0%E1%BB%9Dng+Ph%C3%BA+Th%E1%BB%A9%2C+Qu%E1%BA%ADn+C%C3%A1i+R%C4%83ng%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20S%E1%BB%91%202%20Tr%E1%BA%A7n%20Ho%C3%A0ng%20Na%2C%20S%E1%BB%91%202%20Tr%E1%BA%A7n%20Ho%C3%A0ng%20Na%2C%20Ph%C6%B0%E1%BB%9Dng%20H%C6%B0ng%20Th%E1%BA%A1nh%2C%20Qu%E1%BA%ADn%20C%C3%A1i%20R%C4%83ng%2C%20Th%C3%A0nh%20Ph%E1%BB%91%20C%E1%BA%A7n%20Th%C6%A1%20%28%C4%90C%20c%C5%A9%3A%20KDC%20L%C3%B4%2C%20S%E1%BB%91%206%2C%20Khu%20%C4%90%C3%B4%20Th%E1%BB%8B%20M%E1%BB%9Bi%20Nam%20S%C3%B4ng%20C%E1%BA%A7n%20Th%C6%A1%29</t>
+          <t>https://maps.google.com/?q=WinMart+S%E1%BB%91+2+Tr%E1%BA%A7n+Ho%C3%A0ng+Na%2C+Ph%C6%B0%E1%BB%9Dng+H%C6%B0ng+Th%E1%BA%A1nh%2C+Qu%E1%BA%ADn+C%C3%A1i+R%C4%83ng%2C+Th%C3%A0nh+Ph%E1%BB%91+C%E1%BA%A7n+Th%C6%A1+%28%C4%90C+c%C5%A9%3A+KDC+L%C3%B4%2C+S%E1%BB%91+6%2C+Khu+%C4%90%C3%B4+Th%E1%BB%8B+M%E1%BB%9Bi+Nam+S%C3%B4ng+C%E1%BA%A7n+Th%C6%A1%29%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1174,7 +1174,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20370%20Khu%20v%E1%BB%B1c%20Y%C3%AAn%20Trung%2C%20370%20Khu%20V%E1%BB%B1c%20Y%C3%AAn%20Trung%2C%20Ph%C6%B0%E1%BB%9Dng%20L%C3%AA%20B%C3%ACnh%2C%20Qu%E1%BA%ADn%20C%C3%A1i%20R%C4%83ng</t>
+          <t>https://maps.google.com/?q=WinMart+370+Khu+V%E1%BB%B1c+Y%C3%AAn+Trung%2C+Ph%C6%B0%E1%BB%9Dng+L%C3%AA+B%C3%ACnh%2C+Qu%E1%BA%ADn+C%C3%A1i+R%C4%83ng%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20Th%E1%BB%ADa%2012%20Y%C3%AAn%20Ho%C3%A0%2C%20Th%E1%BB%ADa%2012%20Y%C3%AAn%20Ho%C3%A0%2C%20Ph%C6%B0%E1%BB%9Dng%20L%C3%AA%20B%C3%ACnh%2C%20Qu%E1%BA%ADn%20C%C3%A1i%20R%C4%83ng</t>
+          <t>https://maps.google.com/?q=WinMart+Th%E1%BB%ADa+12+Y%C3%AAn+Ho%C3%A0%2C+Ph%C6%B0%E1%BB%9Dng+L%C3%AA+B%C3%ACnh%2C+Qu%E1%BA%ADn+C%C3%A1i+R%C4%83ng%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VM%2B%20CTO%20390Z%20Nguyen%20Van%20Cu%2C%20390Z%20Nguyen%20Van%20Cu%2C%20phuong%20An%20Khanh%2C%20quan%20Ninh%20Kieu%2C%20thanh%20pho%20Can%20Tho</t>
+          <t>https://maps.google.com/?q=WinMart+390Z+Nguyen+Van+Cu%2C+phuong+An+Khanh%2C+quan+Ninh+Kieu%2C+thanh+pho+Can+Tho</t>
         </is>
       </c>
     </row>
@@ -1297,7 +1297,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VM%2B%20CTO%20160%20Tran%20Quang%20Dieu%2C%20160%20Tran%20Quang%20Dieu%2C%20phuong%20An%20Thoi%2C%20quan%20Binh%20Thuy%2C%20thanh%20pho%20Can%20Tho</t>
+          <t>https://maps.google.com/?q=WinMart+160+Tran+Quang+Dieu%2C+phuong+An+Thoi%2C+quan+Binh+Thuy%2C+thanh+pho+Can+Tho</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2045/9%20L%C3%AA%20H%E1%BB%93ng%20Phong%2C%2045/9%20L%C3%AA%20H%E1%BB%93ng%20Phong%2C%20P.%20B%C3%ACnh%20Th%E1%BB%A7y%2C%20Qu%E1%BA%ADn%20B%C3%ACnh%20Th%E1%BB%A7y</t>
+          <t>https://maps.google.com/?q=WinMart+45%2F9+L%C3%AA+H%E1%BB%93ng+Phong%2C+P.+B%C3%ACnh+Th%E1%BB%A7y%2C+Qu%E1%BA%ADn+B%C3%ACnh+Th%E1%BB%A7y%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1379,7 +1379,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20163H-163H/7%20Nguy%E1%BB%85n%20V%C4%83n%20C%E1%BB%AB%2C%20163H-163H/7%20Nguy%E1%BB%85n%20V%C4%83n%20C%E1%BB%AB%20n%E1%BB%91i%20d%C3%A0i%2C%20Ph%C6%B0%E1%BB%9Dng%20An%20Kh%C3%A1nh%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+163H-163H%2F7+Nguy%E1%BB%85n+V%C4%83n+C%E1%BB%AB+n%E1%BB%91i+d%C3%A0i%2C+Ph%C6%B0%E1%BB%9Dng+An+Kh%C3%A1nh%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1420,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VM%2B%20CTO%20184%20Tran%20Hung%20Dao%2C%20184%20Tran%20Hung%20Dao%2C%20P.%20An%20Nghiep%2C%20Q.Ninh%20Kieu</t>
+          <t>https://maps.google.com/?q=WinMart+184+Tran+Hung+Dao%2C+P.+An+Nghiep%2C+Q.Ninh+Kieu%2C+TP+Can+Tho</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1461,7 @@
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2090A2-92A2%20KDC%20H%C6%B0ng%20Ph%C3%BA%201%2C%2090A2-92A2%20KDC%20H%C6%B0ng%20Ph%C3%BA%201%2C%20P.%20H%C6%B0ng%20Ph%C3%BA%2C%20Qu%E1%BA%ADn%20C%C3%A1i%20R%C4%83ng</t>
+          <t>https://maps.google.com/?q=WinMart+90A2-92A2+KDC+H%C6%B0ng+Ph%C3%BA+1%2C+P.+H%C6%B0ng+Ph%C3%BA%2C+Qu%E1%BA%ADn+C%C3%A1i+R%C4%83ng%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2083-85%20Nguy%E1%BB%85n%20Hi%E1%BB%81n%2C%2083-85%20Nguy%E1%BB%85n%20Hi%E1%BB%81n%2C%20P.%20An%20Kh%C3%A1nh%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+83-85+Nguy%E1%BB%85n+Hi%E1%BB%81n%2C+P.+An+Kh%C3%A1nh%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1543,7 +1543,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20155%20L%C3%BD%20T%E1%BB%B1%20Tr%E1%BB%8Dng%2C%20155%20L%C3%BD%20T%E1%BB%B1%20Tr%E1%BB%8Dng%2C%20Ph%C6%B0%E1%BB%9Dng%20An%20Ph%C3%BA%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+155+L%C3%BD+T%E1%BB%B1+Tr%E1%BB%8Dng%2C+Ph%C6%B0%E1%BB%9Dng+An+Ph%C3%BA%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1584,7 +1584,7 @@
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2086A%20M%E1%BA%ADu%20Th%C3%A2n%2C%2086%20A%20M%E1%BA%ADu%20Th%C3%A2n%2C%20P.%20An%20H%C3%B2a%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+86A+M%E1%BA%ADu+Th%C3%A2n%2C+86+A+M%E1%BA%ADu+Th%C3%A2n%2C+P.+An+H%C3%B2a%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1625,7 +1625,7 @@
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2018%20%C4%91%C6%B0%E1%BB%9Dng%20A1%2C%2018%20%C4%91%C6%B0%E1%BB%9Dng%20A1%20KDC%20H%C6%B0ng%20Ph%C3%BA%201%2C%20KV9%2C%20P.%20H%C6%B0ng%20Ph%C3%BA%2C%20Qu%E1%BA%ADn%20C%C3%A1i%20R%C4%83ng</t>
+          <t>https://maps.google.com/?q=WinMart+18+%C4%91%C6%B0%E1%BB%9Dng+A1+KDC+H%C6%B0ng+Ph%C3%BA+1%2C+KV9%2C+P.+H%C6%B0ng+Ph%C3%BA%2C+Qu%E1%BA%ADn+C%C3%A1i+R%C4%83ng%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1666,7 @@
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20151/19%20Tr%E1%BA%A7n%20Ho%C3%A0ng%20Na%2C%20151/19%20Tr%E1%BA%A7n%20Ho%C3%A0ng%20Na%2C%20Ph%C6%B0%E1%BB%9Dng%20H%C6%B0ng%20L%E1%BB%A3i%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+151%2F19+Tr%E1%BA%A7n+Ho%C3%A0ng+Na%2C+Ph%C6%B0%E1%BB%9Dng+H%C6%B0ng+L%E1%BB%A3i%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1707,7 +1707,7 @@
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO13-15%20Xu%C3%A2n%20Th%E1%BB%A7y%2C%2013-15%20Xu%C3%A2n%20Th%E1%BB%A7y%2C%20KDC%20C%C3%A1i%20S%C6%A1n-%20H%C3%A0ng%20B%C3%A0ng%2C%20Ph%C6%B0%E1%BB%9Dng%20An%20B%C3%ACnh%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+WM%2B+CTO13-15+Xu%C3%A2n+Th%E1%BB%A7y%2C+13-15+Xu%C3%A2n+Th%E1%BB%A7y%2C+KDC+C%C3%A1i+S%C6%A1n-+H%C3%A0ng+B%C3%A0ng%2C+Ph%C6%B0%E1%BB%9Dng+An+B%C3%ACnh%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1748,7 +1748,7 @@
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2044-46%20B%C3%B9i%20Quang%20Trinh%2C%2044-46%20B%C3%B9i%20Quang%20Trinh%2C%20khu%20d%C3%A2n%20c%C6%B0%20586%2C%20Ph%C6%B0%E1%BB%9Dng%20Ph%C3%BA%20Th%E1%BB%A9%2C%20Qu%E1%BA%ADn%20C%C3%A1i%20R%C4%83ng</t>
+          <t>https://maps.google.com/?q=WinMart+44-46+B%C3%B9i+Quang+Trinh%2C+khu+d%C3%A2n+c%C6%B0+586%2C+Ph%C6%B0%E1%BB%9Dng+Ph%C3%BA+Th%E1%BB%A9%2C+Qu%E1%BA%ADn+C%C3%A1i+R%C4%83ng%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2028%20%C4%91%C6%B0%E1%BB%9Dng%203/2%2C%2028%20%C4%91%C6%B0%E1%BB%9Dng%203/2%2C%20Ph%C6%B0%E1%BB%9Dng%20Ch%C3%A2u%20V%C4%83n%20Li%C3%AAm%2C%20Qu%E1%BA%ADn%20%C3%94%20M%C3%B4n</t>
+          <t>https://maps.google.com/?q=WinMart+28+%C4%91%C6%B0%E1%BB%9Dng+3%2F2%2C+Ph%C6%B0%E1%BB%9Dng+Ch%C3%A2u+V%C4%83n+Li%C3%AAm%2C+Qu%E1%BA%ADn+%C3%94+M%C3%B4n%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1830,7 +1830,7 @@
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%201056%20qu%E1%BB%91c%20l%E1%BB%99%2091%2C%201056%20Qu%E1%BB%91c%20l%E1%BB%99%2091%2C%20Ph%C6%B0%E1%BB%9Dng%20Ch%C3%A2u%20V%C4%83n%20Li%C3%AAm%2C%20Qu%E1%BA%ADn%20%C3%94%20M%C3%B4n</t>
+          <t>https://maps.google.com/?q=WinMart+1056+Qu%E1%BB%91c+l%E1%BB%99+91%2C+Ph%C6%B0%E1%BB%9Dng+Ch%C3%A2u+V%C4%83n+Li%C3%AAm%2C+Qu%E1%BA%ADn+%C3%94+M%C3%B4n%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2051%20%C4%91%C6%B0%E1%BB%9Dng%2026/3%2C%2051%20%C4%91%C6%B0%E1%BB%9Dng%2026/3%2C%20p%2C%20Ph%C6%B0%E1%BB%9Dng%20Ch%C3%A2u%20V%C4%83n%20Li%C3%AAm%2C%20Qu%E1%BA%ADn%20%C3%94%20M%C3%B4n</t>
+          <t>https://maps.google.com/?q=WinMart+51+%C4%91%C6%B0%E1%BB%9Dng+26%2F3%2C+p%2C+Ph%C6%B0%E1%BB%9Dng+Ch%C3%A2u+V%C4%83n+Li%C3%AAm%2C+Qu%E1%BA%ADn+%C3%94+M%C3%B4n%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20140B/1%20Nguy%E1%BB%85n%20V%C4%83n%20C%E1%BB%AB%2C%20140B/1%20Nguy%E1%BB%85n%20V%C4%83n%20C%E1%BB%AB%2C%20P.%20An%20H%C3%B2a%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+140B%2F1+Nguy%E1%BB%85n+V%C4%83n+C%E1%BB%AB%2C+P.+An+H%C3%B2a%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1953,7 +1953,7 @@
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2035%20Nguy%E1%BB%85n%20Ch%C3%AD%20Thanh%2C%2035%20Nguy%E1%BB%85n%20Ch%C3%AD%20Thanh%2C%20Ph%C6%B0%E1%BB%9Dng%20Tr%C3%A0%20N%C3%B3c%2C%20Qu%E1%BA%ADn%20B%C3%ACnh%20Th%E1%BB%A7y</t>
+          <t>https://maps.google.com/?q=WinMart+35+Nguy%E1%BB%85n+Ch%C3%AD+Thanh%2C+Ph%C6%B0%E1%BB%9Dng+Tr%C3%A0+N%C3%B3c%2C+Qu%E1%BA%ADn+B%C3%ACnh+Th%E1%BB%A7y%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VM%2BVLG%2068%20duong%202%20thang%209%2C%2068%20Duong%202%20Thang%209%20Phuong%201%2C%20Thanh%20Pho%20Vinh%20Long%2C%20Tinh%20Vinh%20Long</t>
+          <t>https://maps.google.com/?q=WinMart+VM%2BVLG+68+duong+2+thang+9%2C+68+Duong+2+Thang+9+Phuong+1%2C+Thanh+Pho+Vinh+Long%2C+Tinh+Vinh+Long</t>
         </is>
       </c>
     </row>
@@ -2035,7 +2035,7 @@
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2BVLG%2033/15D%20Ph%E1%BA%A1m%20Th%C3%A1i%20B%C6%B0%E1%BB%9Dng%2C%2033/15D%20Ph%E1%BA%A1m%20Th%C3%A1i%20B%C6%B0%E1%BB%9Dng%2CPh%C6%B0%E1%BB%9Dng%204%2C%20Th%C3%A0nh%20ph%E1%BB%91%20V%C4%A9nh%20Long</t>
+          <t>https://maps.google.com/?q=WinMart+WM%2BVLG+33%2F15D+Ph%E1%BA%A1m+Th%C3%A1i+B%C6%B0%E1%BB%9Dng%2C+33%2F15D+Ph%E1%BA%A1m+Th%C3%A1i+B%C6%B0%E1%BB%9Dng%2CPh%C6%B0%E1%BB%9Dng+4%2C+Th%C3%A0nh+ph%E1%BB%91+V%C4%A9nh+Long</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2076,7 @@
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20VLG%2001%20M%E1%BA%ADu%20Th%C3%A2n%2C%2001%20M%E1%BA%ADu%20Th%C3%A2n%2C%20Ph%C6%B0%E1%BB%9Dng%203%2C%20Th%C3%A0nh%20ph%E1%BB%91%20V%C4%A9nh%20Long</t>
+          <t>https://maps.google.com/?q=WinMart+01+M%E1%BA%ADu+Th%C3%A2n%2C+Ph%C6%B0%E1%BB%9Dng+3%2C+Th%C3%A0nh+ph%E1%BB%91+V%C4%A9nh+Long</t>
         </is>
       </c>
     </row>
@@ -2117,7 +2117,7 @@
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VM%2B%20KGG%20Lo%20so%20F14-30%2C%20duong%203/2%2C%20Lo%20so%20F14-30%2C%20duong%203/2%2C%20thuoc%20du%20an%20lan%20bien%20xay%20dung%20khu%20do%20thi%20moi%2C%20TP%20Rach%20Gia%2C%20Kien%20Giang</t>
+          <t>https://maps.google.com/?q=WinMart+Lo+so+F14-30%2C+duong+3%2F2%2C+thuoc+du+an+lan+bien+xay+dung+khu+do+thi+moi%2C+TP+Rach+Gia%2C+Kien+Giang</t>
         </is>
       </c>
     </row>
@@ -2158,7 +2158,7 @@
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20KGG%2007-07A%20Nguy%E1%BB%85n%20B%E1%BB%89nh%20Khi%C3%AAm%2C%2007%20%E2%80%93%2007A%20Nguy%E1%BB%85n%20B%E1%BB%89nh%20Khi%C3%AAm%2C%20P.%20V%C4%A9nh%20Thanh%2C%20Th%C3%A0nh%20ph%E1%BB%91%20R%E1%BA%A1ch%20Gi%C3%A1</t>
+          <t>https://maps.google.com/?q=WinMart+07-07A+Nguy%E1%BB%85n+B%E1%BB%89nh+Khi%C3%AAm%2C+07+%E2%80%93+07A+Nguy%E1%BB%85n+B%E1%BB%89nh+Khi%C3%AAm%2C+P.+V%C4%A9nh+Thanh%2C+Th%C3%A0nh+ph%E1%BB%91+R%E1%BA%A1ch+Gi%C3%A1</t>
         </is>
       </c>
     </row>
@@ -2199,7 +2199,7 @@
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20KGG%20L%C3%B4%20s%E1%BB%91%20D4-25%2C%20%C4%91%C6%B0%E1%BB%9Dng%203/2%2C%20L%C3%B4%20s%E1%BB%91%20D4-25%2C%20%C4%91%C6%B0%E1%BB%9Dng%203/2%2C%20Ph%C6%B0%E1%BB%9Dng%20V%C4%A9nh%20L%E1%BA%A1c%2C%20Th%C3%A0nh%20ph%E1%BB%91%20R%E1%BA%A1ch%20Gi%C3%A1</t>
+          <t>https://maps.google.com/?q=WinMart+L%C3%B4+s%E1%BB%91+D4-25%2C+%C4%91%C6%B0%E1%BB%9Dng+3%2F2%2C+Ph%C6%B0%E1%BB%9Dng+V%C4%A9nh+L%E1%BA%A1c%2C+Th%C3%A0nh+ph%E1%BB%91+R%E1%BA%A1ch+Gi%C3%A1</t>
         </is>
       </c>
     </row>
@@ -2240,7 +2240,7 @@
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20KGG%2021%20Nguy%E1%BB%85n%20V%C4%83n%20C%E1%BB%AB%2C%2021%20Nguy%E1%BB%85n%20V%C4%83n%20C%E1%BB%AB%2C%20KP%201%2C%20P%20An%20H%C3%B2a%2C%20Th%C3%A0nh%20ph%E1%BB%91%20R%E1%BA%A1ch%20Gi%C3%A1</t>
+          <t>https://maps.google.com/?q=WinMart+21+Nguy%E1%BB%85n+V%C4%83n+C%E1%BB%AB%2C+KP+1%2C+P+An+H%C3%B2a%2C+Th%C3%A0nh+ph%E1%BB%91+R%E1%BA%A1ch+Gi%C3%A1</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2281,7 @@
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20KGG%2014%20Tr%E1%BA%A7n%20Quang%20Kh%E1%BA%A3i%2C%2014%20Tr%E1%BA%A7n%20Quang%20Kh%E1%BA%A3i%2C%20Ph%C6%B0%E1%BB%9Dng%20An%20H%C3%B2a%2C%20Th%C3%A0nh%20ph%E1%BB%91%20R%E1%BA%A1ch%20Gi%C3%A1</t>
+          <t>https://maps.google.com/?q=WinMart+14+Tr%E1%BA%A7n+Quang+Kh%E1%BA%A3i%2C+Ph%C6%B0%E1%BB%9Dng+An+H%C3%B2a%2C+Th%C3%A0nh+ph%E1%BB%91+R%E1%BA%A1ch+Gi%C3%A1</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2BVLG%2027A%20L%C3%AA%20V%C4%83n%20T%C3%A1m%2C%2027A%20L%C3%AA%20V%C4%83n%20T%C3%A1m%2C%20Ph%C6%B0%E1%BB%9Dng%201%2C%20Th%C3%A0nh%20ph%E1%BB%91%20V%C4%A9nh%20Long</t>
+          <t>https://maps.google.com/?q=WinMart+WM%2BVLG+27A+L%C3%AA+V%C4%83n+T%C3%A1m%2C+27A+L%C3%AA+V%C4%83n+T%C3%A1m%2C+Ph%C6%B0%E1%BB%9Dng+1%2C+Th%C3%A0nh+ph%E1%BB%91+V%C4%A9nh+Long</t>
         </is>
       </c>
     </row>
@@ -2363,7 +2363,7 @@
       </c>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20KGG%2037%20%C4%91%C6%B0%E1%BB%9Dng%203/2%2C%2037%20%C4%91%C6%B0%E1%BB%9Dng%203/2%2C%20Ph%C6%B0%E1%BB%9Dng%20V%C4%A9nh%20Thanh%20V%C3%A2n%2C%20Th%C3%A0nh%20ph%E1%BB%91%20R%E1%BA%A1ch%20Gi%C3%A1</t>
+          <t>https://maps.google.com/?q=WinMart+37+%C4%91%C6%B0%E1%BB%9Dng+3%2F2%2C+Ph%C6%B0%E1%BB%9Dng+V%C4%A9nh+Thanh+V%C3%A2n%2C+Th%C3%A0nh+ph%E1%BB%91+R%E1%BA%A1ch+Gi%C3%A1</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20KGG%2079%20Quang%20Trung%2C%2079%20Quang%20Trung%2C%20Ph%C6%B0%E1%BB%9Dng%20V%C4%A9nh%20Quang%2C%20Th%C3%A0nh%20ph%E1%BB%91%20R%E1%BA%A1ch%20Gi%C3%A1</t>
+          <t>https://maps.google.com/?q=WinMart+79+Quang+Trung%2C+Ph%C6%B0%E1%BB%9Dng+V%C4%A9nh+Quang%2C+Th%C3%A0nh+ph%E1%BB%91+R%E1%BA%A1ch+Gi%C3%A1</t>
         </is>
       </c>
     </row>
@@ -2445,7 +2445,7 @@
       </c>
       <c r="I48" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VM%2B%20KGG%20208%20Nguyen%20Binh%20Khiem%2C%20208%20duong%20Nguyen%20Binh%20Khiem%2C%20KP%20Dong%20Khoi%2C%20Phuong%20Vinh%20Quang%2C%20TX%20Rach%20Gia%2C%20Tinh%20Kien%20Giang</t>
+          <t>https://maps.google.com/?q=WinMart+208+Nguyen+Binh+Khiem%2C+208+duong+Nguyen+Binh+Khiem%2C+KP+Dong+Khoi%2C+Phuong+Vinh+Quang%2C+TX+Rach+Gia%2C+Tinh+Kien+Giang</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20Th%E1%BB%ADa%201717%2C%20TB%C4%90%207%20V%C5%A9%20%C4%90%C3%ACnh%20Li%2C%20Th%E1%BB%ADa%20%C4%91%E1%BA%A5t%201717%2C%20TB%C4%90%20s%E1%BB%91%207%2C%20%C4%90%C6%B0%E1%BB%9Dng%20V%C5%A9%2C%20%C4%90%C3%ACnh%20Li%E1%BB%87u%2C%20KDC%20L%C3%B4%20S%E1%BB%91%208B%2C%20KDT%20Nam%2C%20C%E1%BA%A7n%20Th%C6%A1%2C%20P.%20H%C6%B0ng%20Th%E1%BA%A1nh%2C%20Q.%20C%C3%A1i%20R%C4%83ng</t>
+          <t>https://maps.google.com/?q=WinMart+Th%E1%BB%ADa+1717%2C+TB%C4%90+7+V%C5%A9+%C4%90%C3%ACnh+Li%2C+Th%E1%BB%ADa+%C4%91%E1%BA%A5t+1717%2C+TB%C4%90+s%E1%BB%91+7%2C+%C4%90%C6%B0%E1%BB%9Dng+V%C5%A9%2C+%C4%90%C3%ACnh+Li%E1%BB%87u%2C+KDC+L%C3%B4+S%E1%BB%91+8B%2C+KDT+Nam%2C+C%E1%BA%A7n+Th%C6%A1%2C+P.+H%C6%B0ng+Th%E1%BA%A1nh%2C+Q.+C%C3%A1i+R%C4%83ng%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -2527,7 +2527,7 @@
       </c>
       <c r="I50" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20KGG%20L%C3%B4%20L7%20%E2%80%93%206%20Hu%E1%BB%B3nh%20Th%C3%BAc%20Kh%C3%A1ng%2C%20L%C3%B4%20L7%20%E2%80%93%206%20Hu%E1%BB%B3nh%20Th%C3%BAc%20Kh%C3%A1ng%2C%20P.%20V%C4%A9nh%20Quang%2C%20Th%C3%A0nh%20ph%E1%BB%91%20R%E1%BA%A1ch%20Gi%C3%A1</t>
+          <t>https://maps.google.com/?q=WinMart+L%C3%B4+L7+%E2%80%93+6+Hu%E1%BB%B3nh+Th%C3%BAc+Kh%C3%A1ng%2C+P.+V%C4%A9nh+Quang%2C+Th%C3%A0nh+ph%E1%BB%91+R%E1%BA%A1ch+Gi%C3%A1</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VM%2B%20KGG%206%20Mai%20Thi%20Hong%20Hanh%2C%206%20Mai%20Thi%20Hong%20Hanh%2C%20KP%201%2C%20P%20Rach%20Soi%2C%20TP%20Rach%20Gia%2C%20Tinh%20Kien%20Giang</t>
+          <t>https://maps.google.com/?q=WinMart+6+Mai+Thi+Hong+Hanh%2C+KP+1%2C+P+Rach+Soi%2C+TP+Rach+Gia%2C+Tinh+Kien+Giang</t>
         </is>
       </c>
     </row>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="I52" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20303%20Nguy%E1%BB%85n%20V%C4%83n%20Linh%2C%20303%20Nguy%E1%BB%85n%20V%C4%83n%20Linh%2C%20KV%204%2C%20Ph%C6%B0%E1%BB%9Dng%20An%20Kh%C3%A1nh%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+303+Nguy%E1%BB%85n+V%C4%83n+Linh%2C+KV+4%2C+Ph%C6%B0%E1%BB%9Dng+An+Kh%C3%A1nh%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -2650,7 +2650,7 @@
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20158%20%C4%91%C6%B0%E1%BB%9Dng%2030/4%2C%20158%20%C4%91%C6%B0%E1%BB%9Dng%2030/4%2C%20Ph%C6%B0%E1%BB%9Dng%20An%20Ph%C3%BA%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+158+%C4%91%C6%B0%E1%BB%9Dng+30%2F4%2C+Ph%C6%B0%E1%BB%9Dng+An+Ph%C3%BA%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       </c>
       <c r="I54" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20399%20Nguy%E1%BB%85n%20%C4%90%E1%BB%87%2C%20399%20Nguy%E1%BB%85n%20%C4%90%E1%BB%87%2C%20P.%20An%20H%C3%B2a%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+399+Nguy%E1%BB%85n+%C4%90%E1%BB%87%2C+P.+An+H%C3%B2a%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -2732,7 +2732,7 @@
       </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20365/14%20Nguy%E1%BB%85n%20V%C4%83n%20C%E1%BB%AB%2C%20365/14%20Nguy%E1%BB%85n%20V%C4%83n%20C%E1%BB%AB%2C%20Ph%C6%B0%E1%BB%9Dng%20An%20Kh%C3%A1nh%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+365%2F14+Nguy%E1%BB%85n+V%C4%83n+C%E1%BB%AB%2C+Ph%C6%B0%E1%BB%9Dng+An+Kh%C3%A1nh%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -2773,7 +2773,7 @@
       </c>
       <c r="I56" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20100-%20102%20Nguy%E1%BB%85n%20Tri%20Ph%C6%B0%C6%A1ng%2C%20100-%20102%20Nguy%E1%BB%85n%20Tri%20Ph%C6%B0%C6%A1ng%2C%20Ph%C6%B0%E1%BB%9Dng%20An%20Kh%C3%A1nh%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+100-+102+Nguy%E1%BB%85n+Tri+Ph%C6%B0%C6%A1ng%2C+Ph%C6%B0%E1%BB%9Dng+An+Kh%C3%A1nh%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -2814,7 +2814,7 @@
       </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20KGG%20186%20-188%20Nguy%E1%BB%85n%20H%C3%B9ng%20S%C6%A1n%2C%20186%20-188%20Nguy%E1%BB%85n%20H%C3%B9ng%20S%C6%A1n%2C%20KP%202%2C%20P.%20V%C4%A9nh%20Thanh%20V%C3%A2n%2C%20Th%C3%A0nh%20ph%E1%BB%91%20R%E1%BA%A1ch%20Gi%C3%A1</t>
+          <t>https://maps.google.com/?q=WinMart+186+-188+Nguy%E1%BB%85n+H%C3%B9ng+S%C6%A1n%2C+KP+2%2C+P.+V%C4%A9nh+Thanh+V%C3%A2n%2C+Th%C3%A0nh+ph%E1%BB%91+R%E1%BA%A1ch+Gi%C3%A1</t>
         </is>
       </c>
     </row>
@@ -2855,7 +2855,7 @@
       </c>
       <c r="I58" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20KGG%20327%20Nguy%E1%BB%85n%20Trung%20Tr%E1%BB%B1c%2C%20327%20%C4%91%C6%B0%E1%BB%9Dng%20Nguy%E1%BB%85n%20Trung%20Tr%E1%BB%B1c%2C%20Ph%C6%B0%E1%BB%9Dng%20V%C4%A9nh%20L%E1%BA%A1c%2C%20Th%C3%A0nh%20ph%E1%BB%91%20R%E1%BA%A1ch%20Gi%C3%A1</t>
+          <t>https://maps.google.com/?q=WinMart+327+Nguy%E1%BB%85n+Trung+Tr%E1%BB%B1c%2C+327+%C4%91%C6%B0%E1%BB%9Dng+Nguy%E1%BB%85n+Trung+Tr%E1%BB%B1c%2C+Ph%C6%B0%E1%BB%9Dng+V%C4%A9nh+L%E1%BA%A1c%2C+Th%C3%A0nh+ph%E1%BB%91+R%E1%BA%A1ch+Gi%C3%A1</t>
         </is>
       </c>
     </row>
@@ -2896,7 +2896,7 @@
       </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20VLG%2086%20Nguy%E1%BB%85n%20Hu%E1%BB%87%2C%2086%20Nguy%E1%BB%85n%20Hu%E1%BB%87%2C%20Ph%C6%B0%E1%BB%9Dng%202%2C%20Th%C3%A0nh%20ph%E1%BB%91%20V%C4%A9nh%20Long</t>
+          <t>https://maps.google.com/?q=WinMart+86+Nguy%E1%BB%85n+Hu%E1%BB%87%2C+Ph%C6%B0%E1%BB%9Dng+2%2C+Th%C3%A0nh+ph%E1%BB%91+V%C4%A9nh+Long</t>
         </is>
       </c>
     </row>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="I60" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2043-45%20V%C3%B5%20Tr%C6%B0%E1%BB%9Dng%20To%E1%BA%A3n%2C%2043-45%20V%C3%B5%20Tr%C6%B0%E1%BB%9Dng%20To%E1%BA%A3n%2C%20P.%20An%20H%C3%B2a%2C%20Q.%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+43-45+V%C3%B5+Tr%C6%B0%E1%BB%9Dng+To%E1%BA%A3n%2C+P.+An+H%C3%B2a%2C+Q.+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -2978,7 +2978,7 @@
       </c>
       <c r="I61" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20131%20-%20133%20%C4%90%E1%BB%93ng%20V%C4%83n%20C%E1%BB%91ng%2C%20131%20%E2%80%93%20133%20%C4%90%E1%BB%93ng%20V%C4%83n%20C%E1%BB%91ng%2C%20P.%20An%20Th%E1%BB%9Bi%2C%20Q.%20B%C3%ACnh%20Th%E1%BB%A7y</t>
+          <t>https://maps.google.com/?q=WinMart+131+-+133+%C4%90%E1%BB%93ng+V%C4%83n+C%E1%BB%91ng%2C+131+%E2%80%93+133+%C4%90%E1%BB%93ng+V%C4%83n+C%E1%BB%91ng%2C+P.+An+Th%E1%BB%9Bi%2C+Q.+B%C3%ACnh+Th%E1%BB%A7y%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -3019,7 +3019,7 @@
       </c>
       <c r="I62" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20VLG%2080%20Nguy%E1%BB%85n%20V%C4%83n%20Th%E1%BA%A3nh%2C%2080%20Nguy%E1%BB%85n%20V%C4%83n%20Th%E1%BA%A3nh%2C%20Kh%C3%B3m%205%2C%20P.%20C%C3%A1i%20V%E1%BB%93n%2C%20Th%E1%BB%8B%20x%C3%A3%20B%C3%ACnh%20Minh</t>
+          <t>https://maps.google.com/?q=WinMart+80+Nguy%E1%BB%85n+V%C4%83n+Th%E1%BA%A3nh%2C+Kh%C3%B3m+5%2C+P.+C%C3%A1i+V%E1%BB%93n%2C+Th%E1%BB%8B+x%C3%A3+B%C3%ACnh+Minh</t>
         </is>
       </c>
     </row>
@@ -3060,7 +3060,7 @@
       </c>
       <c r="I63" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2081B/2%20%C4%91%C6%B0%E1%BB%9Dng%20M%E1%BA%A1c%20Thi%C3%AAn%20T%C3%ADch%2C%2081B/2%2C%20M%E1%BA%A1c%20Thi%C3%AAn%20T%C3%ADch%2C%20P.%20Xu%C3%A2n%20Kh%C3%A1nh%2C%20Q.%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+81B%2F2+%C4%91%C6%B0%E1%BB%9Dng+M%E1%BA%A1c+Thi%C3%AAn+T%C3%ADch%2C+81B%2F2%2C+M%E1%BA%A1c+Thi%C3%AAn+T%C3%ADch%2C+P.+Xu%C3%A2n+Kh%C3%A1nh%2C+Q.+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -3101,7 +3101,7 @@
       </c>
       <c r="I64" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20KGG%20841%20Nguy%E1%BB%85n%20Trung%20Tr%E1%BB%B1c%2C%20841%20Nguy%E1%BB%85n%20Trung%20Tr%E1%BB%B1c%2C%20KP%205%2C%20P.%20An%20B%C3%ACnh%2C%20TP.%20R%E1%BA%A1ch%20Gi%C3%A1</t>
+          <t>https://maps.google.com/?q=WinMart+841+Nguy%E1%BB%85n+Trung+Tr%E1%BB%B1c%2C+KP+5%2C+P.+An+B%C3%ACnh%2C+TP.+R%E1%BA%A1ch+Gi%C3%A1</t>
         </is>
       </c>
     </row>
@@ -3142,7 +3142,7 @@
       </c>
       <c r="I65" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20KGG%20L%C3%B4%20P2%20%E2%80%93%2036%20%2B%2037%20%C4%90%C6%B0%E1%BB%9Dng%203/2%2C%20L%C3%B4%20P2%20%E2%80%93%2036%20%2B%2037%20%C4%90%C6%B0%E1%BB%9Dng%203/2%2C%20P.%20An%20H%C3%B2a%2C%20TP.%20R%E1%BA%A1ch%20Gi%C3%A1</t>
+          <t>https://maps.google.com/?q=WinMart+L%C3%B4+P2+%E2%80%93+36+%2B+37+%C4%90%C6%B0%E1%BB%9Dng+3%2F2%2C+P.+An+H%C3%B2a%2C+TP.+R%E1%BA%A1ch+Gi%C3%A1</t>
         </is>
       </c>
     </row>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="I66" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2056%20Nguy%E1%BB%85n%20V%C4%83n%20C%E1%BB%AB%2C%2056%20Nguy%E1%BB%85n%20V%C4%83n%20C%E1%BB%AB%2C%20Khu%20v%E1%BB%B1c%203%20S%C3%B4ng%20H%E1%BA%ADu%2C%20P.%20C%C3%A1i%20Kh%E1%BA%BF%2C%20Q.%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+56+Nguy%E1%BB%85n+V%C4%83n+C%E1%BB%AB%2C+Khu+v%E1%BB%B1c+3+S%C3%B4ng+H%E1%BA%ADu%2C+P.+C%C3%A1i+Kh%E1%BA%BF%2C+Q.+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -3224,7 +3224,7 @@
       </c>
       <c r="I67" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20VLG%2079/9%20Ph%C3%B3%20C%C6%A1%20%C4%90i%E1%BB%81u%2C%2079/9B%20Ph%C3%B3%20C%C6%A1%20%C4%90i%E1%BB%81u%2C%20P.%203%2C%20TP.%20V%C4%A9nh%20Long</t>
+          <t>https://maps.google.com/?q=WinMart+79%2F9+Ph%C3%B3+C%C6%A1+%C4%90i%E1%BB%81u%2C+79%2F9B+Ph%C3%B3+C%C6%A1+%C4%90i%E1%BB%81u%2C+P.+3%2C+TP.+V%C4%A9nh+Long</t>
         </is>
       </c>
     </row>
@@ -3265,7 +3265,7 @@
       </c>
       <c r="I68" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2095/31%20Nguy%E1%BB%85n%20Th%C3%B4ng%2C%2095%20Nguy%E1%BB%85n%20Th%C3%B4ng%2C%20P.%20An%20Th%E1%BB%9Bi%2C%20Q.%20B%C3%ACnh%20Th%E1%BB%A7y</t>
+          <t>https://maps.google.com/?q=WinMart+95%2F31+Nguy%E1%BB%85n+Th%C3%B4ng%2C+95+Nguy%E1%BB%85n+Th%C3%B4ng%2C+P.+An+Th%E1%BB%9Bi%2C+Q.+B%C3%ACnh+Th%E1%BB%A7y%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -3306,7 +3306,7 @@
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20369/14%20KDC%20B%C3%ACnh%20Nh%E1%BB%B1t%2C%20369/14%20KDC%20B%C3%ACnh%20Nh%E1%BB%B1t%2C%20P.%20Long%20H%C3%B2a%2C%20Q.%20B%C3%ACnh%20Th%E1%BB%A7y</t>
+          <t>https://maps.google.com/?q=WinMart+369%2F14+KDC+B%C3%ACnh+Nh%E1%BB%B1t%2C+P.+Long+H%C3%B2a%2C+Q.+B%C3%ACnh+Th%E1%BB%A7y%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="I70" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2024A%20H%E1%BB%93%20Trung%20Th%C3%A0nh%2C%2024A%20%C4%90%C6%B0%E1%BB%9Dng%20H%E1%BB%93%20Trung%20Th%C3%A0nh%2C%20KV3%20%2C%20Tr%C3%A0%20An%2C%20Q.%20B%C3%ACnh%20Th%E1%BB%A7y</t>
+          <t>https://maps.google.com/?q=WinMart+24A+H%E1%BB%93+Trung+Th%C3%A0nh%2C+24A+%C4%90%C6%B0%E1%BB%9Dng+H%E1%BB%93+Trung+Th%C3%A0nh%2C+KV3+%2C+Tr%C3%A0+An%2C+Q.+B%C3%ACnh+Th%E1%BB%A7y%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -3388,7 +3388,7 @@
       </c>
       <c r="I71" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20KGG%20212%20Ng%C3%B4%20Quy%E1%BB%81n%2C%20212%20Ng%C3%B4%20Quy%E1%BB%81n%2C%20P.%20V%C4%A9nh%20B%E1%BA%A3o%2C%20TP.%20R%E1%BA%A1ch%20Gi%C3%A1</t>
+          <t>https://maps.google.com/?q=WinMart+212+Ng%C3%B4+Quy%E1%BB%81n%2C+P.+V%C4%A9nh+B%E1%BA%A3o%2C+TP.+R%E1%BA%A1ch+Gi%C3%A1</t>
         </is>
       </c>
     </row>
@@ -3429,7 +3429,7 @@
       </c>
       <c r="I72" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20KGG%20686%20M%E1%BA%A1c%20C%E1%BB%ADu%2C%20686%20M%E1%BA%A1c%20C%E1%BB%ADu%2C%20P.%20V%C4%A9nh%20Quang%2C%20TP.%20R%E1%BA%A1ch%20Gi%C3%A1</t>
+          <t>https://maps.google.com/?q=WinMart+686+M%E1%BA%A1c+C%E1%BB%ADu%2C+P.+V%C4%A9nh+Quang%2C+TP.+R%E1%BA%A1ch+Gi%C3%A1</t>
         </is>
       </c>
     </row>
@@ -3470,7 +3470,7 @@
       </c>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2051D1%20%C4%90%C6%B0%E1%BB%9Dng%203/2%2C%2051D1%20%C4%90%C6%B0%E1%BB%9Dng%203/2%2C%20Ph%C6%B0%E1%BB%9Dng%20Xu%C3%A2n%20Kh%C3%A1nh%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+51D1+%C4%90%C6%B0%E1%BB%9Dng+3%2F2%2C+Ph%C6%B0%E1%BB%9Dng+Xu%C3%A2n+Kh%C3%A1nh%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -3511,7 +3511,7 @@
       </c>
       <c r="I74" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2091%20Tr%E1%BA%A7n%20V%C4%83n%20Long%2C%2091%20Tr%E1%BA%A7n%20V%C4%83n%20Long%2C%20KV1%2C%20Khu%20T%C4%90C%20Th%E1%BB%9Bi%20Nh%E1%BB%B1t%202%2C%20P.%20An%20Kh%C3%A1nh</t>
+          <t>https://maps.google.com/?q=WinMart+91+Tr%E1%BA%A7n+V%C4%83n+Long%2C+KV1%2C+Khu+T%C4%90C+Th%E1%BB%9Bi+Nh%E1%BB%B1t+2%2C+P.+An+Kh%C3%A1nh%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -3552,7 +3552,7 @@
       </c>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2031-33%20%E1%BA%A4p%20Th%E1%BB%8B%20T%E1%BB%A9%2C%2031-33%20%E1%BA%A4p%20Th%E1%BB%8B%20T%E1%BB%A9%2C%20TT.%20Phong%20%C4%90i%E1%BB%81n</t>
+          <t>https://maps.google.com/?q=WinMart+31-33+%E1%BA%A4p+Th%E1%BB%8B+T%E1%BB%A9%2C+TT.+Phong+%C4%90i%E1%BB%81n%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -3593,7 +3593,7 @@
       </c>
       <c r="I76" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20KGG%20250%20L%C3%A2m%20Quang%20Ky%2C%20250%20L%C3%A2m%20Quang%20Ky%2C%20Khu%20Ph%E1%BB%91%205%2C%20Ph%C6%B0%E1%BB%9Dng%20V%C4%A9nh%20B%E1%BA%A3o%2C%20TP.%20R%E1%BA%A1ch%20Gi%C3%A1</t>
+          <t>https://maps.google.com/?q=WinMart+250+L%C3%A2m+Quang+Ky%2C+Khu+Ph%E1%BB%91+5%2C+Ph%C6%B0%E1%BB%9Dng+V%C4%A9nh+B%E1%BA%A3o%2C+TP.+R%E1%BA%A1ch+Gi%C3%A1</t>
         </is>
       </c>
     </row>
@@ -3634,7 +3634,7 @@
       </c>
       <c r="I77" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20VLG%2046C%20%C4%90inh%20Ti%C3%AAn%20Ho%C3%A0ng%2C%2046C%20%C4%90inh%20Ti%C3%AAn%20Ho%C3%A0ng%2C%20P.%208%2C%20TP.%20V%C4%A9nh%20Long</t>
+          <t>https://maps.google.com/?q=WinMart+46C+%C4%90inh+Ti%C3%AAn+Ho%C3%A0ng%2C+P.+8%2C+TP.+V%C4%A9nh+Long</t>
         </is>
       </c>
     </row>
@@ -3675,7 +3675,7 @@
       </c>
       <c r="I78" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20KGG%20Qu%E1%BB%91c%20l%E1%BB%99%2063%20T%E1%BA%AFc%20C%E1%BA%ADu%2C%20T%C4%90%202001%2C%20TB%C4%90%2003%2C%20Qu%E1%BB%91c%20l%E1%BB%99%2063%20T%E1%BA%AFc%20C%E1%BA%ADu%2C%20%E1%BA%A4p%20An%20B%C3%ACnh%2C%20X.%20B%C3%ACnh%20An%2C%20H.%20Ch%C3%A2u%20Th%C3%A0nh</t>
+          <t>https://maps.google.com/?q=WinMart+T%C4%90+2001%2C+TB%C4%90+03%2C+Qu%E1%BB%91c+l%E1%BB%99+63+T%E1%BA%AFc+C%E1%BA%ADu%2C+%E1%BA%A4p+An+B%C3%ACnh%2C+X.+B%C3%ACnh+An%2C+H.+Ch%C3%A2u+Th%C3%A0nh</t>
         </is>
       </c>
     </row>
@@ -3716,7 +3716,7 @@
       </c>
       <c r="I79" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20162/1%20Ph%E1%BA%A1m%20Ng%C5%A9%20L%C3%A3o%2C%20162/1%20Ph%E1%BA%A1m%20Ng%C5%A9%20L%C3%A3o%2C%20P.%20An%20H%C3%B2a%2C%20Q.%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+162%2F1+Ph%E1%BA%A1m+Ng%C5%A9+L%C3%A3o%2C+P.+An+H%C3%B2a%2C+Q.+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -3757,7 +3757,7 @@
       </c>
       <c r="I80" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20106%20%E2%80%93%20108%20Tr%E1%BA%A7n%20B%E1%BA%A1ch%20%C4%90%E1%BA%B1ng%2C%20106%20-%20108%20Tr%E1%BA%A7n%20B%E1%BA%A1ch%20%C4%90%E1%BA%B1ng%2C%20Ph%C6%B0%E1%BB%9Dng%20An%20Kh%C3%A1nh%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+106+%E2%80%93+108+Tr%E1%BA%A7n+B%E1%BA%A1ch+%C4%90%E1%BA%B1ng%2C+106+-+108+Tr%E1%BA%A7n+B%E1%BA%A1ch+%C4%90%E1%BA%B1ng%2C+Ph%C6%B0%E1%BB%9Dng+An+Kh%C3%A1nh%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -3798,7 +3798,7 @@
       </c>
       <c r="I81" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20KGG%2024%20M%E1%BA%A1c%20C%E1%BB%ADu%2C%2024%20M%E1%BA%A1c%20C%E1%BB%ADu%2C%20KP.%20C%C6%B0%20X%C3%A1%20M%E1%BB%9Bi%2C%20TT.%20Ki%C3%AAn%20L%C6%B0%C6%A1ng%2C%20H.%20Ki%C3%AAn%20L%C6%B0%C6%A1ng%2C%20T.</t>
+          <t>https://maps.google.com/?q=WinMart+24+M%E1%BA%A1c+C%E1%BB%ADu%2C+KP.+C%C6%B0+X%C3%A1+M%E1%BB%9Bi%2C+TT.+Ki%C3%AAn+L%C6%B0%C6%A1ng%2C+H.+Ki%C3%AAn+L%C6%B0%C6%A1ng%2C+T.</t>
         </is>
       </c>
     </row>
@@ -3839,7 +3839,7 @@
       </c>
       <c r="I82" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20KGG%20537%20Qu%E1%BB%91c%20l%E1%BB%99%2080%2C%20537%20Qu%E1%BB%91c%20l%E1%BB%99%2080%2C%20%E1%BA%A4p%20Thu%E1%BA%ADn%20H%C3%B2a%2C%20X.%20B%C3%ACnh%20S%C6%A1n%2C%20H.%20H%C3%B2n%20%C4%90%E1%BA%A5t%2C%20T.%20Ki</t>
+          <t>https://maps.google.com/?q=WinMart+537+Qu%E1%BB%91c+l%E1%BB%99+80%2C+%E1%BA%A4p+Thu%E1%BA%ADn+H%C3%B2a%2C+X.+B%C3%ACnh+S%C6%A1n%2C+H.+H%C3%B2n+%C4%90%E1%BA%A5t%2C+T.+Ki</t>
         </is>
       </c>
     </row>
@@ -3880,7 +3880,7 @@
       </c>
       <c r="I83" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20695%20L%C3%AA%20Th%E1%BB%8B%20T%E1%BA%A1o%2C%20695%20L%C3%AA%20Th%E1%BB%8B%20T%E1%BA%A1o%2C%20P%2C%20Th%E1%BB%91t%20N%E1%BB%91t%2C%20Q%2C%20Th%E1%BB%91t%20N%E1%BB%91t</t>
+          <t>https://maps.google.com/?q=WinMart+695+L%C3%AA+Th%E1%BB%8B+T%E1%BA%A1o%2C+P%2C+Th%E1%BB%91t+N%E1%BB%91t%2C+Q%2C+Th%E1%BB%91t+N%E1%BB%91t%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -3921,7 +3921,7 @@
       </c>
       <c r="I84" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20KGG%2039%20M%E1%BA%A1c%20C%E1%BB%ADu%2C%2039%20M%E1%BA%A1c%20C%E1%BB%ADu%2C%20P.%20V%C4%A9nh%20Thanh%2C%20TP.%20R%E1%BA%A1ch%20Gi%C3%A1</t>
+          <t>https://maps.google.com/?q=WinMart+39+M%E1%BA%A1c+C%E1%BB%ADu%2C+P.+V%C4%A9nh+Thanh%2C+TP.+R%E1%BA%A1ch+Gi%C3%A1</t>
         </is>
       </c>
     </row>
@@ -3962,7 +3962,7 @@
       </c>
       <c r="I85" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2009%20Tr%E1%BA%A7n%20V%C4%A9nh%20Ki%E1%BA%BFt%2C%2009%20Tr%E1%BA%A7n%20V%C4%A9nh%20Ki%E1%BA%BFt%2C%20P.%20An%20B%C3%ACnh%2C%20Q.%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+09+Tr%E1%BA%A7n+V%C4%A9nh+Ki%E1%BA%BFt%2C+P.+An+B%C3%ACnh%2C+Q.+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -4003,7 +4003,7 @@
       </c>
       <c r="I86" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20KGG%20232%20%C4%90T%20971%2C%20232%20%C4%90T%20971%2C%20t%E1%BB%95%2013%2C%20KP.%20Ki%C3%AAn%20T%C3%A2n%2C%20TT.%20Ki%C3%AAn%20L%C6%B0%C6%A1ng%2C%20H.%20Ki%C3%AAn%20L%C6%B0%C6%A1ng</t>
+          <t>https://maps.google.com/?q=WinMart+232+%C4%90T+971%2C+t%E1%BB%95+13%2C+KP.+Ki%C3%AAn+T%C3%A2n%2C+TT.+Ki%C3%AAn+L%C6%B0%C6%A1ng%2C+H.+Ki%C3%AAn+L%C6%B0%C6%A1ng</t>
         </is>
       </c>
     </row>
@@ -4044,7 +4044,7 @@
       </c>
       <c r="I87" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20118%20%C4%90%C6%B0%E1%BB%9Dng%20Nguy%E1%BB%85n%20V%C4%83n%20C%E1%BB%AB%20N%E1%BB%91i%20D%C3%A0i%2C%20116%20%C4%90%C6%B0%E1%BB%9Dng%20Nguy%E1%BB%85n%20V%C4%83n%20C%E1%BB%AB%20N%E1%BB%91i%20D%C3%A0i%2C%20P.%20An%20B%C3%ACnh%2C%20Q.%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+118+%C4%90%C6%B0%E1%BB%9Dng+Nguy%E1%BB%85n+V%C4%83n+C%E1%BB%AB+N%E1%BB%91i+D%C3%A0i%2C+116+%C4%90%C6%B0%E1%BB%9Dng+Nguy%E1%BB%85n+V%C4%83n+C%E1%BB%AB+N%E1%BB%91i+D%C3%A0i%2C+P.+An+B%C3%ACnh%2C+Q.+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4085,7 @@
       </c>
       <c r="I88" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20154%20Tr%E1%BA%A7n%20Vi%E1%BB%87t%20Ch%C3%A2u%2C%20154%20Tr%E1%BA%A7n%20Vi%E1%BB%87t%20Ch%C3%A2u%2C%20P.%20An%20H%C3%B2a%2C%20Q.%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+154+Tr%E1%BA%A7n+Vi%E1%BB%87t+Ch%C3%A2u%2C+P.+An+H%C3%B2a%2C+Q.+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
       </c>
       <c r="I89" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20KGG%2037%20%C4%90%E1%BB%91ng%20%C4%90a%2C%2037%20%C4%90%E1%BB%91ng%20%C4%90a%2C%20P.%20V%C4%A9nh%20L%E1%BA%A1c%2C%20TP.%20R%E1%BA%A1ch%20Gi%C3%A1</t>
+          <t>https://maps.google.com/?q=WinMart+37+%C4%90%E1%BB%91ng+%C4%90a%2C+P.+V%C4%A9nh+L%E1%BA%A1c%2C+TP.+R%E1%BA%A1ch+Gi%C3%A1</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="I90" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20119-121%20%C4%90%E1%BB%81%20Th%C3%A1m%2C%20119-121%20%C4%90%E1%BB%81%20Th%C3%A1m%2C%20Ph%C6%B0%E1%BB%9Dng%20An%20C%C6%B0%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+119-121+%C4%90%E1%BB%81+Th%C3%A1m%2C+Ph%C6%B0%E1%BB%9Dng+An+C%C6%B0%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -4208,7 +4208,7 @@
       </c>
       <c r="I91" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20108A/3%20%C4%90%C6%B0%E1%BB%9Dng%203/2%2C%20Khu%20v%E1%BB%B1c%201%2C%20Qu%E1%BB%91c%20l%E1%BB%99%201%20%28108A/3%20%C4%90%C6%B0%E1%BB%9Dng%203/2%20c%C5%A9%29%2C%20Ph%C6%B0%E1%BB%9Dng%20An%20B%C3%ACnh%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+Khu+v%E1%BB%B1c+1%2C+Qu%E1%BB%91c+l%E1%BB%99+1+%28108A%2F3+%C4%90%C6%B0%E1%BB%9Dng+3%2F2+c%C5%A9%29%2C+Ph%C6%B0%E1%BB%9Dng+An+B%C3%ACnh%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -4249,7 +4249,7 @@
       </c>
       <c r="I92" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20134A%20%C4%90%C6%B0%E1%BB%9Dng%203/2%2C%20134A%20%C4%90%C6%B0%E1%BB%9Dng%203/2%2C%20Ph%C6%B0%E1%BB%9Dng%20H%C6%B0ng%20L%E1%BB%A3i%2C%20Qu%E1%BA%ADn%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+134A+%C4%90%C6%B0%E1%BB%9Dng+3%2F2%2C+Ph%C6%B0%E1%BB%9Dng+H%C6%B0ng+L%E1%BB%A3i%2C+Qu%E1%BA%ADn+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -4290,7 +4290,7 @@
       </c>
       <c r="I93" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2098%20Nguy%E1%BB%85n%20Th%E1%BB%8B%20Minh%20Khai%2C%2098%20Nguy%E1%BB%85n%20Th%E1%BB%8B%20Minh%20Khai%2C%20P.%20T%C3%A2n%20An%2C%20Q.%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+98+Nguy%E1%BB%85n+Th%E1%BB%8B+Minh+Khai%2C+P.+T%C3%A2n+An%2C+Q.+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -4331,7 +4331,7 @@
       </c>
       <c r="I94" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2028%20B%C3%B9i%20H%E1%BB%AFu%20Ngh%C4%A9a%2C%2028%20B%C3%B9i%20H%E1%BB%AFu%20Ngh%C4%A9a%2C%20P.%20B%C3%ACnh%20Th%E1%BB%A7y%2C%20Q.%20B%C3%ACnh%20Th%E1%BB%A7y</t>
+          <t>https://maps.google.com/?q=WinMart+28+B%C3%B9i+H%E1%BB%AFu+Ngh%C4%A9a%2C+P.+B%C3%ACnh+Th%E1%BB%A7y%2C+Q.+B%C3%ACnh+Th%E1%BB%A7y%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -4372,7 +4372,7 @@
       </c>
       <c r="I95" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2075A2-77A2%20B%C3%B9i%20Quang%20Trinh%2C%2075A2-77A2%20B%C3%B9i%20Quang%20Trinh%2C%20Khu%20T%C4%90C%20Ph%C3%BA%20An%2C%20P.%20Ph%C3%BA%20Th%E1%BB%A9%2C%20Q.%20C%C3%A1i%20R%C4%83ng</t>
+          <t>https://maps.google.com/?q=WinMart+75A2-77A2+B%C3%B9i+Quang+Trinh%2C+Khu+T%C4%90C+Ph%C3%BA+An%2C+P.+Ph%C3%BA+Th%E1%BB%A9%2C+Q.+C%C3%A1i+R%C4%83ng%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -4413,7 +4413,7 @@
       </c>
       <c r="I96" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20380H1%20Tr%E1%BA%A7n%20Nam%20Ph%C3%BA%2C%20380H1%20Tr%E1%BA%A7n%20Nam%20Ph%C3%BA%2C%20P.%20An%20Kh%C3%A1nh%2C%20Q.%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+380H1+Tr%E1%BA%A7n+Nam+Ph%C3%BA%2C+P.+An+Kh%C3%A1nh%2C+Q.+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -4454,7 +4454,7 @@
       </c>
       <c r="I97" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20132%20%C4%90%C6%B0%E1%BB%9Dng%203/2%2C%20132%20%C4%90%C6%B0%E1%BB%9Dng%203/2%2C%20P.%20H%C6%B0ng%20L%E1%BB%A3i%2C%20Q.%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+132+%C4%90%C6%B0%E1%BB%9Dng+3%2F2%2C+P.+H%C6%B0ng+L%E1%BB%A3i%2C+Q.+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -4495,7 +4495,7 @@
       </c>
       <c r="I98" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20KGG%20L%C3%B4%20A7.08-A7.09%20%C4%90%C6%B0%E1%BB%9Dng%20s%E1%BB%91%2027%2C%20L%C3%B4%20A7-08%20v%C3%A0%20A7-09%20%C4%90%C6%B0%E1%BB%9Dng%20s%E1%BB%91%2027%2C%20Khu%20%C4%91%C3%B4%20th%E1%BB%8B%20m%E1%BB%9Bi%20T%C3%A2y%20B%E1%BA%AFc%2C%20P.%20V%C4%A9nh%20Thanh%2C%20TP.%20R%E1%BA%A1ch%20Gi%C3%A1</t>
+          <t>https://maps.google.com/?q=WinMart+L%C3%B4+A7.08-A7.09+%C4%90%C6%B0%E1%BB%9Dng+s%E1%BB%91+27%2C+L%C3%B4+A7-08+v%C3%A0+A7-09+%C4%90%C6%B0%E1%BB%9Dng+s%E1%BB%91+27%2C+Khu+%C4%91%C3%B4+th%E1%BB%8B+m%E1%BB%9Bi+T%C3%A2y+B%E1%BA%AFc%2C+P.+V%C4%A9nh+Thanh%2C+TP.+R%E1%BA%A1ch+Gi%C3%A1</t>
         </is>
       </c>
     </row>
@@ -4536,7 +4536,7 @@
       </c>
       <c r="I99" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20T1-6%20CC%20T%C3%A2y%20Nguy%C3%AAn%20Plaza%2C%20T1-6%20t%E1%BA%A7ng%20tr%E1%BB%87t%2C%20CC%20T%C3%A2y%20Nguy%C3%AAn%20Plaza%2C%20KDC%20l%C3%B4%2011D%2C%20P.%20Ph%C3%BA%20Th%E1%BB%A9%2C%20Q.%20C%C3%A1i%20R%C4%83ng</t>
+          <t>https://maps.google.com/?q=WinMart+T1-6+CC+T%C3%A2y+Nguy%C3%AAn+Plaza%2C+T1-6+t%E1%BA%A7ng+tr%E1%BB%87t%2C+CC+T%C3%A2y+Nguy%C3%AAn+Plaza%2C+KDC+l%C3%B4+11D%2C+P.+Ph%C3%BA+Th%E1%BB%A9%2C+Q.+C%C3%A1i+R%C4%83ng%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -4577,7 +4577,7 @@
       </c>
       <c r="I100" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%208B%20%C4%90%C6%B0%E1%BB%9Dng%20s%E1%BB%91%203%2C%208B%20%C4%90%C6%B0%E1%BB%9Dng%20s%E1%BB%91%203%2C%20KDC%20C%C3%A1i%20S%C6%A1n%20H%C3%A0ng%20B%C3%A0ng%2C%20P.%20An%20B%C3%ACnh%2C%20Q.%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+8B+%C4%90%C6%B0%E1%BB%9Dng+s%E1%BB%91+3%2C+KDC+C%C3%A1i+S%C6%A1n+H%C3%A0ng+B%C3%A0ng%2C+P.+An+B%C3%ACnh%2C+Q.+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -4618,7 +4618,7 @@
       </c>
       <c r="I101" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2092%20X%C3%B4%20Vi%E1%BA%BFt%20Ngh%E1%BB%87%20T%C4%A9nh%2C%2092%20X%C3%B4%20Vi%E1%BA%BFt%20Ngh%E1%BB%87%20T%C4%A9nh%2C%20P.%20T%C3%A2n%20An%2C%20Q.%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+92+X%C3%B4+Vi%E1%BA%BFt+Ngh%E1%BB%87+T%C4%A9nh%2C+P.+T%C3%A2n+An%2C+Q.+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -4659,7 +4659,7 @@
       </c>
       <c r="I102" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20110%20Nguy%E1%BB%85n%20Vi%E1%BB%87t%20H%E1%BB%93ng%2C%20110%20Nguy%E1%BB%85n%20Vi%E1%BB%87t%20H%E1%BB%93ng%2C%20P.%20An%20Ph%C3%BA%2C%20Q.%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+110+Nguy%E1%BB%85n+Vi%E1%BB%87t+H%E1%BB%93ng%2C+P.+An+Ph%C3%BA%2C+Q.+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -4700,7 +4700,7 @@
       </c>
       <c r="I103" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%208C/1%20%C4%90%C6%B0%E1%BB%9Dng%201B%2C%208C/1%20%C4%90%C6%B0%E1%BB%9Dng%201B%2C%20Khu%20v%E1%BB%B1c%203%2C%20P.%20H%C6%B0ng%20Th%E1%BA%A1nh%2C%20Q.%20C%C3%A1i%20R%C4%83ng</t>
+          <t>https://maps.google.com/?q=WinMart+8C%2F1+%C4%90%C6%B0%E1%BB%9Dng+1B%2C+Khu+v%E1%BB%B1c+3%2C+P.+H%C6%B0ng+Th%E1%BA%A1nh%2C+Q.+C%C3%A1i+R%C4%83ng%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -4741,7 +4741,7 @@
       </c>
       <c r="I104" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2057-59%20Nguy%E1%BB%85n%20Tri%20Ph%C6%B0%C6%A1ng%2C%2057-59%20Nguy%E1%BB%85n%20Tri%20Ph%C6%B0%C6%A1ng%2C%20P.%20An%20Kh%C3%A1nh%2C%20Q.%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+57-59+Nguy%E1%BB%85n+Tri+Ph%C6%B0%C6%A1ng%2C+P.+An+Kh%C3%A1nh%2C+Q.+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -4782,7 +4782,7 @@
       </c>
       <c r="I105" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20563C%20Tr%E1%BA%A7n%20Quang%20Di%E1%BB%87u%2C%20563C%20Tr%E1%BA%A7n%20Quang%20Di%E1%BB%87u%2C%20P.%20An%20Th%E1%BB%9Bi%2C%20Q.%20B%C3%ACnh%20Thu%E1%BB%B7</t>
+          <t>https://maps.google.com/?q=WinMart+563C+Tr%E1%BA%A7n+Quang+Di%E1%BB%87u%2C+P.+An+Th%E1%BB%9Bi%2C+Q.+B%C3%ACnh+Thu%E1%BB%B7%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -4823,7 +4823,7 @@
       </c>
       <c r="I106" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20114B-114C%20C%C3%A1ch%20M%E1%BA%A1ng%20Th%C3%A1ng%208%2C%20114B-114C%20C%C3%A1ch%20M%E1%BA%A1ng%20Th%C3%A1ng%208%2C%20P.%20C%C3%A1i%20Kh%E1%BA%BF%2C%20Q.%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+114B-114C+C%C3%A1ch+M%E1%BA%A1ng+Th%C3%A1ng+8%2C+P.+C%C3%A1i+Kh%E1%BA%BF%2C+Q.+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -4864,7 +4864,7 @@
       </c>
       <c r="I107" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%2027%20Tr%E1%BA%A7n%20Ho%C3%A0ng%20Na%2C%20%C4%90%C6%B0%E1%BB%9Dng%20Tr%E1%BA%A7n%20Ho%C3%A0ng%20Na%2C%20P.%20H%C6%B0ng%20L%E1%BB%A3i%2C%20Q.%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+27+Tr%E1%BA%A7n+Ho%C3%A0ng+Na%2C+%C4%90%C6%B0%E1%BB%9Dng+Tr%E1%BA%A7n+Ho%C3%A0ng+Na%2C+P.+H%C6%B0ng+L%E1%BB%A3i%2C+Q.+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -4905,7 +4905,7 @@
       </c>
       <c r="I108" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20%C4%90%C6%B0%E1%BB%9Dng%20V%C3%B2ng%20Cung%2C%20Th%E1%BB%ADa%20%C4%91%E1%BA%A5t%2043%2C%20t%E1%BB%9D%20b%E1%BA%A3n%20%C4%91%E1%BB%93%2081%2C%20Khu%20v%E1%BB%B1c%205%2C%20%C4%91%C6%B0%E1%BB%9Dng%20V%C3%B2ng%20Cung%2C%20P.%20An%20B%C3%ACnh%2C%20Q.%20Ninh%20Ki%E1%BB%81u</t>
+          <t>https://maps.google.com/?q=WinMart+Th%E1%BB%ADa+%C4%91%E1%BA%A5t+43%2C+t%E1%BB%9D+b%E1%BA%A3n+%C4%91%E1%BB%93+81%2C+Khu+v%E1%BB%B1c+5%2C+%C4%91%C6%B0%E1%BB%9Dng+V%C3%B2ng+Cung%2C+P.+An+B%C3%ACnh%2C+Q.+Ninh+Ki%E1%BB%81u%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -4946,7 +4946,7 @@
       </c>
       <c r="I109" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20VLG%2054/7%20M%E1%BA%ADu%20Th%C3%A2n%2C%20Kh%C3%B3m%203%2C%20P.%203%2C%20TP.%20V%C4%A9nh%20Long</t>
+          <t>https://maps.google.com/?q=WinMart+54%2F7+M%E1%BA%ADu+Th%C3%A2n%2C+Kh%C3%B3m+3%2C+P.+3%2C+TP.+V%C4%A9nh+Long</t>
         </is>
       </c>
     </row>
@@ -4987,7 +4987,7 @@
       </c>
       <c r="I110" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20VLG%2060G%20Ph%E1%BA%A1m%20H%C3%B9ng%2C%2060G%2C%20%C4%90%C6%B0%E1%BB%9Dng%20Ph%E1%BA%A1m%20H%C3%B9ng%2C%20P.%209%2C%20TP.%20V%C4%A9nh%20Long</t>
+          <t>https://maps.google.com/?q=WinMart+60G+Ph%E1%BA%A1m+H%C3%B9ng%2C+60G%2C+%C4%90%C6%B0%E1%BB%9Dng+Ph%E1%BA%A1m+H%C3%B9ng%2C+P.+9%2C+TP.+V%C4%A9nh+Long</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="I111" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20VLG%20T%C4%90S%20533%2C%20TB%C4%90%2016%2C%20Tr%E1%BA%A7n%20Ph%C3%BA%2C%2064/4A%20Tr%E1%BA%A7n%20Ph%C3%BA%2C%20P.%20Ph%C6%B0%E1%BB%9Bc%20H%E1%BA%ADu</t>
+          <t>https://maps.google.com/?q=WinMart+T%C4%90S+533%2C+TB%C4%90+16%2C+Tr%E1%BA%A7n+Ph%C3%BA%2C+64%2F4A+Tr%E1%BA%A7n+Ph%C3%BA%2C+P.+Ph%C6%B0%E1%BB%9Bc+H%E1%BA%ADu</t>
         </is>
       </c>
     </row>
@@ -5069,7 +5069,7 @@
       </c>
       <c r="I112" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20%C4%90%C6%B0%E1%BB%9Dng%20N3%2C%20KDC%20Nam%20Long%202%2C%20Th%E1%BB%ADa%20%C4%91%E1%BA%A5t%20s%E1%BB%91%201410-1411%2C%20TB%C4%90%20s%E1%BB%91%2056%2C%20KDC%20Nam%20Long%202%2C%20L%C3%B4%209A%2C%20K%C4%90T%20Nam%20C%E1%BA%A7n%20Th%C6%A1%2C%20P.%20H%C6%B0ng%20Th%E1%BA%A1nh%2C%20Q.%20C%C3%A1i%20R%C4%83ng</t>
+          <t>https://maps.google.com/?q=WinMart+%C4%90%C6%B0%E1%BB%9Dng+N3%2C+KDC+Nam+Long+2%2C+Th%E1%BB%ADa+%C4%91%E1%BA%A5t+s%E1%BB%91+1410-1411%2C+TB%C4%90+s%E1%BB%91+56%2C+KDC+Nam+Long+2%2C+L%C3%B4+9A%2C+K%C4%90T+Nam+C%E1%BA%A7n+Th%C6%A1%2C+P.+H%C6%B0ng+Th%E1%BA%A1nh%2C+Q.+C%C3%A1i+R%C4%83ng%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -5110,7 +5110,7 @@
       </c>
       <c r="I113" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20VLG%20%C4%90%C6%B0%E1%BB%9Dng%202/9%2C%20Duy%C3%AAn%20H%E1%BA%A3i%2C%20%C4%90%C6%B0%E1%BB%9Dng%202%20th%C3%A1ng%209%2C%20TX.%20Duy%C3%AAn%20H%E1%BA%A3i%2C%20T.%20Tr%C3%A0%20vinh</t>
+          <t>https://maps.google.com/?q=WinMart+%C4%90%C6%B0%E1%BB%9Dng+2%2F9%2C+Duy%C3%AAn+H%E1%BA%A3i%2C+%C4%90%C6%B0%E1%BB%9Dng+2+th%C3%A1ng+9%2C+TX.+Duy%C3%AAn+H%E1%BA%A3i%2C+T.+Tr%C3%A0+vinh</t>
         </is>
       </c>
     </row>
@@ -5151,7 +5151,7 @@
       </c>
       <c r="I114" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20VLG%20267%20%C4%90i%E1%BB%87n%20Bi%C3%AAn%20Ph%E1%BB%A7%2C%20Tr%C3%A0%20Vinh%2C%20267%20%C4%90%C6%B0%E1%BB%9Dng%20%C4%90i%E1%BB%87n%20Bi%C3%AAn%20Ph%E1%BB%A7%2C%20Kh%C3%B3m%209%2C%20P.%20Tr%C3%A0%20Vinh</t>
+          <t>https://maps.google.com/?q=WinMart+267+%C4%90i%E1%BB%87n+Bi%C3%AAn+Ph%E1%BB%A7%2C+Tr%C3%A0+Vinh%2C+267+%C4%90%C6%B0%E1%BB%9Dng+%C4%90i%E1%BB%87n+Bi%C3%AAn+Ph%E1%BB%A7%2C+Kh%C3%B3m+9%2C+P.+Tr%C3%A0+Vinh</t>
         </is>
       </c>
     </row>
@@ -5192,7 +5192,7 @@
       </c>
       <c r="I115" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20%E1%BA%A4p%20Ch%C3%A2u%20Th%C3%A0nh%2C%20M%E1%BB%B9%20Xuy%C3%AAn%2C%20Th%E1%BB%ADa%20%C4%91%E1%BA%A5t%20s%E1%BB%91%2065%2C%20t%E1%BB%9D%20b%E1%BA%A3n%20%C4%91%E1%BB%93%2022%2C%20%E1%BA%A4p%20Ch%C3%A2u%20Th%C3%A0nh%2C%20P.%20M%E1%BB%B9%20Xuy%C3%AAn</t>
+          <t>https://maps.google.com/?q=WinMart+%E1%BA%A4p+Ch%C3%A2u+Th%C3%A0nh%2C+M%E1%BB%B9+Xuy%C3%AAn%2C+Th%E1%BB%ADa+%C4%91%E1%BA%A5t+s%E1%BB%91+65%2C+t%E1%BB%9D+b%E1%BA%A3n+%C4%91%E1%BB%93+22%2C+%E1%BA%A4p+Ch%C3%A2u+Th%C3%A0nh%2C+P.+M%E1%BB%B9+Xuy%C3%AAn%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -5233,7 +5233,7 @@
       </c>
       <c r="I116" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20A2-04%2C%20A2-05%20V%C5%A9%20%C4%90%C3%ACnh%20Li%E1%BB%87u%2C%20A2-04%2C%20A2-05%20%C4%90%C6%B0%E1%BB%9Dng%20V%C5%A9%20%C4%90%C3%ACnh%20Li%E1%BB%87u%2C%20P.%20C%C3%A1i%20R%C4%83ng</t>
+          <t>https://maps.google.com/?q=WinMart+A2-04%2C+A2-05+V%C5%A9+%C4%90%C3%ACnh+Li%E1%BB%87u%2C+A2-04%2C+A2-05+%C4%90%C6%B0%E1%BB%9Dng+V%C5%A9+%C4%90%C3%ACnh+Li%E1%BB%87u%2C+P.+C%C3%A1i+R%C4%83ng%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -5274,7 +5274,7 @@
       </c>
       <c r="I117" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CTO%20KDC%20Th%C6%B0%E1%BB%9Dng%20Th%E1%BA%A1nh%20-Tr%C6%B0%E1%BB%9Dng%20%C4%90%E1%BA%A1i%20H%E1%BB%8Dc%2C%20Th%E1%BB%ADa%20%C4%91%E1%BA%A5t%20s%E1%BB%91%204444%2C%20TB%C4%90%20s%E1%BB%91%2063%2C%20L%C3%B4%20A17-39-40%2C%20Tr%C6%B0%C6%A1ng%20V%C4%A9nh%20Nguy%C3%AAn%2C%20KDC%20Th%C6%B0%E1%BB%9Dng%20Th%E1%BA%A1nh%20v%C3%A0%20Tr%C6%B0%E1%BB%9Dng%20%C4%90%E1%BA%A1i%20h%E1%BB%8Dc%2C%20P.%20C%C3%A1i%20R%C4%83ng%2C%20TP.%20%20C%E1%BA%A7n%20Th%C6%A1</t>
+          <t>https://maps.google.com/?q=WinMart+KDC+Th%C6%B0%E1%BB%9Dng+Th%E1%BA%A1nh+-Tr%C6%B0%E1%BB%9Dng+%C4%90%E1%BA%A1i+H%E1%BB%8Dc%2C+Th%E1%BB%ADa+%C4%91%E1%BA%A5t+s%E1%BB%91+4444%2C+TB%C4%90+s%E1%BB%91+63%2C+L%C3%B4+A17-39-40%2C+Tr%C6%B0%C6%A1ng+V%C4%A9nh+Nguy%C3%AAn%2C+KDC+Th%C6%B0%E1%BB%9Dng+Th%E1%BA%A1nh+v%C3%A0+Tr%C6%B0%E1%BB%9Dng+%C4%90%E1%BA%A1i+h%E1%BB%8Dc%2C+P.+C%C3%A1i+R%C4%83ng%2C+TP.+C%E1%BA%A7n+Th%C6%A1</t>
         </is>
       </c>
     </row>
@@ -5319,7 +5319,7 @@
       </c>
       <c r="I118" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VinMart%20An%20Giang%2C%20TTTM%20Vincom%20Long%20Xuy%C3%AAn%2C%20S%E1%BB%91%201242%20%C4%90%C6%B0%E1%BB%9Dng%20Tr%E1%BA%A7n%20H%C6%B0ng%20%C4%90%E1%BA%A1o%2C%20Ph%C6%B0%E1%BB%9Dng%20M%E1%BB%B9%20B%C3%ACnh%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Long%20Xuy%C3%AAn%2C%20T%E1%BB%89nh%20An%20Giang</t>
+          <t>https://maps.google.com/?q=VinMart+An+Giang%2C+TTTM+Vincom+Long+Xuy%C3%AAn%2C+S%E1%BB%91+1242+%C4%90%C6%B0%E1%BB%9Dng+Tr%E1%BA%A7n+H%C6%B0ng+%C4%90%E1%BA%A1o%2C+Ph%C6%B0%E1%BB%9Dng+M%E1%BB%B9+B%C3%ACnh%2C+Th%C3%A0nh+ph%E1%BB%91+Long+Xuy%C3%AAn%2C+T%E1%BB%89nh+An+Giang</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="I119" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VinMart%20B%E1%BA%A1c%20Li%C3%AAu%2C%20TTTM%20Vincom%20B%E1%BA%A1c%20Li%C3%AAu%2C%20S%E1%BB%91%2015%20%C4%90%C6%B0%E1%BB%9Dng%20Tr%E1%BA%A7n%20Ph%C3%BA%2C%20Ph%C6%B0%E1%BB%9Dng%203%2C%20Th%C3%A0nh%20ph%E1%BB%91%20B%E1%BA%A1c%20Li%C3%AAu%2C%20T%E1%BB%89nh%20B%E1%BA%A1c%20Li%C3%AAu</t>
+          <t>https://maps.google.com/?q=VinMart+B%E1%BA%A1c+Li%C3%AAu%2C+TTTM+Vincom+B%E1%BA%A1c+Li%C3%AAu%2C+S%E1%BB%91+15+%C4%90%C6%B0%E1%BB%9Dng+Tr%E1%BA%A7n+Ph%C3%BA%2C+Ph%C6%B0%E1%BB%9Dng+3%2C+Th%C3%A0nh+ph%E1%BB%91+B%E1%BA%A1c+Li%C3%AAu%2C+T%E1%BB%89nh+B%E1%BA%A1c+Li%C3%AAu</t>
         </is>
       </c>
     </row>
@@ -5409,7 +5409,7 @@
       </c>
       <c r="I120" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VinMart%20Tr%C3%A0%20Vinh%2C%20TTTM%20Vincom%20Plaza%20Tr%C3%A0%20Vinh%2C%20S%E1%BB%91%2024%20%C4%90%C6%B0%E1%BB%9Dng%20Nguy%E1%BB%85n%20Th%E1%BB%8B%20Minh%20Khai%2C%20Ph%C6%B0%E1%BB%9Dng%202%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Tr%C3%A0%20Vinh%2C%20T%E1%BB%89nh%20Tr%C3%A0%20Vinh</t>
+          <t>https://maps.google.com/?q=VinMart+Tr%C3%A0+Vinh%2C+TTTM+Vincom+Plaza+Tr%C3%A0+Vinh%2C+S%E1%BB%91+24+%C4%90%C6%B0%E1%BB%9Dng+Nguy%E1%BB%85n+Th%E1%BB%8B+Minh+Khai%2C+Ph%C6%B0%E1%BB%9Dng+2%2C+Th%C3%A0nh+ph%E1%BB%91+Tr%C3%A0+Vinh%2C+T%E1%BB%89nh+Tr%C3%A0+Vinh</t>
         </is>
       </c>
     </row>
@@ -5454,7 +5454,7 @@
       </c>
       <c r="I121" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VinMart%20Long%20An%2C%20G%C3%B3c%20%C4%91%C6%B0%E1%BB%9Dng%20H%C3%B9ng%20V%C6%B0%C6%A1ng%20v%C3%A0%20%C4%90%C6%B0%E1%BB%9Dng%20Mai%20Th%E1%BB%8B%20T%E1%BB%91t%2C%20Ph%C6%B0%E1%BB%9Dng%202%2C%20Th%C3%A0nh%20ph%E1%BB%91%20T%C3%A2n%20An%2C%20T%E1%BB%89nh%20Long%20An</t>
+          <t>https://maps.google.com/?q=VinMart+Long+An%2C+G%C3%B3c+%C4%91%C6%B0%E1%BB%9Dng+H%C3%B9ng+V%C6%B0%C6%A1ng+v%C3%A0+%C4%90%C6%B0%E1%BB%9Dng+Mai+Th%E1%BB%8B+T%E1%BB%91t%2C+Ph%C6%B0%E1%BB%9Dng+2%2C+Th%C3%A0nh+ph%E1%BB%91+T%C3%A2n+An%2C+T%E1%BB%89nh+Long+An</t>
         </is>
       </c>
     </row>
@@ -5499,7 +5499,7 @@
       </c>
       <c r="I122" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VinMart%20%C4%90%E1%BB%93ng%20Th%C3%A1p%2C%20TTTM%20Vincom%2B%20Sa%20%C4%90%C3%A9c%2C%20%C4%90%C6%B0%E1%BB%9Dng%20Nguy%E1%BB%85n%20T%E1%BA%A5t%20Th%C3%A0nh%20%2C%20kh%C3%B3m%204%2C%20Ph%C6%B0%E1%BB%9Dng%201%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Sa%20%C4%90%C3%A9c%2C%20T%E1%BB%89nh%20%C4%90%E1%BB%93ng%20Th%C3%A1p.</t>
+          <t>https://maps.google.com/?q=VinMart+%C4%90%E1%BB%93ng+Th%C3%A1p%2C+TTTM+Vincom%2B+Sa+%C4%90%C3%A9c%2C+%C4%90%C6%B0%E1%BB%9Dng+Nguy%E1%BB%85n+T%E1%BA%A5t+Th%C3%A0nh+%2C+kh%C3%B3m+4%2C+Ph%C6%B0%E1%BB%9Dng+1%2C+Th%C3%A0nh+ph%E1%BB%91+Sa+%C4%90%C3%A9c%2C+T%E1%BB%89nh+%C4%90%E1%BB%93ng+Th%C3%A1p.</t>
         </is>
       </c>
     </row>
@@ -5544,7 +5544,7 @@
       </c>
       <c r="I123" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VinMart%20Cao%20Lanh%2C%20Trung%20tam%20thuong%20mai%20v%C3%A0%20Shophouse%20Cao%20Lanh%20-%20Dong%20Thap%2C%20Phuong%201%2C%20Thanh%20pho%20Cao%20Lanh%2C%20tinh%20Dong%20Thap</t>
+          <t>https://maps.google.com/?q=VinMart+Cao+Lanh%2C+Trung+tam+thuong+mai+v%C3%A0+Shophouse+Cao+Lanh+-+Dong+Thap%2C+Phuong+1%2C+Thanh+pho+Cao+Lanh%2C+tinh+Dong+Thap</t>
         </is>
       </c>
     </row>
@@ -5589,7 +5589,7 @@
       </c>
       <c r="I124" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VinMart%20Soc%20Trang%2C%20Thua%20dat%20so%20310%2C%20to%20ban%20do%20so%2048%2C%20duong%20Tran%20Hung%20Dao%2C%20Phuong%202%2C%20Thanh%20pho%20Soc%20Trang%2C%20Tinh%20Soc%20Trang</t>
+          <t>https://maps.google.com/?q=VinMart+Soc+Trang%2C+Thua+dat+so+310%2C+to+ban+do+so+48%2C+duong+Tran+Hung+Dao%2C+Phuong+2%2C+Thanh+pho+Soc+Trang%2C+Tinh+Soc+Trang</t>
         </is>
       </c>
     </row>
@@ -5634,7 +5634,7 @@
       </c>
       <c r="I125" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VinMart%20C%C3%A0%20Mau%2C%20TTTM%20Vincom%20C%C3%A0%20Mau%2C%20Ph%C6%B0%E1%BB%9Dng%201%2C%20Th%C3%A0nh%20ph%E1%BB%91%20C%C3%A0%20Mau%2C%20T%E1%BB%89nh%20C%C3%A0%20Mau</t>
+          <t>https://maps.google.com/?q=VinMart+C%C3%A0+Mau%2C+TTTM+Vincom+C%C3%A0+Mau%2C+Ph%C6%B0%E1%BB%9Dng+1%2C+Th%C3%A0nh+ph%E1%BB%91+C%C3%A0+Mau%2C+T%E1%BB%89nh+C%C3%A0+Mau</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="I126" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%20VCP%20BLU%20B%E1%BA%A1c%20Li%C3%AAu%2C%20Gian%20h%C3%A0ng%20L2-01%20TTTM%20Vincom%20Plaza%20Tr%E1%BA%A7n%20Hu%E1%BB%B3nh%2C%20B%E1%BA%A1c%20Li%C3%AAu%2C%20s%E1%BB%91%20109%20Tr%E1%BA%A7n%20Hu%E1%BB%B3nh%2C%20P7</t>
+          <t>https://maps.google.com/?q=WinMart+BLU+B%E1%BA%A1c+Li%C3%AAu%2C+Gian+h%C3%A0ng+L2-01+TTTM+Vincom+Plaza+Tr%E1%BA%A7n+Hu%E1%BB%B3nh%2C+B%E1%BA%A1c+Li%C3%AAu%2C+s%E1%BB%91+109+Tr%E1%BA%A7n+Hu%E1%BB%B3nh%2C+P7</t>
         </is>
       </c>
     </row>
@@ -5724,7 +5724,7 @@
       </c>
       <c r="I127" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%20VCP%20TGG%20M%E1%BB%B9%20Tho%2C%201A%20H%C3%B9ng%20V%C6%B0%C6%A1ng%2C%20P1%2C%20th%C3%A0nh%20Ph%E1%BB%91%20M%E1%BB%B9%20Tho</t>
+          <t>https://maps.google.com/?q=WinMart+TGG+M%E1%BB%B9+Tho%2C+1A+H%C3%B9ng+V%C6%B0%C6%A1ng%2C+P1%2C+th%C3%A0nh+Ph%E1%BB%91+M%E1%BB%B9+Tho</t>
         </is>
       </c>
     </row>
@@ -5769,7 +5769,7 @@
       </c>
       <c r="I128" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VM%2B%20TGG%20152%20Ly%20Thuong%20Kiet%2C%20152%20Ly%20Thuong%20Kiet%2C%20Phuong%206%2C%20TP.%20My%20Tho%2C%20Tinh%20Tien%20Giang</t>
+          <t>https://maps.google.com/?q=WinMart+152+Ly+Thuong+Kiet%2C+Phuong+6%2C+TP.+My+Tho%2C+Tinh+Tien+Giang</t>
         </is>
       </c>
     </row>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="I129" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VM%2B%20AGG%20268/4%20va%20268/5%20Hung%20Vuong%2C%20268/4%20va%20268/5%20Duong%20Hung%20Vuong%2C%20phuong%20My%20Long%2C%20Thanh%20pho%20Long%20Xuyen%2C%20Tinh%20An%20Giang</t>
+          <t>https://maps.google.com/?q=WinMart+268%2F4+va+268%2F5+Hung+Vuong%2C+268%2F4+va+268%2F5+Duong+Hung+Vuong%2C+phuong+My+Long%2C+Thanh+pho+Long+Xuyen%2C+Tinh+An+Giang</t>
         </is>
       </c>
     </row>
@@ -5859,7 +5859,7 @@
       </c>
       <c r="I130" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%2054A%20L%C3%BD%20Th%C6%B0%E1%BB%9Dng%20Ki%E1%BB%87t%2C%2054A%20L%C3%BD%20Th%C6%B0%E1%BB%9Dng%20Ki%E1%BB%87t%2C%20Ph%C6%B0%E1%BB%9Dng%20M%E1%BB%B9%20B%C3%ACnh%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Long%20Xuy%C3%AAn</t>
+          <t>https://maps.google.com/?q=WinMart+54A+L%C3%BD+Th%C6%B0%E1%BB%9Dng+Ki%E1%BB%87t%2C+Ph%C6%B0%E1%BB%9Dng+M%E1%BB%B9+B%C3%ACnh%2C+Th%C3%A0nh+ph%E1%BB%91+Long+Xuy%C3%AAn</t>
         </is>
       </c>
     </row>
@@ -5904,7 +5904,7 @@
       </c>
       <c r="I131" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TGG%20203%20L%C3%BD%20Th%C6%B0%E1%BB%9Dng%20Ki%E1%BB%87t%2C%20203%20L%C3%BD%20Th%C6%B0%E1%BB%9Dng%20Ki%E1%BB%87t%2C%20Ph%C6%B0%E1%BB%9Dng%205%2C%20Th%C3%A0nh%20Ph%E1%BB%91%20M%E1%BB%B9%20Tho</t>
+          <t>https://maps.google.com/?q=WinMart+203+L%C3%BD+Th%C6%B0%E1%BB%9Dng+Ki%E1%BB%87t%2C+Ph%C6%B0%E1%BB%9Dng+5%2C+Th%C3%A0nh+Ph%E1%BB%91+M%E1%BB%B9+Tho</t>
         </is>
       </c>
     </row>
@@ -5949,7 +5949,7 @@
       </c>
       <c r="I132" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2BAGG%204Bis%20L%C3%AA%20Minh%20Ng%C6%B0%C6%A1n%2C%204Bis%20L%C3%AA%20Minh%20Ng%C6%B0%C6%A1n%2C%20Ph%C6%B0%E1%BB%9Dng%20M%E1%BB%B9%20Long%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Long%20Xuy%C3%AAn</t>
+          <t>https://maps.google.com/?q=WinMart+WM%2BAGG+4Bis+L%C3%AA+Minh+Ng%C6%B0%C6%A1n%2C+4Bis+L%C3%AA+Minh+Ng%C6%B0%C6%A1n%2C+Ph%C6%B0%E1%BB%9Dng+M%E1%BB%B9+Long%2C+Th%C3%A0nh+ph%E1%BB%91+Long+Xuy%C3%AAn</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="I133" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VM%2BTGG%20200%20Nam%20K%C3%AC%20Kh%E1%BB%9Fi%20Ngh%C4%A9a%2C%20200%20Nam%20K%E1%BB%B3%20Kh%E1%BB%9Fi%20Ngh%C4%A9a%2C%20Ph%C6%B0%E1%BB%9Dng%201%2C%20Th%C3%A0nh%20ph%E1%BB%91%20M%E1%BB%B9%20Tho%2C%20T%E1%BB%89nh%20Ti%E1%BB%81n%20Giang</t>
+          <t>https://maps.google.com/?q=WinMart+VM%2BTGG+200+Nam+K%C3%AC+Kh%E1%BB%9Fi+Ngh%C4%A9a%2C+200+Nam+K%E1%BB%B3+Kh%E1%BB%9Fi+Ngh%C4%A9a%2C+Ph%C6%B0%E1%BB%9Dng+1%2C+Th%C3%A0nh+ph%E1%BB%91+M%E1%BB%B9+Tho%2C+T%E1%BB%89nh+Ti%E1%BB%81n+Giang</t>
         </is>
       </c>
     </row>
@@ -6039,7 +6039,7 @@
       </c>
       <c r="I134" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VM%2B%20AGG%20244-245%20Ham%20Nghi%2C%20VM%2B%20AGG%20%20244-245%20duong%20Ham%20Nghi%2C%20Phuong%20Binh%20Khanh%2C%20Thanh%20pho%20Long%20Xuyen%2C%20Tinh%20An%20Giang</t>
+          <t>https://maps.google.com/?q=WinMart+244-245+Ham+Nghi%2C+VM%2B+AGG+244-245+duong+Ham+Nghi%2C+Phuong+Binh+Khanh%2C+Thanh+pho+Long+Xuyen%2C+Tinh+An+Giang</t>
         </is>
       </c>
     </row>
@@ -6084,7 +6084,7 @@
       </c>
       <c r="I135" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%2077%20Ung%20V%C4%83n%20Khi%C3%AAm%2C%2077%20Ung%20V%C4%83n%20Khi%C3%AAm%2C%20t%E1%BB%95%206%2C%20Kh%C3%B3m%20%C4%90%C3%B4ng%20Th%C3%A0nh%2C%20Ph%C6%B0%E1%BB%9Dng%20%C4%90%C3%B4ng%20Xuy%C3%AAn%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Long%20Xuy%C3%AAn</t>
+          <t>https://maps.google.com/?q=WinMart+77+Ung+V%C4%83n+Khi%C3%AAm%2C+t%E1%BB%95+6%2C+Kh%C3%B3m+%C4%90%C3%B4ng+Th%C3%A0nh%2C+Ph%C6%B0%E1%BB%9Dng+%C4%90%C3%B4ng+Xuy%C3%AAn%2C+Th%C3%A0nh+ph%E1%BB%91+Long+Xuy%C3%AAn</t>
         </is>
       </c>
     </row>
@@ -6129,7 +6129,7 @@
       </c>
       <c r="I136" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20535A%20V%C3%B5%20Th%E1%BB%8B%20S%C3%A1u%2C%20535A%20V%C3%B5%20Th%E1%BB%8B%20S%C3%A1u%2C%20Ph%C6%B0%E1%BB%9Dng%20M%E1%BB%B9%20Xuy%C3%AAn%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Long%20Xuy%C3%AAn</t>
+          <t>https://maps.google.com/?q=WinMart+535A+V%C3%B5+Th%E1%BB%8B+S%C3%A1u%2C+Ph%C6%B0%E1%BB%9Dng+M%E1%BB%B9+Xuy%C3%AAn%2C+Th%C3%A0nh+ph%E1%BB%91+Long+Xuy%C3%AAn</t>
         </is>
       </c>
     </row>
@@ -6174,7 +6174,7 @@
       </c>
       <c r="I137" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VM%2B%20AGG%2001%20Thai%20Phien%2C%20Thua%20dat%20so%2001%2C%20to%20ban%20do%20so%20048%2C%20Binh%20Khanh%2C%20thanh%20pho%20Long%20Xuyen%2C%20tinh%20An%20Giang</t>
+          <t>https://maps.google.com/?q=WinMart+01+Thai+Phien%2C+Thua+dat+so+01%2C+to+ban+do+so+048%2C+Binh+Khanh%2C+thanh+pho+Long+Xuyen%2C+tinh+An+Giang</t>
         </is>
       </c>
     </row>
@@ -6219,7 +6219,7 @@
       </c>
       <c r="I138" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TGG%20915B%20Tr%E1%BA%A7n%20H%C6%B0ng%20%C4%90%E1%BA%A1o%2C%20915B%20Tr%E1%BA%A7n%20H%C6%B0ng%20%C4%90%E1%BA%A1o%2C%20Ph%C6%B0%E1%BB%9Dng%205%2C%20Th%C3%A0nh%20Ph%E1%BB%91%20M%E1%BB%B9%20Tho</t>
+          <t>https://maps.google.com/?q=WinMart+915B+Tr%E1%BA%A7n+H%C6%B0ng+%C4%90%E1%BA%A1o%2C+Ph%C6%B0%E1%BB%9Dng+5%2C+Th%C3%A0nh+Ph%E1%BB%91+M%E1%BB%B9+Tho</t>
         </is>
       </c>
     </row>
@@ -6264,7 +6264,7 @@
       </c>
       <c r="I139" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20104%20%C4%91%C6%B0%E1%BB%9Dng%20Tr%E1%BA%A7n%20Quang%20Kh%E1%BA%A3i%2C%20104%20%C4%91%C6%B0%E1%BB%9Dng%20Tr%E1%BA%A7n%20Quang%20Kh%E1%BA%A3i%2C%20t%E1%BB%95%2036%2C%20Kh%C3%B3m%20Trung%20An%2C%20Ph%C6%B0%E1%BB%9Dng%20M%E1%BB%B9%20Th%E1%BB%9Bi%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Long%20Xuy%C3%AAn</t>
+          <t>https://maps.google.com/?q=WinMart+104+%C4%91%C6%B0%E1%BB%9Dng+Tr%E1%BA%A7n+Quang+Kh%E1%BA%A3i%2C+t%E1%BB%95+36%2C+Kh%C3%B3m+Trung+An%2C+Ph%C6%B0%E1%BB%9Dng+M%E1%BB%B9+Th%E1%BB%9Bi%2C+Th%C3%A0nh+ph%E1%BB%91+Long+Xuy%C3%AAn</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="I140" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20DTP%20163%20T%C3%B4n%20%C4%90%E1%BB%A9c%20Th%E1%BA%AFng%2C%20163%20T%C3%B4n%20%C4%90%E1%BB%A9c%20Th%E1%BA%AFng%2C%20t%E1%BB%95%2034%2C%20kh%C3%B3m%203%2C%20Ph%C6%B0%E1%BB%9Dng%201%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Cao%20L%C3%A3nh</t>
+          <t>https://maps.google.com/?q=WinMart+163+T%C3%B4n+%C4%90%E1%BB%A9c+Th%E1%BA%AFng%2C+t%E1%BB%95+34%2C+kh%C3%B3m+3%2C+Ph%C6%B0%E1%BB%9Dng+1%2C+Th%C3%A0nh+ph%E1%BB%91+Cao+L%C3%A3nh</t>
         </is>
       </c>
     </row>
@@ -6354,7 +6354,7 @@
       </c>
       <c r="I141" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20LAN%20468%20Nguy%E1%BB%85n%20%C4%90%C3%ACnh%20Chi%E1%BB%83u%2C%20468%20Nguy%E1%BB%85n%20%C4%90%C3%ACnh%20Chi%E1%BB%83u%2C%20P.%203%2C%20Tp%20T%C3%A2n%20An</t>
+          <t>https://maps.google.com/?q=WinMart+468+Nguy%E1%BB%85n+%C4%90%C3%ACnh+Chi%E1%BB%83u%2C+P.+3%2C+Tp+T%C3%A2n+An</t>
         </is>
       </c>
     </row>
@@ -6399,7 +6399,7 @@
       </c>
       <c r="I142" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20LAN%2069%20H%C3%B9ng%20V%C6%B0%C6%A1ng%2C%2069%20H%C3%B9ng%20V%C6%B0%C6%A1ng%2C%20P.%202%2C%20Tp%20T%C3%A2n%20An</t>
+          <t>https://maps.google.com/?q=WinMart+69+H%C3%B9ng+V%C6%B0%C6%A1ng%2C+P.+2%2C+Tp+T%C3%A2n+An</t>
         </is>
       </c>
     </row>
@@ -6444,7 +6444,7 @@
       </c>
       <c r="I143" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20T%C4%90S%2047%2C%20TB%C4%90%20001%20Ung%20V%C4%83n%20Khi%2C%20Th%E1%BB%ADa%20%C4%91%E1%BA%A5t%20s%E1%BB%91%2047%2C%20t%E1%BB%9D%20b%E1%BA%A3n%20%C4%91%E1%BB%93%20s%E1%BB%91%20001%20t%E1%BA%A1i%20%C4%91%E1%BB%8Ba%20ch%E1%BB%89%2C%20Ung%20V%C4%83n%20Khi%C3%AAm%2C%20Ph%C6%B0%E1%BB%9Dng%20M%E1%BB%B9%20Ph%C6%B0%E1%BB%9Bc%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Long%20Xuy%C3%AAn</t>
+          <t>https://maps.google.com/?q=WinMart+T%C4%90S+47%2C+TB%C4%90+001+Ung+V%C4%83n+Khi%2C+Th%E1%BB%ADa+%C4%91%E1%BA%A5t+s%E1%BB%91+47%2C+t%E1%BB%9D+b%E1%BA%A3n+%C4%91%E1%BB%93+s%E1%BB%91+001+t%E1%BA%A1i+%C4%91%E1%BB%8Ba+ch%E1%BB%89%2C+Ung+V%C4%83n+Khi%C3%AAm%2C+Ph%C6%B0%E1%BB%9Dng+M%E1%BB%B9+Ph%C6%B0%E1%BB%9Bc%2C+Th%C3%A0nh+ph%E1%BB%91+Long+Xuy%C3%AAn</t>
         </is>
       </c>
     </row>
@@ -6489,7 +6489,7 @@
       </c>
       <c r="I144" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20DTP%20669-671%20Ph%E1%BA%A1m%20H%E1%BB%AFu%20L%E1%BA%A7u%2C%20669-671%20t%E1%BB%95%2011%2C%20kh%C3%B3m%202%2C%20%C4%91%C6%B0%E1%BB%9Dng%20Ph%E1%BA%A1m%20H%E1%BB%AFu%20L%E1%BA%A7u%2C%20Ph%C6%B0%E1%BB%9Dng%206%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Cao%20L%C3%A3nh</t>
+          <t>https://maps.google.com/?q=WinMart+669-671+Ph%E1%BA%A1m+H%E1%BB%AFu+L%E1%BA%A7u%2C+669-671+t%E1%BB%95+11%2C+kh%C3%B3m+2%2C+%C4%91%C6%B0%E1%BB%9Dng+Ph%E1%BA%A1m+H%E1%BB%AFu+L%E1%BA%A7u%2C+Ph%C6%B0%E1%BB%9Dng+6%2C+Th%C3%A0nh+ph%E1%BB%91+Cao+L%C3%A3nh</t>
         </is>
       </c>
     </row>
@@ -6534,7 +6534,7 @@
       </c>
       <c r="I145" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20DTP%2074%20Ph%E1%BA%A1m%20H%E1%BB%AFu%20L%E1%BA%A7u%2C%2074%20Ph%E1%BA%A1m%20H%E1%BB%AFu%20L%E1%BA%A7u%2C%20kh%C3%B3m%202%2C%20Ph%C6%B0%E1%BB%9Dng%204%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Cao%20L%C3%A3nh</t>
+          <t>https://maps.google.com/?q=WinMart+74+Ph%E1%BA%A1m+H%E1%BB%AFu+L%E1%BA%A7u%2C+kh%C3%B3m+2%2C+Ph%C6%B0%E1%BB%9Dng+4%2C+Th%C3%A0nh+ph%E1%BB%91+Cao+L%C3%A3nh</t>
         </is>
       </c>
     </row>
@@ -6579,7 +6579,7 @@
       </c>
       <c r="I146" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20493/26%20Qu%E1%BA%A3n%20C%C6%A1%20Th%C3%A0nh%2C%20493/26%20Qu%E1%BA%A3n%20C%C6%A1%20Th%C3%A0nh%2C%20Ph%C6%B0%E1%BB%9Dng%20B%C3%ACnh%20Kh%C3%A1nh%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Long%20Xuy%C3%AAn</t>
+          <t>https://maps.google.com/?q=WinMart+493%2F26+Qu%E1%BA%A3n+C%C6%A1+Th%C3%A0nh%2C+Ph%C6%B0%E1%BB%9Dng+B%C3%ACnh+Kh%C3%A1nh%2C+Th%C3%A0nh+ph%E1%BB%91+Long+Xuy%C3%AAn</t>
         </is>
       </c>
     </row>
@@ -6624,7 +6624,7 @@
       </c>
       <c r="I147" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VM%2B%20DTP%20106-108%20Ton%20Duc%20Thang%2C%20106%2C%20108%20Ton%20Duc%20Thang%2C%20Phuong%20My%20Phu%2C%20Cao%20Lanh%2C%20Dong%20Thap</t>
+          <t>https://maps.google.com/?q=WinMart+106-108+Ton+Duc+Thang%2C+106%2C+108+Ton+Duc+Thang%2C+Phuong+My+Phu%2C+Cao+Lanh%2C+Dong+Thap</t>
         </is>
       </c>
     </row>
@@ -6669,7 +6669,7 @@
       </c>
       <c r="I148" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20Th%E1%BB%ADa%2075%20v%C3%A0%2074%2C%20TB%C4%90%20017%2C%20Th%E1%BB%ADa%2075%20v%C3%A0%2074%2C%20t%E1%BB%9D%20b%E1%BA%A3n%20%C4%91%E1%BB%93%20s%E1%BB%91%20017%20t%E1%BA%A1i%2C%20Ph%C6%B0%E1%BB%9Dng%20M%E1%BB%B9%20Xuy%C3%AAn%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Long%20Xuy%C3%AAn</t>
+          <t>https://maps.google.com/?q=WinMart+Th%E1%BB%ADa+75+v%C3%A0+74%2C+TB%C4%90+017%2C+Th%E1%BB%ADa+75+v%C3%A0+74%2C+t%E1%BB%9D+b%E1%BA%A3n+%C4%91%E1%BB%93+s%E1%BB%91+017+t%E1%BA%A1i%2C+Ph%C6%B0%E1%BB%9Dng+M%E1%BB%B9+Xuy%C3%AAn%2C+Th%C3%A0nh+ph%E1%BB%91+Long+Xuy%C3%AAn</t>
         </is>
       </c>
     </row>
@@ -6714,7 +6714,7 @@
       </c>
       <c r="I149" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20Th%E1%BB%ADa%20173%2C%20TB%C4%90%206%2C%20Th%E1%BB%ADa%20173%2C%20TB%C4%90%206%2C%20M%E1%BB%B9%20Ph%C6%B0%E1%BB%9Bc%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Long%20Xuy%C3%AAn</t>
+          <t>https://maps.google.com/?q=WinMart+Th%E1%BB%ADa+173%2C+TB%C4%90+6%2C+M%E1%BB%B9+Ph%C6%B0%E1%BB%9Bc%2C+Th%C3%A0nh+ph%E1%BB%91+Long+Xuy%C3%AAn</t>
         </is>
       </c>
     </row>
@@ -6759,7 +6759,7 @@
       </c>
       <c r="I150" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VM%2B%20STG%2080%20Ton%20Duc%20Thang%2C%2080%20Ton%20Duc%20Thang%2C%20Phuong%208%2C%20TP%20Soc%20Trang%2C%20tinh%20Soc%20Trang</t>
+          <t>https://maps.google.com/?q=WinMart+80+Ton+Duc+Thang%2C+Phuong+8%2C+TP+Soc+Trang%2C+tinh+Soc+Trang</t>
         </is>
       </c>
     </row>
@@ -6804,7 +6804,7 @@
       </c>
       <c r="I151" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20STG%2062%20%C4%91%C6%B0%E1%BB%9Dng%2030%20th%C3%A1ng%204%2C%2062%20%C4%91%C6%B0%E1%BB%9Dng%2030%20th%C3%A1ng%204%2C%20Ph%C6%B0%E1%BB%9Dng%203%2C%20Th%C3%A0nh%20ph%E1%BB%91%20S%C3%B3c%20Tr%C4%83ng</t>
+          <t>https://maps.google.com/?q=WinMart+62+%C4%91%C6%B0%E1%BB%9Dng+30+th%C3%A1ng+4%2C+Ph%C6%B0%E1%BB%9Dng+3%2C+Th%C3%A0nh+ph%E1%BB%91+S%C3%B3c+Tr%C4%83ng</t>
         </is>
       </c>
     </row>
@@ -6849,7 +6849,7 @@
       </c>
       <c r="I152" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20LAN%2010-11-12%20Tr%C6%B0%C6%A1ng%20%C4%90%E1%BB%8Bnh%2C%2010-11-12%20Tr%C6%B0%C6%A1ng%20%C4%90%E1%BB%8Bnh%2C%20P%201%2C%20Tp%20T%C3%A2n%20An</t>
+          <t>https://maps.google.com/?q=WinMart+10-11-12+Tr%C6%B0%C6%A1ng+%C4%90%E1%BB%8Bnh%2C+P+1%2C+Tp+T%C3%A2n+An</t>
         </is>
       </c>
     </row>
@@ -6894,7 +6894,7 @@
       </c>
       <c r="I153" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VM%2B%20DTP%20335-337%20Duong%2030/4%2C%20335-337%20duong%2030/4%2C%20phuong%201%2C%20thanh%20pho%20Cao%20Lanh%2C%20Dong%20Thap</t>
+          <t>https://maps.google.com/?q=WinMart+335-337+duong+30%2F4%2C+phuong+1%2C+thanh+pho+Cao+Lanh%2C+Dong+Thap</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="I154" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CMU%20128%20h%E1%BA%BBm%20B%C3%AA%20T%C3%B4ng%2C%20Nguy%E1%BB%85n%20Tr%C3%A3%2C%20128%20h%E1%BA%BBm%20B%C3%AA%20T%C3%B4ng%2C%20Nguy%E1%BB%85n%20Tr%C3%A3i%2C%20Ph%C6%B0%E1%BB%9Dng%209%2C%20Th%C3%A0nh%20ph%E1%BB%91%20C%C3%A0%20Mau</t>
+          <t>https://maps.google.com/?q=WinMart+128+h%E1%BA%BBm+B%C3%AA+T%C3%B4ng%2C+Nguy%E1%BB%85n+Tr%C3%A3i%2C+Ph%C6%B0%E1%BB%9Dng+9%2C+Th%C3%A0nh+ph%E1%BB%91+C%C3%A0+Mau</t>
         </is>
       </c>
     </row>
@@ -6984,7 +6984,7 @@
       </c>
       <c r="I155" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VM%2B%20CMU%2081%20Hung%20Vuong%2C%2081%20duong%20Hung%20Vuong%2C%20khom%204%2C%20phuong%205%2C%20TP%20Ca%20Mau%2C%20tinh%20Ca%20Mau.</t>
+          <t>https://maps.google.com/?q=WinMart+81+Hung+Vuong%2C+81+duong+Hung+Vuong%2C+khom+4%2C+phuong+5%2C+TP+Ca+Mau%2C+tinh+Ca+Mau.</t>
         </is>
       </c>
     </row>
@@ -7029,7 +7029,7 @@
       </c>
       <c r="I156" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20DTP%2098%20L%C3%AA%20L%E1%BB%A3i%2C%2098%20L%C3%AA%20L%E1%BB%A3i%2C%20Ph%C6%B0%E1%BB%9Dng%202%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Cao%20L%C3%A3nh</t>
+          <t>https://maps.google.com/?q=WinMart+98+L%C3%AA+L%E1%BB%A3i%2C+Ph%C6%B0%E1%BB%9Dng+2%2C+Th%C3%A0nh+ph%E1%BB%91+Cao+L%C3%A3nh</t>
         </is>
       </c>
     </row>
@@ -7074,7 +7074,7 @@
       </c>
       <c r="I157" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CMU%20418%20Tr%E1%BA%A7n%20V%C4%83n%20Th%E1%BB%9Di%2C%20418%20Tr%E1%BA%A7n%20V%C4%83n%20Th%E1%BB%9Di%2C%20Kh%C3%B3m%203%2C%20Ph%C6%B0%E1%BB%9Dng%206%2C%20Th%C3%A0nh%20ph%E1%BB%91%20C%C3%A0%20Mau</t>
+          <t>https://maps.google.com/?q=WinMart+418+Tr%E1%BA%A7n+V%C4%83n+Th%E1%BB%9Di%2C+Kh%C3%B3m+3%2C+Ph%C6%B0%E1%BB%9Dng+6%2C+Th%C3%A0nh+ph%E1%BB%91+C%C3%A0+Mau</t>
         </is>
       </c>
     </row>
@@ -7119,7 +7119,7 @@
       </c>
       <c r="I158" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CMU%20517%20Nguy%E1%BB%85n%20T%E1%BA%A5t%20Th%C3%A0nh%2C%20517%20Nguy%E1%BB%85n%20T%E1%BA%A5t%20Th%C3%A0nh%2C%20X%C3%A3%20L%C3%BD%20V%C4%83n%2C%20L%C3%A2m%2C%20Th%C3%A0nh%20ph%E1%BB%91%20C%C3%A0%20Mau</t>
+          <t>https://maps.google.com/?q=WinMart+517+Nguy%E1%BB%85n+T%E1%BA%A5t+Th%C3%A0nh%2C+X%C3%A3+L%C3%BD+V%C4%83n%2C+L%C3%A2m%2C+Th%C3%A0nh+ph%E1%BB%91+C%C3%A0+Mau</t>
         </is>
       </c>
     </row>
@@ -7164,7 +7164,7 @@
       </c>
       <c r="I159" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20BTE%2080%20Nguy%E1%BB%85n%20Hu%E1%BB%87%2C%2080%20Nguy%E1%BB%85n%20Hu%E1%BB%87%2C%20Ph%C6%B0%E1%BB%9Dng%20An%20H%E1%BB%99i%2C%20Th%C3%A0nh%20ph%E1%BB%91%20B%E1%BA%BFn%20Tre</t>
+          <t>https://maps.google.com/?q=WinMart+80+Nguy%E1%BB%85n+Hu%E1%BB%87%2C+Ph%C6%B0%E1%BB%9Dng+An+H%E1%BB%99i%2C+Th%C3%A0nh+ph%E1%BB%91+B%E1%BA%BFn+Tre</t>
         </is>
       </c>
     </row>
@@ -7209,7 +7209,7 @@
       </c>
       <c r="I160" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20LAN%20218/2%20%E1%BA%A4p%20X%C3%B3m%20C%E1%BB%91ng%2C%20218/2%20%E1%BA%A4p%20X%C3%B3m%20C%E1%BB%91ng%2C%20Th%E1%BB%8B%20tr%E1%BA%A5n%20B%E1%BA%BFn%20L%E1%BB%A9c%2C%20Huy%E1%BB%87n%20B%E1%BA%BFn%20L%E1%BB%A9c</t>
+          <t>https://maps.google.com/?q=WinMart+218%2F2+%E1%BA%A4p+X%C3%B3m+C%E1%BB%91ng%2C+Th%E1%BB%8B+tr%E1%BA%A5n+B%E1%BA%BFn+L%E1%BB%A9c%2C+Huy%E1%BB%87n+B%E1%BA%BFn+L%E1%BB%A9c</t>
         </is>
       </c>
     </row>
@@ -7254,7 +7254,7 @@
       </c>
       <c r="I161" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20BTE%20298F%20Khu%20ph%E1%BB%91%202%2C%20298F%20Nguy%E1%BB%85n%20Hu%E1%BB%87%2C%20khu%20ph%E1%BB%91%202%2C%20Ph%C6%B0%E1%BB%9Dng%20Ph%C3%BA%20Kh%C6%B0%C6%A1ng%2C%20Th%C3%A0nh%20ph%E1%BB%91%20B%E1%BA%BFn%20Tre</t>
+          <t>https://maps.google.com/?q=WinMart+298F+Khu+ph%E1%BB%91+2%2C+298F+Nguy%E1%BB%85n+Hu%E1%BB%87%2C+khu+ph%E1%BB%91+2%2C+Ph%C6%B0%E1%BB%9Dng+Ph%C3%BA+Kh%C6%B0%C6%A1ng%2C+Th%C3%A0nh+ph%E1%BB%91+B%E1%BA%BFn+Tre</t>
         </is>
       </c>
     </row>
@@ -7299,7 +7299,7 @@
       </c>
       <c r="I162" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20BTE%20401B%20Nguy%E1%BB%85n%20%C4%90%C3%ACnh%20Chi%E1%BB%83u%2C%20401B%20Nguy%E1%BB%85n%20%C4%90%C3%ACnh%20Chi%E1%BB%83u%2C%20Ph%C6%B0%E1%BB%9Dng%208%2C%20Th%C3%A0nh%20ph%E1%BB%91%20B%E1%BA%BFn%20Tre</t>
+          <t>https://maps.google.com/?q=WinMart+401B+Nguy%E1%BB%85n+%C4%90%C3%ACnh+Chi%E1%BB%83u%2C+Ph%C6%B0%E1%BB%9Dng+8%2C+Th%C3%A0nh+ph%E1%BB%91+B%E1%BA%BFn+Tre</t>
         </is>
       </c>
     </row>
@@ -7344,7 +7344,7 @@
       </c>
       <c r="I163" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20BTE%20261K%20%C4%90%C6%B0%E1%BB%9Dng%20S%E1%BB%91%201%2C%20261K%20%C4%90%C6%B0%E1%BB%9Dng%20s%E1%BB%91%201%2C%20Khu%20ph%E1%BB%91%20III%2C%20Ph%C6%B0%E1%BB%9Dng%20Ph%C3%BA%20T%C3%A2n%2C%20Th%C3%A0nh%20ph%E1%BB%91%20B%E1%BA%BFn%20Tre</t>
+          <t>https://maps.google.com/?q=WinMart+261K+%C4%90%C6%B0%E1%BB%9Dng+s%E1%BB%91+1%2C+Khu+ph%E1%BB%91+III%2C+Ph%C6%B0%E1%BB%9Dng+Ph%C3%BA+T%C3%A2n%2C+Th%C3%A0nh+ph%E1%BB%91+B%E1%BA%BFn+Tre</t>
         </is>
       </c>
     </row>
@@ -7389,7 +7389,7 @@
       </c>
       <c r="I164" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20BTE%2063/2%20Phan%20%C4%90%C3%ACnh%20Ph%C3%B9ng%2C%2063/2%20Phan%20%C4%90%C3%ACnh%20Ph%C3%B9ng%2C%20Ph%C6%B0%E1%BB%9Dng%204%2C%20Th%C3%A0nh%20ph%E1%BB%91%20B%E1%BA%BFn%20Tre</t>
+          <t>https://maps.google.com/?q=WinMart+63%2F2+Phan+%C4%90%C3%ACnh+Ph%C3%B9ng%2C+Ph%C6%B0%E1%BB%9Dng+4%2C+Th%C3%A0nh+ph%E1%BB%91+B%E1%BA%BFn+Tre</t>
         </is>
       </c>
     </row>
@@ -7434,7 +7434,7 @@
       </c>
       <c r="I165" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TVH%2028-29%20H%C3%B9ng%20V%C6%B0%C6%A1ng%2C%2028-29%20H%C3%B9ng%20V%C6%B0%C6%A1ng%2C%20kh%C3%B3m%202%2C%20Ph%C6%B0%E1%BB%9Dng%205%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Tr%C3%A0%20Vinh</t>
+          <t>https://maps.google.com/?q=WinMart+28-29+H%C3%B9ng+V%C6%B0%C6%A1ng%2C+kh%C3%B3m+2%2C+Ph%C6%B0%E1%BB%9Dng+5%2C+Th%C3%A0nh+ph%E1%BB%91+Tr%C3%A0+Vinh</t>
         </is>
       </c>
     </row>
@@ -7479,7 +7479,7 @@
       </c>
       <c r="I166" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VM%2B%20TVH%20142A%20Nguyen%20Dang%2C%20142A%20Nguyen%20Dang%2C%20khom%208%2C%20phuong%206%2C%20TP%20Tra%20Vinh%2C%20tinh%20Tra%20Vinh</t>
+          <t>https://maps.google.com/?q=WinMart+142A+Nguyen+Dang%2C+khom+8%2C+phuong+6%2C+TP+Tra+Vinh%2C+tinh+Tra+Vinh</t>
         </is>
       </c>
     </row>
@@ -7524,7 +7524,7 @@
       </c>
       <c r="I167" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TVH%20491%20Nguy%E1%BB%85n%20Th%E1%BB%8B%20Minh%20Khai%2C%20491%20Nguy%E1%BB%85n%20Th%E1%BB%8B%20Minh%20Khai%2C%20kh%C3%B3m%207%2C%20Ph%C6%B0%E1%BB%9Dng%207%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Tr%C3%A0%20Vinh</t>
+          <t>https://maps.google.com/?q=WinMart+491+Nguy%E1%BB%85n+Th%E1%BB%8B+Minh+Khai%2C+kh%C3%B3m+7%2C+Ph%C6%B0%E1%BB%9Dng+7%2C+Th%C3%A0nh+ph%E1%BB%91+Tr%C3%A0+Vinh</t>
         </is>
       </c>
     </row>
@@ -7569,7 +7569,7 @@
       </c>
       <c r="I168" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VM%2B%20BTE%20116A1%20Truong%20Dinh%2C%20116A1%20Truong%20Dinh%2C%20khu%20pho%20Binh%20Khoi%2C%20Phuong%206%2C%20Thanh%20pho%20Ben%20Tre</t>
+          <t>https://maps.google.com/?q=WinMart+116A1+Truong+Dinh%2C+khu+pho+Binh+Khoi%2C+Phuong+6%2C+Thanh+pho+Ben+Tre</t>
         </is>
       </c>
     </row>
@@ -7614,7 +7614,7 @@
       </c>
       <c r="I169" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CMU%20168%20L%C3%BD%20Th%C6%B0%E1%BB%9Dng%20Ki%E1%BB%87t%2C%20168%20L%C3%BD%20Th%C6%B0%E1%BB%9Dng%20Ki%E1%BB%87t%2C%20Ph%C6%B0%E1%BB%9Dng%206%2C%20Th%C3%A0nh%20ph%E1%BB%91%20C%C3%A0%20Mau</t>
+          <t>https://maps.google.com/?q=WinMart+168+L%C3%BD+Th%C6%B0%E1%BB%9Dng+Ki%E1%BB%87t%2C+Ph%C6%B0%E1%BB%9Dng+6%2C+Th%C3%A0nh+ph%E1%BB%91+C%C3%A0+Mau</t>
         </is>
       </c>
     </row>
@@ -7659,7 +7659,7 @@
       </c>
       <c r="I170" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TVH%20363%20kh%C3%B3m%208%2C%20363%2C%20kh%C3%B3m%208%2C%20Ph%C6%B0%E1%BB%9Dng%207%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Tr%C3%A0%20Vinh</t>
+          <t>https://maps.google.com/?q=WinMart+363+kh%C3%B3m+8%2C+363%2C+kh%C3%B3m+8%2C+Ph%C6%B0%E1%BB%9Dng+7%2C+Th%C3%A0nh+ph%E1%BB%91+Tr%C3%A0+Vinh</t>
         </is>
       </c>
     </row>
@@ -7704,7 +7704,7 @@
       </c>
       <c r="I171" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TVH%20214%20L%C3%AA%20L%E1%BB%A3i%2C%20214%20%C4%91%C6%B0%E1%BB%9Dng%20L%C3%AA%20L%E1%BB%A3i%2C%20kh%C3%B3m%201%2C%20Ph%C6%B0%E1%BB%9Dng%201%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Tr%C3%A0%20Vinh</t>
+          <t>https://maps.google.com/?q=WinMart+214+L%C3%AA+L%E1%BB%A3i%2C+214+%C4%91%C6%B0%E1%BB%9Dng+L%C3%AA+L%E1%BB%A3i%2C+kh%C3%B3m+1%2C+Ph%C6%B0%E1%BB%9Dng+1%2C+Th%C3%A0nh+ph%E1%BB%91+Tr%C3%A0+Vinh</t>
         </is>
       </c>
     </row>
@@ -7749,7 +7749,7 @@
       </c>
       <c r="I172" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TGG%2042/4%20Nguy%E1%BB%85n%20Hu%E1%BB%B3nh%20%C4%90%E1%BB%A9c%2C%2042/4%20Nguy%E1%BB%85n%20Hu%E1%BB%B3nh%20%C4%90%E1%BB%A9c%2C%20Ph%C6%B0%E1%BB%9Dng%208%2C%20Th%C3%A0nh%20Ph%E1%BB%91%20M%E1%BB%B9%20Tho</t>
+          <t>https://maps.google.com/?q=WinMart+42%2F4+Nguy%E1%BB%85n+Hu%E1%BB%B3nh+%C4%90%E1%BB%A9c%2C+Ph%C6%B0%E1%BB%9Dng+8%2C+Th%C3%A0nh+Ph%E1%BB%91+M%E1%BB%B9+Tho</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="I173" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20STG%20177%20Nguy%E1%BB%85n%20Hu%E1%BB%87%2C%20177%20Nguy%E1%BB%85n%20Hu%E1%BB%87%2C%20kh%C3%B3m%203%2C%20Ph%C6%B0%E1%BB%9Dng%201%2C%20TX.%20S%C3%B3c%20Tr%C4%83ng%2C%20Th%C3%A0nh%20ph%E1%BB%91%20S%C3%B3c%20Tr%C4%83ng</t>
+          <t>https://maps.google.com/?q=WinMart+177+Nguy%E1%BB%85n+Hu%E1%BB%87%2C+kh%C3%B3m+3%2C+Ph%C6%B0%E1%BB%9Dng+1%2C+TX.+S%C3%B3c+Tr%C4%83ng%2C+Th%C3%A0nh+ph%E1%BB%91+S%C3%B3c+Tr%C4%83ng</t>
         </is>
       </c>
     </row>
@@ -7839,7 +7839,7 @@
       </c>
       <c r="I174" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TVH%2057%20%C4%90%E1%BB%93ng%20Kh%E1%BB%9Fi%2C%2057%20%C4%91%C6%B0%E1%BB%9Dng%20%C4%90%E1%BB%93ng%20Kh%E1%BB%9Fi%2C%20kh%C3%B3m%209%2C%20Ph%C6%B0%E1%BB%9Dng%206%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Tr%C3%A0%20Vinh</t>
+          <t>https://maps.google.com/?q=WinMart+57+%C4%90%E1%BB%93ng+Kh%E1%BB%9Fi%2C+57+%C4%91%C6%B0%E1%BB%9Dng+%C4%90%E1%BB%93ng+Kh%E1%BB%9Fi%2C+kh%C3%B3m+9%2C+Ph%C6%B0%E1%BB%9Dng+6%2C+Th%C3%A0nh+ph%E1%BB%91+Tr%C3%A0+Vinh</t>
         </is>
       </c>
     </row>
@@ -7884,7 +7884,7 @@
       </c>
       <c r="I175" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20BTE%20600B1%20Nguy%E1%BB%85n%20Th%E1%BB%8B%20%C4%90%E1%BB%8Bnh%2C%20600B1%20Nguy%E1%BB%85n%20Th%E1%BB%8B%20%C4%90%E1%BB%8Bnh%2C%20Ph%C6%B0%E1%BB%9Dng%20Ph%C3%BA%20Kh%C6%B0%C6%A1ng%2C%20Th%C3%A0nh%20ph%E1%BB%91%20B%E1%BA%BFn%20Tre</t>
+          <t>https://maps.google.com/?q=WinMart+600B1+Nguy%E1%BB%85n+Th%E1%BB%8B+%C4%90%E1%BB%8Bnh%2C+Ph%C6%B0%E1%BB%9Dng+Ph%C3%BA+Kh%C6%B0%C6%A1ng%2C+Th%C3%A0nh+ph%E1%BB%91+B%E1%BA%BFn+Tre</t>
         </is>
       </c>
     </row>
@@ -7929,7 +7929,7 @@
       </c>
       <c r="I176" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20STG%20491%20L%C3%AA%20H%E1%BB%93ng%20Phong%2C%20491%20L%C3%AA%20H%E1%BB%93ng%20Phong%2C%20kh%C3%B3m%205%2C%20Ph%C6%B0%E1%BB%9Dng%203%2C%20Th%C3%A0nh%20ph%E1%BB%91%20S%C3%B3c%20Tr%C4%83ng</t>
+          <t>https://maps.google.com/?q=WinMart+491+L%C3%AA+H%E1%BB%93ng+Phong%2C+kh%C3%B3m+5%2C+Ph%C6%B0%E1%BB%9Dng+3%2C+Th%C3%A0nh+ph%E1%BB%91+S%C3%B3c+Tr%C4%83ng</t>
         </is>
       </c>
     </row>
@@ -7974,7 +7974,7 @@
       </c>
       <c r="I177" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20STG%20176%20L%C3%AA%20H%E1%BB%93ng%20Phong%2C%20176%20L%C3%AA%20H%E1%BB%93ng%20Phong%2C%20kh%C3%B3m%204%2C%20Ph%C6%B0%E1%BB%9Dng%203%2C%20Th%C3%A0nh%20ph%E1%BB%91%20S%C3%B3c%20Tr%C4%83ng</t>
+          <t>https://maps.google.com/?q=WinMart+176+L%C3%AA+H%E1%BB%93ng+Phong%2C+kh%C3%B3m+4%2C+Ph%C6%B0%E1%BB%9Dng+3%2C+Th%C3%A0nh+ph%E1%BB%91+S%C3%B3c+Tr%C4%83ng</t>
         </is>
       </c>
     </row>
@@ -8019,7 +8019,7 @@
       </c>
       <c r="I178" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CMU%2013%20%C4%90o%C3%A0n%20Th%E1%BB%8B%20%C4%90i%E1%BB%83m%2C%2013%20%C4%90o%C3%A0n%20Th%E1%BB%8B%20%C4%90i%E1%BB%83m%2C%20Ph%C6%B0%E1%BB%9Dng%207%2C%20Th%C3%A0nh%20ph%E1%BB%91%20C%C3%A0%20Mau</t>
+          <t>https://maps.google.com/?q=WinMart+13+%C4%90o%C3%A0n+Th%E1%BB%8B+%C4%90i%E1%BB%83m%2C+Ph%C6%B0%E1%BB%9Dng+7%2C+Th%C3%A0nh+ph%E1%BB%91+C%C3%A0+Mau</t>
         </is>
       </c>
     </row>
@@ -8064,7 +8064,7 @@
       </c>
       <c r="I179" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CMU%20127%20Nguy%E1%BB%85n%20C%C3%B4ng%20Tr%E1%BB%A9%2C%20127%20Nguy%E1%BB%85n%20C%C3%B4ng%20Tr%E1%BB%A9%2C%20Ph%C6%B0%E1%BB%9Dng%208%2C%20Th%C3%A0nh%20ph%E1%BB%91%20C%C3%A0%20Mau</t>
+          <t>https://maps.google.com/?q=WinMart+127+Nguy%E1%BB%85n+C%C3%B4ng+Tr%E1%BB%A9%2C+Ph%C6%B0%E1%BB%9Dng+8%2C+Th%C3%A0nh+ph%E1%BB%91+C%C3%A0+Mau</t>
         </is>
       </c>
     </row>
@@ -8109,7 +8109,7 @@
       </c>
       <c r="I180" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CMU%2069%20Ph%E1%BA%A1m%20H%E1%BB%93ng%20Th%C3%A1m%2C%2069%20Ph%E1%BA%A1m%20H%E1%BB%93ng%20Th%C3%A1m%2C%20Ph%C6%B0%E1%BB%9Dng%204%2C%20Th%C3%A0nh%20ph%E1%BB%91%20C%C3%A0%20Mau</t>
+          <t>https://maps.google.com/?q=WinMart+69+Ph%E1%BA%A1m+H%E1%BB%93ng+Th%C3%A1m%2C+Ph%C6%B0%E1%BB%9Dng+4%2C+Th%C3%A0nh+ph%E1%BB%91+C%C3%A0+Mau</t>
         </is>
       </c>
     </row>
@@ -8154,7 +8154,7 @@
       </c>
       <c r="I181" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TVH%20120%20Tr%E1%BA%A7n%20Qu%E1%BB%91c%20Tu%E1%BA%A5n%2C%20120%20Tr%E1%BA%A7n%20Qu%E1%BB%91c%20Tu%E1%BA%A5n%2C%20Ph%C6%B0%E1%BB%9Dng%202%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Tr%C3%A0%20Vinh</t>
+          <t>https://maps.google.com/?q=WinMart+120+Tr%E1%BA%A7n+Qu%E1%BB%91c+Tu%E1%BA%A5n%2C+Ph%C6%B0%E1%BB%9Dng+2%2C+Th%C3%A0nh+ph%E1%BB%91+Tr%C3%A0+Vinh</t>
         </is>
       </c>
     </row>
@@ -8199,7 +8199,7 @@
       </c>
       <c r="I182" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20141/5%20Nguy%E1%BB%85n%20Th%C3%A1i%20H%E1%BB%8Dc%2C%20141/5%20Nguy%E1%BB%85n%20Th%C3%A1i%20H%E1%BB%8Dc%2C%20Ph%C6%B0%E1%BB%9Dng%20M%E1%BB%B9%20B%C3%ACnh%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Long%20Xuy%C3%AAn</t>
+          <t>https://maps.google.com/?q=WinMart+141%2F5+Nguy%E1%BB%85n+Th%C3%A1i+H%E1%BB%8Dc%2C+Ph%C6%B0%E1%BB%9Dng+M%E1%BB%B9+B%C3%ACnh%2C+Th%C3%A0nh+ph%E1%BB%91+Long+Xuy%C3%AAn</t>
         </is>
       </c>
     </row>
@@ -8244,7 +8244,7 @@
       </c>
       <c r="I183" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TVH%2010%20Ph%E1%BA%A1m%20H%E1%BB%93ng%20Th%C3%A1i%2C%2010%20Ph%E1%BA%A1m%20H%E1%BB%93ng%20Th%C3%A1i%2C%20kh%C3%B3m%203%2C%20Ph%C6%B0%E1%BB%9Dng%203%2C%20Th%C3%A0nh%20ph%E1%BB%91%20Tr%C3%A0%20Vinh</t>
+          <t>https://maps.google.com/?q=WinMart+10+Ph%E1%BA%A1m+H%E1%BB%93ng+Th%C3%A1i%2C+kh%C3%B3m+3%2C+Ph%C6%B0%E1%BB%9Dng+3%2C+Th%C3%A0nh+ph%E1%BB%91+Tr%C3%A0+Vinh</t>
         </is>
       </c>
     </row>
@@ -8289,7 +8289,7 @@
       </c>
       <c r="I184" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VM%2B%20LAN%20320%20Quoc%20lo%2062%2C%20320%20Quoc%20lo%2062%2C%20Phuong%206%2C%20Thanh%20pho%20Tan%20An%2C%20Tinh%20Long%20An</t>
+          <t>https://maps.google.com/?q=WinMart+320+Quoc+lo+62%2C+Phuong+6%2C+Thanh+pho+Tan+An%2C+Tinh+Long+An</t>
         </is>
       </c>
     </row>
@@ -8334,7 +8334,7 @@
       </c>
       <c r="I185" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20STG%2078%20M%E1%BA%A1c%20%C4%90%E1%BB%89nh%20Chi%2C%2078%20M%E1%BA%A1c%20%C4%90%E1%BB%89nh%20Chi%2C%20kh%C3%B3m%203%2C%20Ph%C6%B0%E1%BB%9Dng%209%2C%20Th%C3%A0nh%20ph%E1%BB%91%20S%C3%B3c%20Tr%C4%83ng</t>
+          <t>https://maps.google.com/?q=WinMart+78+M%E1%BA%A1c+%C4%90%E1%BB%89nh+Chi%2C+kh%C3%B3m+3%2C+Ph%C6%B0%E1%BB%9Dng+9%2C+Th%C3%A0nh+ph%E1%BB%91+S%C3%B3c+Tr%C4%83ng</t>
         </is>
       </c>
     </row>
@@ -8379,7 +8379,7 @@
       </c>
       <c r="I186" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20225%20Tho%E1%BA%A1i%20Ng%E1%BB%8Dc%20H%E1%BA%A7u%2C%20225%2C%20%C4%91%C6%B0%E1%BB%9Dng%20Tho%E1%BA%A1i%20Ng%E1%BB%8Dc%20H%E1%BA%A7u%2C%20kh%C3%B3m%20%C4%90%C3%B4ng%20Th%E1%BB%8Bnh%203%2C%20P.%20M%E1%BB%B9%20Ph%C6%B0%E1%BB%9Bc%2C%20TP.%20Long%20Xuy%C3%AAn</t>
+          <t>https://maps.google.com/?q=WinMart+225+Tho%E1%BA%A1i+Ng%E1%BB%8Dc+H%E1%BA%A7u%2C+225%2C+%C4%91%C6%B0%E1%BB%9Dng+Tho%E1%BA%A1i+Ng%E1%BB%8Dc+H%E1%BA%A7u%2C+kh%C3%B3m+%C4%90%C3%B4ng+Th%E1%BB%8Bnh+3%2C+P.+M%E1%BB%B9+Ph%C6%B0%E1%BB%9Bc%2C+TP.+Long+Xuy%C3%AAn</t>
         </is>
       </c>
     </row>
@@ -8424,7 +8424,7 @@
       </c>
       <c r="I187" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20LAN%201B%20Tr%E1%BA%A7n%20Phong%20S%E1%BA%AFc%2C%201B%20Tr%E1%BA%A7n%20Phong%20S%E1%BA%AFc%2C%20Ph%C6%B0%E1%BB%9Dng%204%2C%20TP%20T%C3%A2n%20An</t>
+          <t>https://maps.google.com/?q=WinMart+1B+Tr%E1%BA%A7n+Phong+S%E1%BA%AFc%2C+Ph%C6%B0%E1%BB%9Dng+4%2C+TP+T%C3%A2n+An</t>
         </is>
       </c>
     </row>
@@ -8469,7 +8469,7 @@
       </c>
       <c r="I188" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20LAN%20236A%20%E2%80%93%20238%20Ch%C3%A2u%20Th%E1%BB%8B%20Kim%2C%20236A%20%E2%80%93%20238%20Ch%C3%A2u%20Th%E1%BB%8B%20Kim%2C%20KP%20B%C3%ACnh%20An%202%2C%20Ph%C6%B0%E1%BB%9Dng%207%2C%20TP%20T%C3%A2n%20An</t>
+          <t>https://maps.google.com/?q=WinMart+236A+%E2%80%93+238+Ch%C3%A2u+Th%E1%BB%8B+Kim%2C+KP+B%C3%ACnh+An+2%2C+Ph%C6%B0%E1%BB%9Dng+7%2C+TP+T%C3%A2n+An</t>
         </is>
       </c>
     </row>
@@ -8514,7 +8514,7 @@
       </c>
       <c r="I189" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20LAN%2078%20Nguy%E1%BB%85n%20C%E1%BB%ADu%20V%C3%A2n%2C%2078%20Nguy%E1%BB%85n%20C%E1%BB%ADu%20V%C3%A2n%2C%20Ph%C6%B0%E1%BB%9Dng%204%2C%20Th%C3%A0nh%20ph%E1%BB%91%20T%C3%A2n%20An</t>
+          <t>https://maps.google.com/?q=WinMart+78+Nguy%E1%BB%85n+C%E1%BB%ADu+V%C3%A2n%2C+Ph%C6%B0%E1%BB%9Dng+4%2C+Th%C3%A0nh+ph%E1%BB%91+T%C3%A2n+An</t>
         </is>
       </c>
     </row>
@@ -8559,7 +8559,7 @@
       </c>
       <c r="I190" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CMU%20758%20%C4%91%C6%B0%E1%BB%9Dng%20Ng%C3%B4%20Quy%E1%BB%81n%2C%20758%2C%20%C4%91%C6%B0%E1%BB%9Dng%20Ng%C3%B4%20Quy%E1%BB%81n%2C%20P.%201%2C%20TP.%20C%C3%A0%20Mau</t>
+          <t>https://maps.google.com/?q=WinMart+758+%C4%91%C6%B0%E1%BB%9Dng+Ng%C3%B4+Quy%E1%BB%81n%2C+758%2C+%C4%91%C6%B0%E1%BB%9Dng+Ng%C3%B4+Quy%E1%BB%81n%2C+P.+1%2C+TP.+C%C3%A0+Mau</t>
         </is>
       </c>
     </row>
@@ -8604,7 +8604,7 @@
       </c>
       <c r="I191" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%201%20Nguy%E1%BB%85n%20Tr%C6%B0%E1%BB%9Dng%20T%E1%BB%99%2C%201%20Nguy%E1%BB%85n%20Tr%C6%B0%E1%BB%9Dng%20T%E1%BB%99%2C%20P.%20B%C3%ACnh%20Kh%C3%A1nh%2C%20TP.%20Long%20Xuy%C3%AAn</t>
+          <t>https://maps.google.com/?q=WinMart+1+Nguy%E1%BB%85n+Tr%C6%B0%E1%BB%9Dng+T%E1%BB%99%2C+P.+B%C3%ACnh+Kh%C3%A1nh%2C+TP.+Long+Xuy%C3%AAn</t>
         </is>
       </c>
     </row>
@@ -8649,7 +8649,7 @@
       </c>
       <c r="I192" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TGG%206A%20Nguy%E1%BB%85n%20Hu%E1%BB%87%2C%206A%20Nguy%E1%BB%85n%20Hu%E1%BB%87%2C%20KP.%201%2C%20P.%202%2C%20TX.%20G%C3%B2%20C%C3%B4ng</t>
+          <t>https://maps.google.com/?q=WinMart+6A+Nguy%E1%BB%85n+Hu%E1%BB%87%2C+KP.+1%2C+P.+2%2C+TX.+G%C3%B2+C%C3%B4ng</t>
         </is>
       </c>
     </row>
@@ -8694,7 +8694,7 @@
       </c>
       <c r="I193" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TGG%202%20%C4%91%C6%B0%E1%BB%9Dng%20Nguy%E1%BB%85n%20Tr%C3%A3i%2C%202%20%C4%91%C6%B0%E1%BB%9Dng%20Nguy%E1%BB%85n%20Tr%C3%A3i%2C%20KP.%202%2C%20P.%202%2C%20TX.%20G%C3%B2%20C%C3%B4ng</t>
+          <t>https://maps.google.com/?q=WinMart+2+%C4%91%C6%B0%E1%BB%9Dng+Nguy%E1%BB%85n+Tr%C3%A3i%2C+KP.+2%2C+P.+2%2C+TX.+G%C3%B2+C%C3%B4ng</t>
         </is>
       </c>
     </row>
@@ -8739,7 +8739,7 @@
       </c>
       <c r="I194" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TVH%20320A%20Ph%E1%BA%A1m%20Ng%C5%A9%20L%C3%A3o%2C%20320A%20Ph%E1%BA%A1m%20Ng%C5%A9%20L%C3%A3o%2C%20Kh%C3%B3m%203%2C%20P.%201%2C%20TP%20Tr%C3%A0%20Vinh</t>
+          <t>https://maps.google.com/?q=WinMart+320A+Ph%E1%BA%A1m+Ng%C5%A9+L%C3%A3o%2C+Kh%C3%B3m+3%2C+P.+1%2C+TP+Tr%C3%A0+Vinh</t>
         </is>
       </c>
     </row>
@@ -8784,7 +8784,7 @@
       </c>
       <c r="I195" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=VM%2B%20STG%20106%20Tr%E1%BA%A7n%20H%C6%B0ng%20%C4%90%E1%BA%A1o%2C%20106%20Tr%E1%BA%A7n%20H%C6%B0ng%20%C4%90%E1%BA%A1o%2C%20Kh%C3%B3m%202%2C%20P.%202%2C%20TP.%20S%C3%B3c%20Tr%C4%83ng</t>
+          <t>https://maps.google.com/?q=WinMart+106+Tr%E1%BA%A7n+H%C6%B0ng+%C4%90%E1%BA%A1o%2C+Kh%C3%B3m+2%2C+P.+2%2C+TP.+S%C3%B3c+Tr%C4%83ng</t>
         </is>
       </c>
     </row>
@@ -8829,7 +8829,7 @@
       </c>
       <c r="I196" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20210%20Th%E1%BB%A5c%20Ph%C3%A1n%2C%20210%20%C4%91%C6%B0%E1%BB%9Dng%20Th%E1%BB%A5c%20Ph%C3%A1n%20%E2%80%93%20K%C4%90T%20Sao%20Mai%20B%C3%ACnh%20Kh%C3%A1nh%203%20%2C%20K.%20B%C3%ACnh%20Kh%C3%A1nh%207%2C%20P.%20B%C3%ACnh%20Kh%C3%A1nh</t>
+          <t>https://maps.google.com/?q=WinMart+210+Th%E1%BB%A5c+Ph%C3%A1n%2C+210+%C4%91%C6%B0%E1%BB%9Dng+Th%E1%BB%A5c+Ph%C3%A1n+%E2%80%93+K%C4%90T+Sao+Mai+B%C3%ACnh+Kh%C3%A1nh+3+%2C+K.+B%C3%ACnh+Kh%C3%A1nh+7%2C+P.+B%C3%ACnh+Kh%C3%A1nh</t>
         </is>
       </c>
     </row>
@@ -8874,7 +8874,7 @@
       </c>
       <c r="I197" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CMU%2010%20L%C3%AA%20H%E1%BB%93ng%20Phong%2C%2010%20L%C3%AA%20H%E1%BB%93ng%20Phong%2C%20P.%208%2C%20TP.%20C%C3%A0%20Mau</t>
+          <t>https://maps.google.com/?q=WinMart+10+L%C3%AA+H%E1%BB%93ng+Phong%2C+P.+8%2C+TP.+C%C3%A0+Mau</t>
         </is>
       </c>
     </row>
@@ -8919,7 +8919,7 @@
       </c>
       <c r="I198" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TGG%20339%20Qu%E1%BB%91c%20L%E1%BB%99%2050%2C%20S%E1%BB%91%20339%20Qu%E1%BB%91c%20L%E1%BB%99%2050%2C%20Ph%C6%B0%E1%BB%9Dng%209%2C%20Th%C3%A0nh%20Ph%E1%BB%91%20M%E1%BB%B9%20Tho%2C%20T%E1%BB%89nh%20Ti%E1%BB%81n%20Giang</t>
+          <t>https://maps.google.com/?q=WinMart+S%E1%BB%91+339+Qu%E1%BB%91c+L%E1%BB%99+50%2C+Ph%C6%B0%E1%BB%9Dng+9%2C+Th%C3%A0nh+Ph%E1%BB%91+M%E1%BB%B9+Tho%2C+T%E1%BB%89nh+Ti%E1%BB%81n+Giang</t>
         </is>
       </c>
     </row>
@@ -8964,7 +8964,7 @@
       </c>
       <c r="I199" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TGG%2048%20%C4%90%C6%B0%E1%BB%9Dng%2030/4%2C%2048%20%C4%91%C6%B0%E1%BB%9Dng%2030%20th%C3%A1ng%204%2C%20TT.%20Cai%20L%E1%BA%ADy%2C%20TX.%20Cai%20L%E1%BA%ADy</t>
+          <t>https://maps.google.com/?q=WinMart+48+%C4%90%C6%B0%E1%BB%9Dng+30%2F4%2C+48+%C4%91%C6%B0%E1%BB%9Dng+30+th%C3%A1ng+4%2C+TT.+Cai+L%E1%BA%ADy%2C+TX.+Cai+L%E1%BA%ADy</t>
         </is>
       </c>
     </row>
@@ -9009,7 +9009,7 @@
       </c>
       <c r="I200" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%20%2B%20AGG%20Th%E1%BB%ADa%204082%20%E2%80%93%204122%20%C4%91%C6%B0%E1%BB%9Dng%20Ung%2C%20Th%E1%BB%ADa%204082%20%E2%80%93%204122%20%C4%91%2C%20Ung%20V%C4%83n%20Khi%C3%AAm%2C%20TP.%20Long%20Xuy%C3%AAn</t>
+          <t>https://maps.google.com/?q=WinMart+WM+%2B+AGG+Th%E1%BB%ADa+4082+%E2%80%93+4122+%C4%91%C6%B0%E1%BB%9Dng+Ung%2C+Th%E1%BB%ADa+4082+%E2%80%93+4122+%C4%91%2C+Ung+V%C4%83n+Khi%C3%AAm%2C+TP.+Long+Xuy%C3%AAn</t>
         </is>
       </c>
     </row>
@@ -9054,7 +9054,7 @@
       </c>
       <c r="I201" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20LAN%20128E-F%20Khu%20I%2C%20128E%20-%20F%2C%20Khu%20I%2C%20%E1%BA%A4p%20Ch%E1%BB%A3%2C%20X.%20Ph%C6%B0%E1%BB%9Bc%20L%E1%BB%A3i%2C%20H.%20B%E1%BA%BFn%20L%E1%BB%A9c</t>
+          <t>https://maps.google.com/?q=WinMart+128E-F+Khu+I%2C+128E+-+F%2C+Khu+I%2C+%E1%BA%A4p+Ch%E1%BB%A3%2C+X.+Ph%C6%B0%E1%BB%9Bc+L%E1%BB%A3i%2C+H.+B%E1%BA%BFn+L%E1%BB%A9c</t>
         </is>
       </c>
     </row>
@@ -9099,7 +9099,7 @@
       </c>
       <c r="I202" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20LAN%2074%20%C4%90%C6%B0%E1%BB%9Dng%20t%E1%BB%89nh%20832%2C%2074%20%C4%90%C6%B0%E1%BB%9Dng%20t%E1%BB%89nh%20832%2C%20%E1%BA%A4p%201%2C%20X.%20Nh%E1%BB%B1t%20Ch%C3%A1nh%2C%20H.%20B%E1%BA%BFn%20L%E1%BB%A9c%2C%20T.%20Long</t>
+          <t>https://maps.google.com/?q=WinMart+74+%C4%90%C6%B0%E1%BB%9Dng+t%E1%BB%89nh+832%2C+%E1%BA%A4p+1%2C+X.+Nh%E1%BB%B1t+Ch%C3%A1nh%2C+H.+B%E1%BA%BFn+L%E1%BB%A9c%2C+T.+Long</t>
         </is>
       </c>
     </row>
@@ -9144,7 +9144,7 @@
       </c>
       <c r="I203" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20T%C4%90%20140%2B142%2C%20TB%C4%90%20S%E1%BB%91%205%2C%20%C4%90%C6%B0%E1%BB%9Dng%2C%20T%C4%90%20140%20%2B142%2C%20TB%C4%90%20s%E1%BB%91%205%2C%20%C4%90%C6%B0%E1%BB%9Dng%20H%E1%BB%AFu%20Ngh%E1%BB%8B%2C%20TT.%20T%E1%BB%8Bnh%20Bi%C3%AAn%2C%20H.%20T%E1%BB%8Bnh%20Bi%C3%AAn</t>
+          <t>https://maps.google.com/?q=WinMart+T%C4%90+140%2B142%2C+TB%C4%90+S%E1%BB%91+5%2C+%C4%90%C6%B0%E1%BB%9Dng%2C+T%C4%90+140+%2B142%2C+TB%C4%90+s%E1%BB%91+5%2C+%C4%90%C6%B0%E1%BB%9Dng+H%E1%BB%AFu+Ngh%E1%BB%8B%2C+TT.+T%E1%BB%8Bnh+Bi%C3%AAn%2C+H.+T%E1%BB%8Bnh+Bi%C3%AAn</t>
         </is>
       </c>
     </row>
@@ -9189,7 +9189,7 @@
       </c>
       <c r="I204" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20107%20Nguy%E1%BB%85n%20Tri%20Ph%C6%B0%C6%A1ng%2C%20107%20Nguy%E1%BB%85n%20Tri%20Ph%C6%B0%C6%A1ng%2C%20P.%20Long%20Th%E1%BA%A1nh%2C%20TX.%20T%C3%A2n%20Ch%C3%A2u</t>
+          <t>https://maps.google.com/?q=WinMart+107+Nguy%E1%BB%85n+Tri+Ph%C6%B0%C6%A1ng%2C+P.+Long+Th%E1%BA%A1nh%2C+TX.+T%C3%A2n+Ch%C3%A2u</t>
         </is>
       </c>
     </row>
@@ -9234,7 +9234,7 @@
       </c>
       <c r="I205" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20582%20%C4%91%C6%B0%E1%BB%9Dng%20Nguy%E1%BB%85n%20Hu%E1%BB%87%2C%20582%20%C4%90%C6%B0%E1%BB%9Dng%20Nguy%E1%BB%85n%20Hu%E1%BB%87%2C%20TT.%20N%C3%BAi%20S%E1%BA%ADp%2C%20H.%20Tho%E1%BA%A1i%20S%C6%A1n</t>
+          <t>https://maps.google.com/?q=WinMart+582+%C4%90%C6%B0%E1%BB%9Dng+Nguy%E1%BB%85n+Hu%E1%BB%87%2C+TT.+N%C3%BAi+S%E1%BA%ADp%2C+H.+Tho%E1%BA%A1i+S%C6%A1n</t>
         </is>
       </c>
     </row>
@@ -9279,7 +9279,7 @@
       </c>
       <c r="I206" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TGG%201%20V%C3%B5%20Thanh%20T%C3%A2m%2C%201%20V%C3%B5%20Thanh%20T%C3%A2m%2C%20KP1%2C%20P.%204%2C%20TX.%20Cai%20L%E1%BA%ADy%2C%20%20T.%20B%C3%ACnh%20D%C6%B0%C6%A1ng</t>
+          <t>https://maps.google.com/?q=WinMart+1+V%C3%B5+Thanh+T%C3%A2m%2C+KP1%2C+P.+4%2C+TX.+Cai+L%E1%BA%ADy%2C+T.+B%C3%ACnh+D%C6%B0%C6%A1ng</t>
         </is>
       </c>
     </row>
@@ -9324,7 +9324,7 @@
       </c>
       <c r="I207" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20LAN%2016%20Nguy%E1%BB%85n%20V%C4%83n%20Ti%E1%BA%BFp%2C%2016%20Nguy%E1%BB%85n%20V%C4%83n%20Ti%E1%BA%BFp%2C%20P.5%2C%20TP.%20T%C3%A2n%20An</t>
+          <t>https://maps.google.com/?q=WinMart+16+Nguy%E1%BB%85n+V%C4%83n+Ti%E1%BA%BFp%2C+P.5%2C+TP.+T%C3%A2n+An</t>
         </is>
       </c>
     </row>
@@ -9369,7 +9369,7 @@
       </c>
       <c r="I208" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TGG%2074/7%20L%C3%AA%20Th%E1%BB%8B%20H%E1%BB%93ng%20G%E1%BA%A5m%2C%2074/7%20L%C3%AA%20Th%E1%BB%8B%20H%E1%BB%93ng%20G%E1%BA%A5m%2C%20KP.4%2C%20P.6%2C%20TP.%20M%E1%BB%B9%20Tho</t>
+          <t>https://maps.google.com/?q=WinMart+74%2F7+L%C3%AA+Th%E1%BB%8B+H%E1%BB%93ng+G%E1%BA%A5m%2C+KP.4%2C+P.6%2C+TP.+M%E1%BB%B9+Tho</t>
         </is>
       </c>
     </row>
@@ -9414,7 +9414,7 @@
       </c>
       <c r="I209" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20581%20%C4%90%C6%B0%E1%BB%9Dng%20V%C3%B2ng%20N%C3%BAi%20Sam%2C%20581%20%C4%90%C6%B0%E1%BB%9Dng%20V%C3%B2ng%20N%C3%BAi%20Sam%2C%20P.%20N%C3%BAi%20Sam%2C%20TP.%20Ch%C3%A2u%20%C4%90%E1%BB%91c%2C%20T.%20An%20Gian</t>
+          <t>https://maps.google.com/?q=WinMart+581+%C4%90%C6%B0%E1%BB%9Dng+V%C3%B2ng+N%C3%BAi+Sam%2C+P.+N%C3%BAi+Sam%2C+TP.+Ch%C3%A2u+%C4%90%E1%BB%91c%2C+T.+An+Gian</t>
         </is>
       </c>
     </row>
@@ -9459,7 +9459,7 @@
       </c>
       <c r="I210" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TGG%20378%20L%C3%AA%20Th%E1%BB%8B%20H%E1%BB%93ng%20G%E1%BA%A5m%2C%20378%20L%C3%AA%20Th%E1%BB%8B%20H%E1%BB%93ng%20G%E1%BA%A5m%2C%20P.%206%2C%20TP.%20M%E1%BB%B9%20Tho</t>
+          <t>https://maps.google.com/?q=WinMart+378+L%C3%AA+Th%E1%BB%8B+H%E1%BB%93ng+G%E1%BA%A5m%2C+P.+6%2C+TP.+M%E1%BB%B9+Tho</t>
         </is>
       </c>
     </row>
@@ -9504,7 +9504,7 @@
       </c>
       <c r="I211" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20108%20Tr%C6%B0ng%20N%E1%BB%AF%20V%C6%B0%C6%A1ng%2C%20108%20Tr%C6%B0ng%20N%E1%BB%AF%20V%C6%B0%C6%A1ng%2C%20P.%20Ch%C3%A2u%20Ph%C3%BA%20B%2C%20TP.%20Ch%C3%A2u%20%C4%90%E1%BB%91c</t>
+          <t>https://maps.google.com/?q=WinMart+108+Tr%C6%B0ng+N%E1%BB%AF+V%C6%B0%C6%A1ng%2C+P.+Ch%C3%A2u+Ph%C3%BA+B%2C+TP.+Ch%C3%A2u+%C4%90%E1%BB%91c</t>
         </is>
       </c>
     </row>
@@ -9549,7 +9549,7 @@
       </c>
       <c r="I212" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20LAN%2078%20Hu%E1%BB%B3nh%20Vi%E1%BB%87t%20Thanh%2C%2078%20Hu%E1%BB%B3nh%20Vi%E1%BB%87t%20Thanh%2C%20P.%202%2C%20TP.%20T%C3%A2n%20An</t>
+          <t>https://maps.google.com/?q=WinMart+78+Hu%E1%BB%B3nh+Vi%E1%BB%87t+Thanh%2C+P.+2%2C+TP.+T%C3%A2n+An</t>
         </is>
       </c>
     </row>
@@ -9594,7 +9594,7 @@
       </c>
       <c r="I213" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20191%20Th%E1%BB%A7%20Khoa%20Ngh%C4%A9a%2C%20191%20Th%E1%BB%A7%20Khoa%20Ngh%C4%A9a%2C%20P.%20Ch%C3%A2u%20Ph%C3%BA%20A%2C%20TP.%20Ch%C3%A2u%20%C4%90%E1%BB%91c</t>
+          <t>https://maps.google.com/?q=WinMart+191+Th%E1%BB%A7+Khoa+Ngh%C4%A9a%2C+P.+Ch%C3%A2u+Ph%C3%BA+A%2C+TP.+Ch%C3%A2u+%C4%90%E1%BB%91c</t>
         </is>
       </c>
     </row>
@@ -9639,7 +9639,7 @@
       </c>
       <c r="I214" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%2054-56%20Nguy%E1%BB%85n%20V%C4%83n%20C%E1%BB%AB%2C%2054-56%20Nguy%E1%BB%85n%20V%C4%83n%20C%E1%BB%AB%2C%20TT.%20An%20Ch%C3%A2u%2C%20H.%20Ch%C3%A2u%20Th%C3%A0nh</t>
+          <t>https://maps.google.com/?q=WinMart+54-56+Nguy%E1%BB%85n+V%C4%83n+C%E1%BB%AB%2C+TT.+An+Ch%C3%A2u%2C+H.+Ch%C3%A2u+Th%C3%A0nh</t>
         </is>
       </c>
     </row>
@@ -9684,7 +9684,7 @@
       </c>
       <c r="I215" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20342%20Qu%E1%BB%91c%20l%E1%BB%99%2091%2C%20342%20Qu%E1%BB%91c%20l%E1%BB%99%2091%2C%20TT.%20C%C3%A1i%20D%E1%BA%A7u%2C%20H.%20Ch%C3%A2u%20Ph%C3%BA</t>
+          <t>https://maps.google.com/?q=WinMart+342+Qu%E1%BB%91c+l%E1%BB%99+91%2C+TT.+C%C3%A1i+D%E1%BA%A7u%2C+H.+Ch%C3%A2u+Ph%C3%BA</t>
         </is>
       </c>
     </row>
@@ -9729,7 +9729,7 @@
       </c>
       <c r="I216" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TGG%2093%20V%C3%B5%20Duy%20Linh%2C%2093%20V%C3%B5%20Duy%20Linh%2C%20KP.%20H%C3%B2a%20Th%C6%A1m%201%2C%20TT.%20T%C3%A2n%20H%C3%B2a%2C%20H.%20G%C3%B2%20C%C3%B4ng%20%C4%90%C3%B4ng</t>
+          <t>https://maps.google.com/?q=WinMart+93+V%C3%B5+Duy+Linh%2C+KP.+H%C3%B2a+Th%C6%A1m+1%2C+TT.+T%C3%A2n+H%C3%B2a%2C+H.+G%C3%B2+C%C3%B4ng+%C4%90%C3%B4ng</t>
         </is>
       </c>
     </row>
@@ -9774,7 +9774,7 @@
       </c>
       <c r="I217" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20STG%20133%20Tr%C6%B0%C6%A1ng%20C%C3%B4ng%20%C4%90%E1%BB%8Bnh%2C%20133%20Tr%C6%B0%C6%A1ng%20C%C3%B4ng%20%C4%90%E1%BB%8Bnh%2C%20P.%202%2C%20TP.%20S%C3%B3c%20Tr%C4%83ng</t>
+          <t>https://maps.google.com/?q=WinMart+133+Tr%C6%B0%C6%A1ng+C%C3%B4ng+%C4%90%E1%BB%8Bnh%2C+P.+2%2C+TP.+S%C3%B3c+Tr%C4%83ng</t>
         </is>
       </c>
     </row>
@@ -9819,7 +9819,7 @@
       </c>
       <c r="I218" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20T%E1%BB%95%208%2C%20%E1%BA%A4p%20H%C3%B2a%20H%E1%BA%A1%2C%20T%E1%BB%95%208%2C%20%E1%BA%A4p%20H%C3%B2a%20H%E1%BA%A1%2C%20X.%20Ki%E1%BA%BFn%20An%2C%20H.%20Ch%E1%BB%A3%20M%E1%BB%9Bi</t>
+          <t>https://maps.google.com/?q=WinMart+T%E1%BB%95+8%2C+%E1%BA%A4p+H%C3%B2a+H%E1%BA%A1%2C+X.+Ki%E1%BA%BFn+An%2C+H.+Ch%E1%BB%A3+M%E1%BB%9Bi</t>
         </is>
       </c>
     </row>
@@ -9864,7 +9864,7 @@
       </c>
       <c r="I219" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20T%E1%BB%95%201%2C%20%C4%90.%20T%C3%A2n%20L%E1%BB%99%20Ki%E1%BB%81u%20L%C6%B0%C6%A1ng%2C%20T%E1%BB%95%201%2C%20%C4%90.%20T%C3%A2n%20L%E1%BB%99%20Ki%E1%BB%81u%20L%C6%B0%C6%A1ng%2C%20Kh%C3%B3m%20V%C4%A9nh%20T%C3%A2y%203%2C%20P.%20N%C3%BAi%20Sam%2C%20TP.%20Ch%C3%A2u%20%C4%90%E1%BB%91c</t>
+          <t>https://maps.google.com/?q=WinMart+T%E1%BB%95+1%2C+%C4%90.+T%C3%A2n+L%E1%BB%99+Ki%E1%BB%81u+L%C6%B0%C6%A1ng%2C+Kh%C3%B3m+V%C4%A9nh+T%C3%A2y+3%2C+P.+N%C3%BAi+Sam%2C+TP.+Ch%C3%A2u+%C4%90%E1%BB%91c</t>
         </is>
       </c>
     </row>
@@ -9909,7 +9909,7 @@
       </c>
       <c r="I220" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TGG%20T%C4%90S%20308%2C%20TB%C4%90S%2019%20Qu%E1%BB%91c%20l%E1%BB%99%2050%2C%20T%C4%90S%20308%2C%20TB%C4%90S%2019%2C%20Qu%E1%BB%91c%20l%E1%BB%99%2050%2C%20P.%204%2C%20TX.%20G%C3%B2%20C%C3%B4ng</t>
+          <t>https://maps.google.com/?q=WinMart+T%C4%90S+308%2C+TB%C4%90S+19+Qu%E1%BB%91c+l%E1%BB%99+50%2C+T%C4%90S+308%2C+TB%C4%90S+19%2C+Qu%E1%BB%91c+l%E1%BB%99+50%2C+P.+4%2C+TX.+G%C3%B2+C%C3%B4ng</t>
         </is>
       </c>
     </row>
@@ -9954,7 +9954,7 @@
       </c>
       <c r="I221" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TGG%20147A%20Tr%E1%BA%A7n%20C%C3%B4ng%20T%C6%B0%E1%BB%9Dng%2C%20147A%20Tr%E1%BA%A7n%20C%C3%B4ng%20T%C6%B0%E1%BB%9Dng%2C%20P.%205%2C%20TX.%20G%C3%B2%20C%C3%B4ng</t>
+          <t>https://maps.google.com/?q=WinMart+147A+Tr%E1%BA%A7n+C%C3%B4ng+T%C6%B0%E1%BB%9Dng%2C+P.+5%2C+TX.+G%C3%B2+C%C3%B4ng</t>
         </is>
       </c>
     </row>
@@ -9999,7 +9999,7 @@
       </c>
       <c r="I222" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20BLU%20T%C4%90%20287%2C%20TB%C4%90S%2025%20Ninh%20B%C3%ACnh%2C%20T%C4%90S%20287%2C%20TB%C4%90S%2025%20%C4%90%C6%B0%E1%BB%9Dng%20Ninh%20B%C3%ACnh%2C%20Kh%C3%B3m%204%2C%20P.%202%2C%20TP.%20B%E1%BA%A1c%20Li%C3%AAu</t>
+          <t>https://maps.google.com/?q=WinMart+T%C4%90+287%2C+TB%C4%90S+25+Ninh+B%C3%ACnh%2C+T%C4%90S+287%2C+TB%C4%90S+25+%C4%90%C6%B0%E1%BB%9Dng+Ninh+B%C3%ACnh%2C+Kh%C3%B3m+4%2C+P.+2%2C+TP.+B%E1%BA%A1c+Li%C3%AAu</t>
         </is>
       </c>
     </row>
@@ -10044,7 +10044,7 @@
       </c>
       <c r="I223" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20BLU%20361%20V%C3%B5%20Th%E1%BB%8B%20S%C3%A1u%2C%20361%20V%C3%B5%20Th%E1%BB%8B%20S%C3%A1u%2C%20Kh%C3%B3m%204%2C%20P.%207%2C%20TP.%20B%E1%BA%A1c%20Li%C3%AAu</t>
+          <t>https://maps.google.com/?q=WinMart+361+V%C3%B5+Th%E1%BB%8B+S%C3%A1u%2C+Kh%C3%B3m+4%2C+P.+7%2C+TP.+B%E1%BA%A1c+Li%C3%AAu</t>
         </is>
       </c>
     </row>
@@ -10089,7 +10089,7 @@
       </c>
       <c r="I224" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CMU%20315%20L%C3%BD%20Th%C6%B0%E1%BB%9Dng%20Ki%E1%BB%87t%2C%20315%20L%C3%BD%20Th%C6%B0%E1%BB%9Dng%20Ki%E1%BB%87t%2C%20P.%206%2C%20TP.%20C%C3%A0%20Mau</t>
+          <t>https://maps.google.com/?q=WinMart+315+L%C3%BD+Th%C6%B0%E1%BB%9Dng+Ki%E1%BB%87t%2C+P.+6%2C+TP.+C%C3%A0+Mau</t>
         </is>
       </c>
     </row>
@@ -10134,7 +10134,7 @@
       </c>
       <c r="I225" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20BLU%206%20L%C3%AA%20Du%E1%BA%A9n%2C%2006%20L%C3%AA%20Du%E1%BA%A9n%2C%20P.%201%2C%20TP.%20B%E1%BA%A1c%20Li%C3%AAu</t>
+          <t>https://maps.google.com/?q=WinMart+06+L%C3%AA+Du%E1%BA%A9n%2C+P.+1%2C+TP.+B%E1%BA%A1c+Li%C3%AAu</t>
         </is>
       </c>
     </row>
@@ -10179,7 +10179,7 @@
       </c>
       <c r="I226" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20662%20Tr%E1%BA%A7n%20H%C6%B0ng%20%C4%90%E1%BA%A1o%2C%20662%20Tr%E1%BA%A7n%20H%C6%B0ng%20%C4%90%E1%BA%A1o%2C%20t%E1%BB%95%2062%20B%C3%ACnh%20%C4%90%E1%BB%A9c%201%2C%20P.%20B%C3%ACnh%20%C4%90%E1%BB%A9c%2C%20TP.%20Long%20Xuy%C3%AAn</t>
+          <t>https://maps.google.com/?q=WinMart+662+Tr%E1%BA%A7n+H%C6%B0ng+%C4%90%E1%BA%A1o%2C+t%E1%BB%95+62+B%C3%ACnh+%C4%90%E1%BB%A9c+1%2C+P.+B%C3%ACnh+%C4%90%E1%BB%A9c%2C+TP.+Long+Xuy%C3%AAn</t>
         </is>
       </c>
     </row>
@@ -10224,7 +10224,7 @@
       </c>
       <c r="I227" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TGG%20489%20Qu%E1%BB%91c%20l%E1%BB%99%2050%2C%20489%20Qu%E1%BB%91c%20l%E1%BB%99%2050%2C%20khu%20ph%E1%BB%91%204%2C%20P.%209%2C%20TP.%20M%E1%BB%B9%20Tho</t>
+          <t>https://maps.google.com/?q=WinMart+489+Qu%E1%BB%91c+l%E1%BB%99+50%2C+khu+ph%E1%BB%91+4%2C+P.+9%2C+TP.+M%E1%BB%B9+Tho</t>
         </is>
       </c>
     </row>
@@ -10269,7 +10269,7 @@
       </c>
       <c r="I228" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20STG%204-6%20Pasteur%2C%204-6%20Pasteur%2C%20Kh%C3%B3m%202%2C%20P.%208%2C%20TP.%20S%C3%B3c%20Tr%C4%83ng</t>
+          <t>https://maps.google.com/?q=WinMart+4-6+Pasteur%2C+Kh%C3%B3m+2%2C+P.+8%2C+TP.+S%C3%B3c+Tr%C4%83ng</t>
         </is>
       </c>
     </row>
@@ -10314,7 +10314,7 @@
       </c>
       <c r="I229" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20STG%20T%C4%90%20195-TB%C4%90%2018%20Ung%20C%C3%B4ng%20U%E1%BA%A9n%2C%20Th%E1%BB%ADa%20%C4%91%E1%BA%A5t%20s%E1%BB%91%20195%2C%20T%E1%BB%9D%20b%E1%BA%A3n%20%C4%91%E1%BB%93%20s%E1%BB%91%2018%2C%20%C4%91%C6%B0%E1%BB%9Dng%20Ung%20C%C3%B4ng%20U%E1%BA%A9n%2C%20%E1%BA%A4p%20An%20Th%C3%A0nh%2C%20TT.%20K%E1%BA%BF%20S%C3%A1ch%2C%20H.%20K%E1%BA%BF%20S%C3%A1ch</t>
+          <t>https://maps.google.com/?q=WinMart+T%C4%90+195-TB%C4%90+18+Ung+C%C3%B4ng+U%E1%BA%A9n%2C+Th%E1%BB%ADa+%C4%91%E1%BA%A5t+s%E1%BB%91+195%2C+T%E1%BB%9D+b%E1%BA%A3n+%C4%91%E1%BB%93+s%E1%BB%91+18%2C+%C4%91%C6%B0%E1%BB%9Dng+Ung+C%C3%B4ng+U%E1%BA%A9n%2C+%E1%BA%A4p+An+Th%C3%A0nh%2C+TT.+K%E1%BA%BF+S%C3%A1ch%2C+H.+K%E1%BA%BF+S%C3%A1ch</t>
         </is>
       </c>
     </row>
@@ -10359,7 +10359,7 @@
       </c>
       <c r="I230" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20BTE%20TB%C4%90%2075%20Nguy%E1%BB%85n%20Th%E1%BB%8B%20%C4%90%E1%BB%8Bnh%2C%20Th%E1%BB%ADa%20%C4%91%E1%BA%A5t%20106%2C%20108%2C%20109%20t%E1%BB%9D%20b%E1%BA%A3n%20%C4%91%E1%BB%93%20s%E1%BB%91%2075%2C%20%C4%90%C6%B0%E1%BB%9Dng%20Nguy%E1%BB%85n%20Th%E1%BB%8B%20%C4%90%E1%BB%8Bnh%2C%20KP.%201%2C%20TT.%20Gi%E1%BB%93ng%20Tr%C3%B4m%2C%20H.%20Gi%E1%BB%93ng%20Tr%C3%B4m</t>
+          <t>https://maps.google.com/?q=WinMart+TB%C4%90+75+Nguy%E1%BB%85n+Th%E1%BB%8B+%C4%90%E1%BB%8Bnh%2C+Th%E1%BB%ADa+%C4%91%E1%BA%A5t+106%2C+108%2C+109+t%E1%BB%9D+b%E1%BA%A3n+%C4%91%E1%BB%93+s%E1%BB%91+75%2C+%C4%90%C6%B0%E1%BB%9Dng+Nguy%E1%BB%85n+Th%E1%BB%8B+%C4%90%E1%BB%8Bnh%2C+KP.+1%2C+TT.+Gi%E1%BB%93ng+Tr%C3%B4m%2C+H.+Gi%E1%BB%93ng+Tr%C3%B4m</t>
         </is>
       </c>
     </row>
@@ -10404,7 +10404,7 @@
       </c>
       <c r="I231" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20STG%20%C4%90%C6%B0%E1%BB%9Dng%20t%E1%BB%89nh%20937B%2C%20%E1%BA%A4p%20Ch%E1%BB%A3%20M%E1%BB%9Bi%2C%20Th%E1%BB%ADa%20%C4%91%E1%BA%A5t%20s%E1%BB%91%2095%2C%20T%E1%BB%9D%20b%E1%BA%A3n%20%C4%91%E1%BB%93%20s%E1%BB%91%2012%2C%20%C4%90%C6%B0%E1%BB%9Dng%20t%E1%BB%89nh%20937B%2C%20%E1%BA%A4p%20Ch%E1%BB%A3%20M%E1%BB%9Bi%2C%20TT.%20H%C6%B0ng%20L%E1%BB%A3i%2C%20H.%20Th%E1%BA%A1nh%20Tr%E1%BB%8B</t>
+          <t>https://maps.google.com/?q=WinMart+Th%E1%BB%ADa+%C4%91%E1%BA%A5t+s%E1%BB%91+95%2C+T%E1%BB%9D+b%E1%BA%A3n+%C4%91%E1%BB%93+s%E1%BB%91+12%2C+%C4%90%C6%B0%E1%BB%9Dng+t%E1%BB%89nh+937B%2C+%E1%BA%A4p+Ch%E1%BB%A3+M%E1%BB%9Bi%2C+TT.+H%C6%B0ng+L%E1%BB%A3i%2C+H.+Th%E1%BA%A1nh+Tr%E1%BB%8B</t>
         </is>
       </c>
     </row>
@@ -10449,7 +10449,7 @@
       </c>
       <c r="I232" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TVH%20172%20%C4%90%C6%B0%E1%BB%9Dng%2019/5%2C%20172%20%C4%90%C6%B0%E1%BB%9Dng%2019/5%20Kh%C3%B3m%202%2C%20P.%201%2C%20TX.%20Duy%C3%AAn%20H%E1%BA%A3i</t>
+          <t>https://maps.google.com/?q=WinMart+172+%C4%90%C6%B0%E1%BB%9Dng+19%2F5+Kh%C3%B3m+2%2C+P.+1%2C+TX.+Duy%C3%AAn+H%E1%BA%A3i</t>
         </is>
       </c>
     </row>
@@ -10494,7 +10494,7 @@
       </c>
       <c r="I233" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20TGG%20202%20Nam%20K%E1%BB%B3%20Kh%E1%BB%9Fi%20Ngh%C4%A9a%2C%20202%20%C4%90%C6%B0%E1%BB%9Dng%20Nam%20K%E1%BB%B3%20Kh%E1%BB%9Fi%20Ngh%C4%A9a%2C%20P.%201%2C%20TP.%20M%E1%BB%B9%20Tho</t>
+          <t>https://maps.google.com/?q=WinMart+202+Nam+K%E1%BB%B3+Kh%E1%BB%9Fi+Ngh%C4%A9a%2C+202+%C4%90%C6%B0%E1%BB%9Dng+Nam+K%E1%BB%B3+Kh%E1%BB%9Fi+Ngh%C4%A9a%2C+P.+1%2C+TP.+M%E1%BB%B9+Tho</t>
         </is>
       </c>
     </row>
@@ -10539,7 +10539,7 @@
       </c>
       <c r="I234" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20332-334%20L%C3%BD%20Th%C3%A1i%20T%E1%BB%95%2C%20332-334%20L%C3%BD%20Th%C3%A1i%20T%E1%BB%95%2C%20P.%20M%E1%BB%B9%20Long%2C%20TP.%20Long%20Xuy%C3%AAn</t>
+          <t>https://maps.google.com/?q=WinMart+332-334+L%C3%BD+Th%C3%A1i+T%E1%BB%95%2C+P.+M%E1%BB%B9+Long%2C+TP.+Long+Xuy%C3%AAn</t>
         </is>
       </c>
     </row>
@@ -10584,7 +10584,7 @@
       </c>
       <c r="I235" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20%C4%90%C6%B0%E1%BB%9Dng%20Tr%E1%BA%A7n%20H%C6%B0ng%20%C4%90%E1%BA%A1o%2C%20P.%20M%E1%BB%B9%20Th%E1%BB%9Bi%2C%20TP.%20Long%20Xuy%C3%AAn</t>
+          <t>https://maps.google.com/?q=WinMart+%C4%90%C6%B0%E1%BB%9Dng+Tr%E1%BA%A7n+H%C6%B0ng+%C4%90%E1%BA%A1o%2C+P.+M%E1%BB%B9+Th%E1%BB%9Bi%2C+TP.+Long+Xuy%C3%AAn</t>
         </is>
       </c>
     </row>
@@ -10629,7 +10629,7 @@
       </c>
       <c r="I236" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CMU%20%E1%BA%A4p%205%2C%20T%C3%A2n%20L%E1%BB%99c%2C%20Th%E1%BB%ADa%20%C4%91%E1%BA%A5t%20s%E1%BB%91%20187%2C%20T%E1%BB%9D%20b%E1%BA%A3n%20%C4%91%E1%BB%93%20s%E1%BB%91%2017%2C%20%E1%BA%A4p%205%2C%20X.%20T%C3%A2n%20L%E1%BB%99c</t>
+          <t>https://maps.google.com/?q=WinMart+%E1%BA%A4p+5%2C+T%C3%A2n+L%E1%BB%99c%2C+Th%E1%BB%ADa+%C4%91%E1%BA%A5t+s%E1%BB%91+187%2C+T%E1%BB%9D+b%E1%BA%A3n+%C4%91%E1%BB%93+s%E1%BB%91+17%2C+%E1%BA%A4p+5%2C+X.+T%C3%A2n+L%E1%BB%99c</t>
         </is>
       </c>
     </row>
@@ -10674,7 +10674,7 @@
       </c>
       <c r="I237" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CMU%20%E1%BA%A4p%20T%C3%A2n%20Hi%E1%BB%87p%2C%20Tr%E1%BA%A7n%20V%C4%83n%20Th%E1%BB%9Di%2C%20Th%E1%BB%ADa%20%C4%91%E1%BA%A5t%20s%E1%BB%91%201%20v%C3%A0%20Th%E1%BB%ADa%20%C4%91%E1%BA%A5t%20s%E1%BB%91%202%2C%20T%E1%BB%9D%20B%E1%BA%A3n%20%C4%90%E1%BB%93%2028%2C%20%E1%BA%A4p%20T%C3%A2n%20Hi%E1%BB%87p%2C%20X.%20Tr%E1%BA%A7n%20V%C4%83n%20Th%E1%BB%9Di</t>
+          <t>https://maps.google.com/?q=WinMart+%E1%BA%A4p+T%C3%A2n+Hi%E1%BB%87p%2C+Tr%E1%BA%A7n+V%C4%83n+Th%E1%BB%9Di%2C+Th%E1%BB%ADa+%C4%91%E1%BA%A5t+s%E1%BB%91+1+v%C3%A0+Th%E1%BB%ADa+%C4%91%E1%BA%A5t+s%E1%BB%91+2%2C+T%E1%BB%9D+B%E1%BA%A3n+%C4%90%E1%BB%93+28%2C+%E1%BA%A4p+T%C3%A2n+Hi%E1%BB%87p%2C+X.+Tr%E1%BA%A7n+V%C4%83n+Th%E1%BB%9Di</t>
         </is>
       </c>
     </row>
@@ -10719,7 +10719,7 @@
       </c>
       <c r="I238" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CMU%20QL1A%2C%20L%C6%B0%C6%A1ng%20Th%E1%BA%BF%20Tr%C3%A2n%2C%20Th%E1%BB%ADa%20%C4%90%E1%BA%A5t%20s%E1%BB%91%2033%20v%C3%A0%2048%2C%20T%E1%BB%9D%20B%E1%BA%A3n%20%C4%90%E1%BB%93%20s%E1%BB%91%2043%2C%20%C4%90%C6%B0%E1%BB%9Dng%20Qu%E1%BB%91c%20l%E1%BB%99%201A%2C%20X.%20L%C6%B0%C6%A1ng%20Th%E1%BA%BF%20Tr%C3%A2n</t>
+          <t>https://maps.google.com/?q=WinMart+QL1A%2C+L%C6%B0%C6%A1ng+Th%E1%BA%BF+Tr%C3%A2n%2C+Th%E1%BB%ADa+%C4%90%E1%BA%A5t+s%E1%BB%91+33+v%C3%A0+48%2C+T%E1%BB%9D+B%E1%BA%A3n+%C4%90%E1%BB%93+s%E1%BB%91+43%2C+%C4%90%C6%B0%E1%BB%9Dng+Qu%E1%BB%91c+l%E1%BB%99+1A%2C+X.+L%C6%B0%C6%A1ng+Th%E1%BA%BF+Tr%C3%A2n</t>
         </is>
       </c>
     </row>
@@ -10764,7 +10764,7 @@
       </c>
       <c r="I239" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CMU%20%E1%BA%A4p%20C%C3%A1i%20N%E1%BA%A9y%2C%20N%C4%83m%20C%C4%83n%2C%20Th%E1%BB%ADa%20%C4%90%E1%BA%A5t%20s%E1%BB%91%20265%2C%20266%20v%C3%A0%20267%2C%20T%E1%BB%9D%20B%E1%BA%A3n%20%C4%90%E1%BB%93%20s%E1%BB%91%2011%2C%20%E1%BA%A4p%20C%C3%A1i%20N%E1%BA%A9y%2C%20X.%20N%C4%83m%20C%C4%83n</t>
+          <t>https://maps.google.com/?q=WinMart+%E1%BA%A4p+C%C3%A1i+N%E1%BA%A9y%2C+N%C4%83m+C%C4%83n%2C+Th%E1%BB%ADa+%C4%90%E1%BA%A5t+s%E1%BB%91+265%2C+266+v%C3%A0+267%2C+T%E1%BB%9D+B%E1%BA%A3n+%C4%90%E1%BB%93+s%E1%BB%91+11%2C+%E1%BA%A4p+C%C3%A1i+N%E1%BA%A9y%2C+X.+N%C4%83m+C%C4%83n</t>
         </is>
       </c>
     </row>
@@ -10809,7 +10809,7 @@
       </c>
       <c r="I240" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CMU%20232A%20L%C3%BD%20V%C4%83n%20L%C3%A2m%2C%20232A%20L%C3%BD%20V%C4%83n%20L%C3%A2m%2C%20P.%20An%20Xuy%C3%AAn</t>
+          <t>https://maps.google.com/?q=WinMart+232A+L%C3%BD+V%C4%83n+L%C3%A2m%2C+P.+An+Xuy%C3%AAn</t>
         </is>
       </c>
     </row>
@@ -10854,7 +10854,7 @@
       </c>
       <c r="I241" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%2011B-12%20B%C3%B9i%20Th%E1%BB%8B%20Xu%C3%A2n%2C%20Long%20Xuy%C3%AAn%2C%2011B%20-%2012%20B%C3%B9i%20Th%E1%BB%8B%20Xu%C3%A2n%2C%20P.%20Long%20Xuy%C3%AAn</t>
+          <t>https://maps.google.com/?q=WinMart+11B-12+B%C3%B9i+Th%E1%BB%8B+Xu%C3%A2n%2C+Long+Xuy%C3%AAn%2C+11B+-+12+B%C3%B9i+Th%E1%BB%8B+Xu%C3%A2n%2C+P.+Long+Xuy%C3%AAn</t>
         </is>
       </c>
     </row>
@@ -10899,7 +10899,7 @@
       </c>
       <c r="I242" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20AGG%20Ama%20138%20%C4%90%C6%B0%E1%BB%9Dng%20Amalfi%2C%20Ama%20138%20%C4%90%C6%B0%E1%BB%9Dng%20Amalfi%2C%20Th%E1%BB%8B%20Tr%E1%BA%A5n%20Sunset%20Town%2C%20KP6%20An%20Th%E1%BB%9Bi%2C%20TP.%20Ph%C3%BA%20Qu%E1%BB%91c%2C%20T%E1%BB%89nh%20Ki%C3%AAn%20Giang</t>
+          <t>https://maps.google.com/?q=WinMart+Ama+138+%C4%90%C6%B0%E1%BB%9Dng+Amalfi%2C+Th%E1%BB%8B+Tr%E1%BA%A5n+Sunset+Town%2C+KP6+An+Th%E1%BB%9Bi%2C+TP.+Ph%C3%BA+Qu%E1%BB%91c%2C+T%E1%BB%89nh+Ki%C3%AAn+Giang</t>
         </is>
       </c>
     </row>
@@ -10944,7 +10944,7 @@
       </c>
       <c r="I243" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CMU%2049%20%C4%90%C6%B0%E1%BB%9Dng%203/2%2C%20T%C3%A2n%20Th%C3%A0nh%2C%20S%E1%BB%91%2049%2C%20%C4%90%C6%B0%E1%BB%9Dng%203%20th%C3%A1ng%202%2C%20P.%20T%C3%A2n%20Th%C3%A0nh</t>
+          <t>https://maps.google.com/?q=WinMart+49+%C4%90%C6%B0%E1%BB%9Dng+3%2F2%2C+T%C3%A2n+Th%C3%A0nh%2C+S%E1%BB%91+49%2C+%C4%90%C6%B0%E1%BB%9Dng+3+th%C3%A1ng+2%2C+P.+T%C3%A2n+Th%C3%A0nh</t>
         </is>
       </c>
     </row>
@@ -10989,7 +10989,7 @@
       </c>
       <c r="I244" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CMU%20H%E1%BA%A3i%20Th%C6%B0%E1%BB%A3ng%20L%C3%A3n%20%C3%94ng%2C%20H%C3%B2a%20Th%C3%A0nh%2C%20Th%E1%BB%ADa%20%C4%90%E1%BA%A5t%20s%E1%BB%91%2058%2C%20T%E1%BB%9D%20B%E1%BA%A3n%20%C4%90%E1%BB%93%20s%E1%BB%91%2049%2C%20%C4%90%C6%B0%E1%BB%9Dng%20H%E1%BA%A3i%20Th%C6%B0%E1%BB%A3ng%20L%C3%A3n%20%C3%94ng%2C%20P.%20H%C3%B2a%20Th%C3%A0nh</t>
+          <t>https://maps.google.com/?q=WinMart+H%E1%BA%A3i+Th%C6%B0%E1%BB%A3ng+L%C3%A3n+%C3%94ng%2C+H%C3%B2a+Th%C3%A0nh%2C+Th%E1%BB%ADa+%C4%90%E1%BA%A5t+s%E1%BB%91+58%2C+T%E1%BB%9D+B%E1%BA%A3n+%C4%90%E1%BB%93+s%E1%BB%91+49%2C+%C4%90%C6%B0%E1%BB%9Dng+H%E1%BA%A3i+Th%C6%B0%E1%BB%A3ng+L%C3%A3n+%C3%94ng%2C+P.+H%C3%B2a+Th%C3%A0nh</t>
         </is>
       </c>
     </row>
@@ -11034,7 +11034,7 @@
       </c>
       <c r="I245" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CMU%20%E1%BA%A4p%201%2C%20Th%E1%BB%9Bi%20B%C3%ACnh%2C%20Th%E1%BB%ADa%20%C4%91%E1%BA%A5t%20293%2C%20T%E1%BB%9D%20B%E1%BA%A3n%20%C4%90%E1%BB%93%20s%E1%BB%91%2038%2C%20%E1%BA%A4p%201%2C%20X.%20Th%E1%BB%9Bi%20B%C3%ACnh</t>
+          <t>https://maps.google.com/?q=WinMart+%E1%BA%A4p+1%2C+Th%E1%BB%9Bi+B%C3%ACnh%2C+Th%E1%BB%ADa+%C4%91%E1%BA%A5t+293%2C+T%E1%BB%9D+B%E1%BA%A3n+%C4%90%E1%BB%93+s%E1%BB%91+38%2C+%E1%BA%A4p+1%2C+X.+Th%E1%BB%9Bi+B%C3%ACnh</t>
         </is>
       </c>
     </row>
@@ -11079,7 +11079,7 @@
       </c>
       <c r="I246" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CMU%20T%E1%BA%A1%20An%20Kh%C6%B0%C6%A1ng%2C%20%C4%90%E1%BA%A7m%20D%C6%A1i%2C%20Th%E1%BB%ADa%20%C4%90%E1%BA%A5t%20s%E1%BB%91%20262%2C%20T%E1%BB%9D%20B%E1%BA%A3n%20%C4%90%E1%BB%93%20s%E1%BB%91%2014%2C%20%C4%90%C6%B0%E1%BB%9Dng%20T%E1%BA%A1%20An%20Kh%C6%B0%C6%A1ng%2C%20X.%20%C4%90%E1%BA%A7m%20D%C6%A1i</t>
+          <t>https://maps.google.com/?q=WinMart+T%E1%BA%A1+An+Kh%C6%B0%C6%A1ng%2C+%C4%90%E1%BA%A7m+D%C6%A1i%2C+Th%E1%BB%ADa+%C4%90%E1%BA%A5t+s%E1%BB%91+262%2C+T%E1%BB%9D+B%E1%BA%A3n+%C4%90%E1%BB%93+s%E1%BB%91+14%2C+%C4%90%C6%B0%E1%BB%9Dng+T%E1%BA%A1+An+Kh%C6%B0%C6%A1ng%2C+X.+%C4%90%E1%BA%A7m+D%C6%A1i</t>
         </is>
       </c>
     </row>
@@ -11124,7 +11124,7 @@
       </c>
       <c r="I247" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=WM%2B%20CMU%20%E1%BA%A4p%2011%2C%20Kh%C3%A1nh%20L%C3%A2m%2C%20Th%E1%BB%ADa%20%C4%91%E1%BA%A5t%20s%E1%BB%91%20118%2C%20T%E1%BB%9D%20b%E1%BA%A3n%20%C4%91%E1%BB%93%20s%E1%BB%91%2064%2C%20%E1%BA%A4p%2011%2C%20X.%20Kh%C3%A1nh%20L%C3%A2m</t>
+          <t>https://maps.google.com/?q=WinMart+%E1%BA%A4p+11%2C+Kh%C3%A1nh+L%C3%A2m%2C+Th%E1%BB%ADa+%C4%91%E1%BA%A5t+s%E1%BB%91+118%2C+T%E1%BB%9D+b%E1%BA%A3n+%C4%91%E1%BB%93+s%E1%BB%91+64%2C+%E1%BA%A4p+11%2C+X.+Kh%C3%A1nh+L%C3%A2m</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(nvxl): correct inverted telegram tags for Bao Toan (@Nguyen_Toan) and Trong Bang (@pinca0602)
</commit_message>
<xml_diff>
--- a/danh_sach_dinh_vi_winmart_mt01.xlsx
+++ b/danh_sach_dinh_vi_winmart_mt01.xlsx
@@ -585,7 +585,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -913,7 +913,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -1487,7 +1487,7 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>Trần Trọng Bằng (@Nguyen_Toan)</t>
+          <t>Trần Trọng Bằng (@pinca0602)</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Trần Trọng Bằng (@Nguyen_Toan)</t>
+          <t>Trần Trọng Bằng (@pinca0602)</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Trần Trọng Bằng (@Nguyen_Toan)</t>
+          <t>Trần Trọng Bằng (@pinca0602)</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
@@ -2225,7 +2225,7 @@
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
@@ -2594,7 +2594,7 @@
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
@@ -2717,7 +2717,7 @@
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G56" s="3" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
@@ -3168,7 +3168,7 @@
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
@@ -3250,7 +3250,7 @@
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
@@ -3291,7 +3291,7 @@
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
@@ -3332,7 +3332,7 @@
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G74" s="3" t="inlineStr">
@@ -3701,7 +3701,7 @@
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G79" s="3" t="inlineStr">
@@ -3742,7 +3742,7 @@
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G80" s="3" t="inlineStr">
@@ -3865,7 +3865,7 @@
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>Trần Trọng Bằng (@Nguyen_Toan)</t>
+          <t>Trần Trọng Bằng (@pinca0602)</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr">
@@ -4070,7 +4070,7 @@
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G88" s="3" t="inlineStr">
@@ -4152,7 +4152,7 @@
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G90" s="3" t="inlineStr">
@@ -4275,7 +4275,7 @@
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G93" s="3" t="inlineStr">
@@ -4316,7 +4316,7 @@
       </c>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G94" s="3" t="inlineStr">
@@ -4398,7 +4398,7 @@
       </c>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G96" s="3" t="inlineStr">
@@ -4603,7 +4603,7 @@
       </c>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G101" s="3" t="inlineStr">
@@ -4644,7 +4644,7 @@
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr">
@@ -4726,7 +4726,7 @@
       </c>
       <c r="F104" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G104" s="3" t="inlineStr">
@@ -4767,7 +4767,7 @@
       </c>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G105" s="3" t="inlineStr">
@@ -4808,7 +4808,7 @@
       </c>
       <c r="F106" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Phước Bảo Toàn (@pinca0602)</t>
+          <t>Nguyễn Phước Bảo Toàn (@Nguyen_Toan)</t>
         </is>
       </c>
       <c r="G106" s="3" t="inlineStr">

</xml_diff>